<commit_message>
Recupero idee 28-29-30 maggio 2026 (routine era disabilitata)
16 idee (4+4+8) aggiunte al Master Idee xlsx e salvate in 02_Generazione_Idee.
Causa: routine auto-disabilitata per mancato accesso al repo GitHub.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -23,8 +23,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -302,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -380,7 +380,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -390,6 +390,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -835,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R69"/>
+  <dimension ref="A1:R85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="2"/>
@@ -4013,7 +4016,7 @@
       <c r="R61" s="17" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="31" t="n">
+      <c r="A62" s="35" t="n">
         <v>46168</v>
       </c>
       <c r="B62" s="32" t="inlineStr">
@@ -4071,7 +4074,7 @@
       <c r="R62" s="32" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="31" t="n">
+      <c r="A63" s="35" t="n">
         <v>46168</v>
       </c>
       <c r="B63" s="32" t="inlineStr">
@@ -4129,7 +4132,7 @@
       <c r="R63" s="32" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="31" t="n">
+      <c r="A64" s="35" t="n">
         <v>46168</v>
       </c>
       <c r="B64" s="32" t="inlineStr">
@@ -4187,7 +4190,7 @@
       <c r="R64" s="32" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="31" t="n">
+      <c r="A65" s="35" t="n">
         <v>46168</v>
       </c>
       <c r="B65" s="32" t="inlineStr">
@@ -4245,7 +4248,7 @@
       <c r="R65" s="32" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="31" t="n">
+      <c r="A66" s="35" t="n">
         <v>46169</v>
       </c>
       <c r="B66" s="32" t="inlineStr">
@@ -4303,7 +4306,7 @@
       <c r="R66" s="32" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="31" t="n">
+      <c r="A67" s="35" t="n">
         <v>46169</v>
       </c>
       <c r="B67" s="32" t="inlineStr">
@@ -4361,7 +4364,7 @@
       <c r="R67" s="32" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="31" t="n">
+      <c r="A68" s="35" t="n">
         <v>46169</v>
       </c>
       <c r="B68" s="32" t="inlineStr">
@@ -4419,7 +4422,7 @@
       <c r="R68" s="32" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="31" t="n">
+      <c r="A69" s="35" t="n">
         <v>46169</v>
       </c>
       <c r="B69" s="32" t="inlineStr">
@@ -4475,6 +4478,934 @@
       <c r="P69" s="32" t="n"/>
       <c r="Q69" s="32" t="n"/>
       <c r="R69" s="32" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="35" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B70" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C70" s="33" t="inlineStr">
+        <is>
+          <t>Acqua calda dal sole anche d'inverno: il solare termico oggi funziona così</t>
+        </is>
+      </c>
+      <c r="D70" s="33" t="inlineStr">
+        <is>
+          <t>Confonde solare termico e fotovoltaico, pensa sia tecnologia vecchia e che d'inverno non serva a niente.</t>
+        </is>
+      </c>
+      <c r="E70" s="33" t="inlineStr">
+        <is>
+          <t>60 secondi su come il pannello solare termico scalda l'acqua direttamente. Impianto reale che lavora anche con cielo coperto e in giornate fredde. Quando ha senso e quando no.</t>
+        </is>
+      </c>
+      <c r="F70" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Solari</t>
+        </is>
+      </c>
+      <c r="G70" s="32" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H70" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J70" s="32" t="n"/>
+      <c r="K70" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L70" s="32" t="n"/>
+      <c r="M70" s="33" t="n"/>
+      <c r="N70" s="32" t="n"/>
+      <c r="O70" s="32" t="n"/>
+      <c r="P70" s="32" t="n"/>
+      <c r="Q70" s="32" t="n"/>
+      <c r="R70" s="32" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="35" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B71" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C71" s="33" t="inlineStr">
+        <is>
+          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
+        </is>
+      </c>
+      <c r="D71" s="33" t="inlineStr">
+        <is>
+          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
+        </is>
+      </c>
+      <c r="E71" s="33" t="inlineStr">
+        <is>
+          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
+        </is>
+      </c>
+      <c r="F71" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H71" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J71" s="32" t="n"/>
+      <c r="K71" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L71" s="32" t="n"/>
+      <c r="M71" s="33" t="n"/>
+      <c r="N71" s="32" t="n"/>
+      <c r="O71" s="32" t="n"/>
+      <c r="P71" s="32" t="n"/>
+      <c r="Q71" s="32" t="n"/>
+      <c r="R71" s="32" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="35" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B72" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C72" s="33" t="inlineStr">
+        <is>
+          <t>Tetto in eternit? Cosa sapere prima di mettere il fotovoltaico</t>
+        </is>
+      </c>
+      <c r="D72" s="33" t="inlineStr">
+        <is>
+          <t>Vuole il fotovoltaico ma scopre di avere l'eternit sul tetto e pensa che non si possa fare nulla.</t>
+        </is>
+      </c>
+      <c r="E72" s="33" t="inlineStr">
+        <is>
+          <t>Serve la bonifica prima dell'installazione, ci sono incentivi dedicati a chi rimuove l'amianto e mette pannelli, e cosa controllare prima del sopralluogo.</t>
+        </is>
+      </c>
+      <c r="F72" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>Domanda burocratica / normativa</t>
+        </is>
+      </c>
+      <c r="H72" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J72" s="32" t="n"/>
+      <c r="K72" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L72" s="32" t="n"/>
+      <c r="M72" s="33" t="n"/>
+      <c r="N72" s="32" t="n"/>
+      <c r="O72" s="32" t="n"/>
+      <c r="P72" s="32" t="n"/>
+      <c r="Q72" s="32" t="n"/>
+      <c r="R72" s="32" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="35" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B73" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C73" s="33" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo: dopo 10 anni che capacità ha davvero?</t>
+        </is>
+      </c>
+      <c r="D73" s="33" t="inlineStr">
+        <is>
+          <t>Teme che la batteria diventi un costo a perdere e che dopo la garanzia debba buttare tutto.</t>
+        </is>
+      </c>
+      <c r="E73" s="33" t="inlineStr">
+        <is>
+          <t>Cosa dice la garanzia tipica del produttore, quanto cala la capacità nel tempo, come capire se conviene sostituirla o tenerla qualche anno in più. Esempio di impianto reale.</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>Garanzie / Assistenza post-vendita</t>
+        </is>
+      </c>
+      <c r="H73" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J73" s="32" t="n"/>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="n"/>
+      <c r="M73" s="33" t="n"/>
+      <c r="N73" s="32" t="n"/>
+      <c r="O73" s="32" t="n"/>
+      <c r="P73" s="32" t="n"/>
+      <c r="Q73" s="32" t="n"/>
+      <c r="R73" s="32" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="35" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B74" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C74" s="33" t="inlineStr">
+        <is>
+          <t>Stufa a pellet: ogni quanto va davvero fatta la manutenzione?</t>
+        </is>
+      </c>
+      <c r="D74" s="33" t="inlineStr">
+        <is>
+          <t>La rimandano per risparmiare e poi pagano riparazioni più care.</t>
+        </is>
+      </c>
+      <c r="E74" s="33" t="inlineStr">
+        <is>
+          <t>Calendario semplice della manutenzione annuale: cosa controlla il tecnico, cosa puoi fare tu, cosa succede se salti un anno.</t>
+        </is>
+      </c>
+      <c r="F74" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Stufe</t>
+        </is>
+      </c>
+      <c r="G74" s="32" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H74" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J74" s="32" t="n"/>
+      <c r="K74" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L74" s="32" t="n"/>
+      <c r="M74" s="33" t="n"/>
+      <c r="N74" s="32" t="n"/>
+      <c r="O74" s="32" t="n"/>
+      <c r="P74" s="32" t="n"/>
+      <c r="Q74" s="32" t="n"/>
+      <c r="R74" s="32" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="35" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B75" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C75" s="33" t="inlineStr">
+        <is>
+          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
+        </is>
+      </c>
+      <c r="D75" s="33" t="inlineStr">
+        <is>
+          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
+        </is>
+      </c>
+      <c r="E75" s="33" t="inlineStr">
+        <is>
+          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
+        </is>
+      </c>
+      <c r="F75" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G75" s="32" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H75" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I75" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J75" s="32" t="n"/>
+      <c r="K75" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L75" s="32" t="n"/>
+      <c r="M75" s="33" t="n"/>
+      <c r="N75" s="32" t="n"/>
+      <c r="O75" s="32" t="n"/>
+      <c r="P75" s="32" t="n"/>
+      <c r="Q75" s="32" t="n"/>
+      <c r="R75" s="32" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="35" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B76" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C76" s="33" t="inlineStr">
+        <is>
+          <t>Cucina economica a legna: dove si può davvero installare?</t>
+        </is>
+      </c>
+      <c r="D76" s="33" t="inlineStr">
+        <is>
+          <t>Pensano serva una grande cucina rustica e ci rinunciano in partenza.</t>
+        </is>
+      </c>
+      <c r="E76" s="33" t="inlineStr">
+        <is>
+          <t>3 case reali dove l'abbiamo installata: villetta, casa di campagna, baita. Cosa serve sopra (canna fumaria) e sotto (pavimento).</t>
+        </is>
+      </c>
+      <c r="F76" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Cucine economiche</t>
+        </is>
+      </c>
+      <c r="G76" s="32" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H76" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I76" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J76" s="32" t="n"/>
+      <c r="K76" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L76" s="32" t="n"/>
+      <c r="M76" s="33" t="n"/>
+      <c r="N76" s="32" t="n"/>
+      <c r="O76" s="32" t="n"/>
+      <c r="P76" s="32" t="n"/>
+      <c r="Q76" s="32" t="n"/>
+      <c r="R76" s="32" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="35" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B77" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C77" s="33" t="inlineStr">
+        <is>
+          <t>Chi siamo: la squadra che entra davvero a casa tua</t>
+        </is>
+      </c>
+      <c r="D77" s="33" t="inlineStr">
+        <is>
+          <t>Hanno paura di non sapere chi gli arriva in casa e rimandano il sopralluogo.</t>
+        </is>
+      </c>
+      <c r="E77" s="33" t="inlineStr">
+        <is>
+          <t>Presentiamo i tecnici che fanno installazione e manutenzione: volti, ruoli, da quanti anni lavorano insieme. Niente discorsi aziendali.</t>
+        </is>
+      </c>
+      <c r="F77" s="32" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G77" s="32" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H77" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I77" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J77" s="32" t="n"/>
+      <c r="K77" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L77" s="32" t="n"/>
+      <c r="M77" s="33" t="n"/>
+      <c r="N77" s="32" t="n"/>
+      <c r="O77" s="32" t="n"/>
+      <c r="P77" s="32" t="n"/>
+      <c r="Q77" s="32" t="n"/>
+      <c r="R77" s="32" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B78" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C78" s="33" t="inlineStr">
+        <is>
+          <t>Solare Italiano: in quali zone interveniamo davvero?</t>
+        </is>
+      </c>
+      <c r="D78" s="33" t="inlineStr">
+        <is>
+          <t>Non sa se l'azienda copre la sua zona e non chiede per paura di perdere tempo.</t>
+        </is>
+      </c>
+      <c r="E78" s="33" t="inlineStr">
+        <is>
+          <t>Mappa rapida delle aree in cui interveniamo per installazione e manutenzione. Se sei al limite, scrivici lo stesso, controlliamo.</t>
+        </is>
+      </c>
+      <c r="F78" s="32" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G78" s="32" t="inlineStr">
+        <is>
+          <t>Sedi / Zone operative</t>
+        </is>
+      </c>
+      <c r="H78" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J78" s="32" t="n"/>
+      <c r="K78" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L78" s="32" t="n"/>
+      <c r="M78" s="33" t="n"/>
+      <c r="N78" s="32" t="n"/>
+      <c r="O78" s="32" t="n"/>
+      <c r="P78" s="32" t="n"/>
+      <c r="Q78" s="32" t="n"/>
+      <c r="R78" s="32" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B79" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C79" s="33" t="inlineStr">
+        <is>
+          <t>Termostufa a pellet: dove può andare davvero in casa tua?</t>
+        </is>
+      </c>
+      <c r="D79" s="33" t="inlineStr">
+        <is>
+          <t>Pensa serva una stanza tecnica come per la caldaia e rinuncia in partenza.</t>
+        </is>
+      </c>
+      <c r="E79" s="33" t="inlineStr">
+        <is>
+          <t>3 posizioni tipiche in cui una termostufa può andare in una casa esistente, con ingombri reali e cosa serve sopra (canna fumaria) e sotto (impianto).</t>
+        </is>
+      </c>
+      <c r="F79" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Termostufe</t>
+        </is>
+      </c>
+      <c r="G79" s="32" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H79" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J79" s="32" t="n"/>
+      <c r="K79" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L79" s="32" t="n"/>
+      <c r="M79" s="33" t="n"/>
+      <c r="N79" s="32" t="n"/>
+      <c r="O79" s="32" t="n"/>
+      <c r="P79" s="32" t="n"/>
+      <c r="Q79" s="32" t="n"/>
+      <c r="R79" s="32" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B80" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C80" s="33" t="inlineStr">
+        <is>
+          <t>La pompa di calore fa rumore? Cosa controllare prima di installarla</t>
+        </is>
+      </c>
+      <c r="D80" s="33" t="inlineStr">
+        <is>
+          <t>Paura che l'unità esterna disturbi vicini e camera da letto, blocca la decisione.</t>
+        </is>
+      </c>
+      <c r="E80" s="33" t="inlineStr">
+        <is>
+          <t>Cosa significano i dB dichiarati, dove posizionare l'unità esterna in una casa singola o bifamiliare e cosa succede di notte in modalità silenziosa.</t>
+        </is>
+      </c>
+      <c r="F80" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G80" s="32" t="inlineStr">
+        <is>
+          <t>Paura / Scetticismo</t>
+        </is>
+      </c>
+      <c r="H80" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J80" s="32" t="n"/>
+      <c r="K80" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L80" s="32" t="n"/>
+      <c r="M80" s="33" t="n"/>
+      <c r="N80" s="32" t="n"/>
+      <c r="O80" s="32" t="n"/>
+      <c r="P80" s="32" t="n"/>
+      <c r="Q80" s="32" t="n"/>
+      <c r="R80" s="32" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B81" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C81" s="33" t="inlineStr">
+        <is>
+          <t>Solare termico o scaldabagno elettrico: cosa scegliere per l'acqua calda?</t>
+        </is>
+      </c>
+      <c r="D81" s="33" t="inlineStr">
+        <is>
+          <t>Confonde solare termico e fotovoltaico e alla fine resta col vecchio scaldabagno elettrico.</t>
+        </is>
+      </c>
+      <c r="E81" s="33" t="inlineStr">
+        <is>
+          <t>La differenza tra solare termico e scaldabagno elettrico per l'acqua calda sanitaria e in quali case il solare termico ha davvero senso.</t>
+        </is>
+      </c>
+      <c r="F81" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Solari</t>
+        </is>
+      </c>
+      <c r="G81" s="32" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H81" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J81" s="32" t="n"/>
+      <c r="K81" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L81" s="32" t="n"/>
+      <c r="M81" s="33" t="n"/>
+      <c r="N81" s="32" t="n"/>
+      <c r="O81" s="32" t="n"/>
+      <c r="P81" s="32" t="n"/>
+      <c r="Q81" s="32" t="n"/>
+      <c r="R81" s="32" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B82" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C82" s="33" t="inlineStr">
+        <is>
+          <t>Inserto a pellet: posso usare la canna fumaria che ho già?</t>
+        </is>
+      </c>
+      <c r="D82" s="33" t="inlineStr">
+        <is>
+          <t>Pensano di dover rifare tutto da capo e rinunciano prima ancora di chiedere.</t>
+        </is>
+      </c>
+      <c r="E82" s="33" t="inlineStr">
+        <is>
+          <t>I 3 casi che troviamo nelle case: canna a norma, da intubare, da rifare. Esempio reale con cosa cambia per il cliente.</t>
+        </is>
+      </c>
+      <c r="F82" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G82" s="32" t="inlineStr">
+        <is>
+          <t>Domanda burocratica / normativa</t>
+        </is>
+      </c>
+      <c r="H82" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J82" s="32" t="n"/>
+      <c r="K82" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L82" s="32" t="n"/>
+      <c r="M82" s="33" t="n"/>
+      <c r="N82" s="32" t="n"/>
+      <c r="O82" s="32" t="n"/>
+      <c r="P82" s="32" t="n"/>
+      <c r="Q82" s="32" t="n"/>
+      <c r="R82" s="32" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B83" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C83" s="33" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo: dove la mettiamo a casa tua?</t>
+        </is>
+      </c>
+      <c r="D83" s="33" t="inlineStr">
+        <is>
+          <t>Pensano di non avere lo spazio giusto e bocciano l'idea prima del preventivo.</t>
+        </is>
+      </c>
+      <c r="E83" s="33" t="inlineStr">
+        <is>
+          <t>3 posizioni tipiche dove la installiamo (garage, lavanderia, parete esterna) con misure reali e cosa serve attorno.</t>
+        </is>
+      </c>
+      <c r="F83" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G83" s="32" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H83" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I83" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J83" s="32" t="n"/>
+      <c r="K83" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L83" s="32" t="n"/>
+      <c r="M83" s="33" t="n"/>
+      <c r="N83" s="32" t="n"/>
+      <c r="O83" s="32" t="n"/>
+      <c r="P83" s="32" t="n"/>
+      <c r="Q83" s="32" t="n"/>
+      <c r="R83" s="32" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B84" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C84" s="33" t="inlineStr">
+        <is>
+          <t>Colonnina di ricarica a casa: quanto tempo passa dal sopralluogo all'auto attaccata?</t>
+        </is>
+      </c>
+      <c r="D84" s="33" t="inlineStr">
+        <is>
+          <t>Pensano sia un'opera lunga e burocratica e rimandano la decisione.</t>
+        </is>
+      </c>
+      <c r="E84" s="33" t="inlineStr">
+        <is>
+          <t>Tappa per tappa: sopralluogo, preventivo, installazione, attivazione. Tempi reali su un caso recente, senza promesse gonfiate.</t>
+        </is>
+      </c>
+      <c r="F84" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G84" s="32" t="inlineStr">
+        <is>
+          <t>Sopralluogo</t>
+        </is>
+      </c>
+      <c r="H84" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I84" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J84" s="32" t="n"/>
+      <c r="K84" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L84" s="32" t="n"/>
+      <c r="M84" s="33" t="n"/>
+      <c r="N84" s="32" t="n"/>
+      <c r="O84" s="32" t="n"/>
+      <c r="P84" s="32" t="n"/>
+      <c r="Q84" s="32" t="n"/>
+      <c r="R84" s="32" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="35" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B85" s="32" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C85" s="33" t="inlineStr">
+        <is>
+          <t>Termocamino: come fa ad arrivare anche ai termosifoni del piano di sopra?</t>
+        </is>
+      </c>
+      <c r="D85" s="33" t="inlineStr">
+        <is>
+          <t>Pensano non basti per scaldare tutta la casa e non ci credono.</t>
+        </is>
+      </c>
+      <c r="E85" s="33" t="inlineStr">
+        <is>
+          <t>Schema semplice del circuito (focolare, scambiatore, puffer, termosifoni) raccontato senza tecnicismi, con un'installazione reale.</t>
+        </is>
+      </c>
+      <c r="F85" s="32" t="inlineStr">
+        <is>
+          <t>Prodotto - Termocamini</t>
+        </is>
+      </c>
+      <c r="G85" s="32" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H85" s="33" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I85" s="32" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J85" s="32" t="n"/>
+      <c r="K85" s="32" t="inlineStr">
+        <is>
+          <t>Maggio</t>
+        </is>
+      </c>
+      <c r="L85" s="32" t="n"/>
+      <c r="M85" s="33" t="n"/>
+      <c r="N85" s="32" t="n"/>
+      <c r="O85" s="32" t="n"/>
+      <c r="P85" s="32" t="n"/>
+      <c r="Q85" s="32" t="n"/>
+      <c r="R85" s="32" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:M61">

</xml_diff>

<commit_message>
Master Idee 2026-07-13: nuove idee notturne
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -23,8 +23,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -351,7 +351,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -361,6 +361,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5206,7 +5209,7 @@
       <c r="J97" s="17" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="29" t="n">
+      <c r="A98" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B98" s="30" t="inlineStr">
@@ -5252,7 +5255,7 @@
       <c r="J98" s="30" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="29" t="n">
+      <c r="A99" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B99" s="30" t="inlineStr">
@@ -5298,7 +5301,7 @@
       <c r="J99" s="30" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="29" t="n">
+      <c r="A100" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B100" s="30" t="inlineStr">
@@ -5344,7 +5347,7 @@
       <c r="J100" s="30" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="29" t="n">
+      <c r="A101" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B101" s="30" t="inlineStr">
@@ -5390,7 +5393,7 @@
       <c r="J101" s="30" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="29" t="n">
+      <c r="A102" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B102" s="30" t="inlineStr">
@@ -5436,7 +5439,7 @@
       <c r="J102" s="30" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="29" t="n">
+      <c r="A103" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B103" s="30" t="inlineStr">
@@ -5482,7 +5485,7 @@
       <c r="J103" s="30" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="29" t="n">
+      <c r="A104" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B104" s="30" t="inlineStr">
@@ -5528,7 +5531,7 @@
       <c r="J104" s="30" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="29" t="n">
+      <c r="A105" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B105" s="30" t="inlineStr">
@@ -5574,7 +5577,7 @@
       <c r="J105" s="30" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="29" t="n">
+      <c r="A106" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B106" s="30" t="inlineStr">
@@ -5620,7 +5623,7 @@
       <c r="J106" s="30" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="29" t="n">
+      <c r="A107" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B107" s="30" t="inlineStr">
@@ -5666,7 +5669,7 @@
       <c r="J107" s="30" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="29" t="n">
+      <c r="A108" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B108" s="30" t="inlineStr">
@@ -5712,7 +5715,7 @@
       <c r="J108" s="30" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="29" t="n">
+      <c r="A109" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B109" s="30" t="inlineStr">
@@ -5758,7 +5761,7 @@
       <c r="J109" s="30" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="29" t="n">
+      <c r="A110" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B110" s="30" t="inlineStr">
@@ -5804,7 +5807,7 @@
       <c r="J110" s="30" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="29" t="n">
+      <c r="A111" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B111" s="30" t="inlineStr">
@@ -5850,7 +5853,7 @@
       <c r="J111" s="30" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="29" t="n">
+      <c r="A112" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B112" s="30" t="inlineStr">
@@ -5896,7 +5899,7 @@
       <c r="J112" s="30" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="29" t="n">
+      <c r="A113" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B113" s="30" t="inlineStr">
@@ -5942,7 +5945,7 @@
       <c r="J113" s="30" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="29" t="n">
+      <c r="A114" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B114" s="30" t="inlineStr">
@@ -5988,7 +5991,7 @@
       <c r="J114" s="30" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="29" t="n">
+      <c r="A115" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B115" s="30" t="inlineStr">
@@ -6034,7 +6037,7 @@
       <c r="J115" s="30" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="29" t="n">
+      <c r="A116" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B116" s="30" t="inlineStr">
@@ -6080,7 +6083,7 @@
       <c r="J116" s="30" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="29" t="n">
+      <c r="A117" s="33" t="n">
         <v>46214</v>
       </c>
       <c r="B117" s="30" t="inlineStr">
@@ -6125,11 +6128,236 @@
       </c>
       <c r="J117" s="30" t="n"/>
     </row>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
+    <row r="118">
+      <c r="A118" s="33" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B118" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C118" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: funziona davvero quando fuori ci sono -5°C?</t>
+        </is>
+      </c>
+      <c r="D118" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito che si blocca col gelo — vero o mito?</t>
+        </is>
+      </c>
+      <c r="E118" s="31" t="inlineStr">
+        <is>
+          <t>Sfatiamo il mito più diffuso: molte pompe di calore moderne lavorano fino a -20°C. Il reel mostra cosa succede realmente all'unità esterna in una notte gelata e perché la casa rimane calda.</t>
+        </is>
+      </c>
+      <c r="F118" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G118" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H118" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I118" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J118" s="30" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="33" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B119" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C119" s="31" t="inlineStr">
+        <is>
+          <t>Stufa a pellet: 3 segnali che ti dice che è ora di cambiarla</t>
+        </is>
+      </c>
+      <c r="D119" s="31" t="inlineStr">
+        <is>
+          <t>La mia stufa ha 8 anni e scalda ancora — la tengo o la cambio?</t>
+        </is>
+      </c>
+      <c r="E119" s="31" t="inlineStr">
+        <is>
+          <t>Non aspettare il guasto totale. Il reel elenca i tre sintomi che indicano che la stufa sta per cedere e perché intervenire prima conviene in termini di efficienza e incentivi disponibili.</t>
+        </is>
+      </c>
+      <c r="F119" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Stufe</t>
+        </is>
+      </c>
+      <c r="G119" s="30" t="inlineStr">
+        <is>
+          <t>Quando sostituirlo</t>
+        </is>
+      </c>
+      <c r="H119" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I119" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J119" s="30" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="33" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B120" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C120" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 2025: chi può richiederlo e per quali prodotti?</t>
+        </is>
+      </c>
+      <c r="D120" s="31" t="inlineStr">
+        <is>
+          <t>Sento parlare di Conto Termico ma non so se spetta anche a me</t>
+        </is>
+      </c>
+      <c r="E120" s="31" t="inlineStr">
+        <is>
+          <t>Spiegazione semplice: cos'è il Conto Termico, chi ha diritto (privati inclusi), quali impianti coprono e come si fa domanda senza un commercialista. Pensato per chi ha sentito il nome ma non ha mai capito come funziona.</t>
+        </is>
+      </c>
+      <c r="F120" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G120" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H120" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I120" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J120" s="30" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="33" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B121" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C121" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a legna in condominio: si può installare o è vietato?</t>
+        </is>
+      </c>
+      <c r="D121" s="31" t="inlineStr">
+        <is>
+          <t>Vogrei il fuoco vero in casa ma abito in un palazzo — è impossibile?</t>
+        </is>
+      </c>
+      <c r="E121" s="31" t="inlineStr">
+        <is>
+          <t>Moltissimi rinunciano senza nemmeno chiedere. Il reel spiega le condizioni che rendono possibile l'installazione di un inserto in un appartamento (canna fumaria dedicata, regolamento condominiale, norme vigenti) e quando invece non si può.</t>
+        </is>
+      </c>
+      <c r="F121" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G121" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H121" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I121" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J121" s="30" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="33" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B122" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C122" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a gas vs pompa di calore: come scelgo quella giusta per la mia casa?</t>
+        </is>
+      </c>
+      <c r="D122" s="31" t="inlineStr">
+        <is>
+          <t>Mi dicono di passare alla pompa di calore ma ho sempre usato il gas — come decido?</t>
+        </is>
+      </c>
+      <c r="E122" s="31" t="inlineStr">
+        <is>
+          <t>Non esiste la scelta universalmente migliore. Il reel guida in modo semplice: tipo di abitazione, clima della zona, impianto radiante o termosifoni — un mini-percorso decisionale per il proprietario di casa non tecnico.</t>
+        </is>
+      </c>
+      <c r="F122" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G122" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H122" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I122" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J122" s="30" t="n"/>
+    </row>
     <row r="123"/>
     <row r="124"/>
     <row r="125"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-14: nuove idee notturne
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -6358,883 +6358,236 @@
       </c>
       <c r="J122" s="30" t="n"/>
     </row>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
+    <row r="123">
+      <c r="A123" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B123" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C123" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: quanto spazio serve davvero per l'unità esterna?</t>
+        </is>
+      </c>
+      <c r="D123" s="31" t="inlineStr">
+        <is>
+          <t>Voglio la pompa di calore ma ho paura che il motore esterno non ci stia</t>
+        </is>
+      </c>
+      <c r="E123" s="31" t="inlineStr">
+        <is>
+          <t>Mostriamo con esempi reali quanto spazio occupa un'unità esterna (balcone stretto, nicchia, parete laterale). Sfatiamo la paura che servano grandi spazi.</t>
+        </is>
+      </c>
+      <c r="F123" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G123" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H123" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I123" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J123" s="30" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B124" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C124" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a pellet: il mio camino è abbastanza grande?</t>
+        </is>
+      </c>
+      <c r="D124" s="31" t="inlineStr">
+        <is>
+          <t>Ho un vecchio camino e non so se posso mettere un inserto a pellet senza demolire tutto</t>
+        </is>
+      </c>
+      <c r="E124" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo le misure di apertura minima e massima per un inserto a pellet. Mostriamo anche cosa controllare sulla canna fumaria prima di chiamarci.</t>
+        </is>
+      </c>
+      <c r="F124" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G124" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H124" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I124" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J124" s="30" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B125" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C125" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 2026: dal sopralluogo ai soldi sul conto, quanto tempo passa?</t>
+        </is>
+      </c>
+      <c r="D125" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito parlare del Conto Termico ma ho paura che i soldi non arrivino mai o che ci voglia un anno</t>
+        </is>
+      </c>
+      <c r="E125" s="31" t="inlineStr">
+        <is>
+          <t>Illustriamo passo per passo la tempistica reale: sopralluogo → lavori → domanda GSE → pagamento. Rassicurazione concreta su tempi medi.</t>
+        </is>
+      </c>
+      <c r="F125" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G125" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H125" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I125" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J125" s="30" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B126" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C126" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: la lasci accesa la notte o la spegni? L'errore che fa salire la bolletta</t>
+        </is>
+      </c>
+      <c r="D126" s="31" t="inlineStr">
+        <is>
+          <t>Uso la pompa di calore da mesi ma non so se sto sbagliando qualcosa nella gestione quotidiana</t>
+        </is>
+      </c>
+      <c r="E126" s="31" t="inlineStr">
+        <is>
+          <t>Sveliamo il contro-intuitivo: spegnerla e riaccenderla ogni giorno consuma più di tenerla a temperatura bassa di notte. Concetto di 'inerzia termica' spiegato senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F126" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G126" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H126" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I126" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J126" s="30" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B127" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C127" s="31" t="inlineStr">
+        <is>
+          <t>Stufa a pellet rumorosa di notte: è normale o c'è qualcosa che non va?</t>
+        </is>
+      </c>
+      <c r="D127" s="31" t="inlineStr">
+        <is>
+          <t>La mia stufa a pellet fa rumori strani la sera e non so se chiamare il tecnico o se è tutto normale</t>
+        </is>
+      </c>
+      <c r="E127" s="31" t="inlineStr">
+        <is>
+          <t>Distinguiamo i rumori normali (coclea, ventola di scarico) da quelli che richiedono assistenza (bruciatore, caricamento irregolare). Regola pratica: quando chiamare vs quando no.</t>
+        </is>
+      </c>
+      <c r="F127" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Stufe</t>
+        </is>
+      </c>
+      <c r="G127" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H127" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I127" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J127" s="30" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Shortlist 15 2026-07-14: idee riportate nel Master
8 Confermate → Produzione, 1 Posticipata → Nuova, 3 Scartate rimosse.
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J127"/>
+  <dimension ref="A1:J136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -6587,6 +6587,400 @@
         </is>
       </c>
       <c r="J127" s="30" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="33" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B128" s="30" t="inlineStr">
+        <is>
+          <t>Topic mese</t>
+        </is>
+      </c>
+      <c r="C128" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
+        </is>
+      </c>
+      <c r="D128" s="31" t="inlineStr">
+        <is>
+          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
+        </is>
+      </c>
+      <c r="E128" s="31" t="inlineStr">
+        <is>
+          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
+        </is>
+      </c>
+      <c r="F128" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G128" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H128" s="31" t="inlineStr">
+        <is>
+          <t>Topic mese: climatizzazione estiva privati</t>
+        </is>
+      </c>
+      <c r="I128" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J128" s="30" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="33" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B129" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C129" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
+        </is>
+      </c>
+      <c r="D129" s="31" t="inlineStr">
+        <is>
+          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
+        </is>
+      </c>
+      <c r="E129" s="31" t="inlineStr">
+        <is>
+          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
+        </is>
+      </c>
+      <c r="F129" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G129" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H129" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I129" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J129" s="30" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="33" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B130" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C130" s="31" t="inlineStr">
+        <is>
+          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
+        </is>
+      </c>
+      <c r="D130" s="31" t="inlineStr">
+        <is>
+          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
+        </is>
+      </c>
+      <c r="E130" s="31" t="inlineStr">
+        <is>
+          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
+        </is>
+      </c>
+      <c r="F130" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G130" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H130" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I130" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J130" s="30" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="33" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B131" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C131" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore: come scelgo il modello giusto per casa mia?</t>
+        </is>
+      </c>
+      <c r="D131" s="31" t="inlineStr">
+        <is>
+          <t>Non sa da dove partire nella scelta — marca, BTU, classe energetica gli sembrano tutti uguali</t>
+        </is>
+      </c>
+      <c r="E131" s="31" t="inlineStr">
+        <is>
+          <t>I 3 parametri pratici che fanno la differenza nella scelta di un climatizzatore, spiegati senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F131" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G131" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H131" s="31" t="inlineStr"/>
+      <c r="I131" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J131" s="30" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="33" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B132" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C132" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico: copre anche la sostituzione del vecchio condizionatore?</t>
+        </is>
+      </c>
+      <c r="D132" s="31" t="inlineStr">
+        <is>
+          <t>Pensa che il Conto Termico valga solo per caldaie e pompe di calore, non per i climatizzatori</t>
+        </is>
+      </c>
+      <c r="E132" s="31" t="inlineStr">
+        <is>
+          <t>Quando la rottamazione di un vecchio climatizzatore dà diritto al Conto Termico e come richiederlo.</t>
+        </is>
+      </c>
+      <c r="F132" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G132" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica / normativa</t>
+        </is>
+      </c>
+      <c r="H132" s="31" t="inlineStr"/>
+      <c r="I132" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J132" s="30" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="33" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B133" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C133" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: non devi rifare tutto l'impianto. E il fotovoltaico può aiutarti.</t>
+        </is>
+      </c>
+      <c r="D133" s="31" t="inlineStr">
+        <is>
+          <t>Rinunciano alla PdC convinti serva un cantiere enorme — non sanno che si può partire in piccolo</t>
+        </is>
+      </c>
+      <c r="E133" s="31" t="inlineStr">
+        <is>
+          <t>Perché in molti casi basta un impianto più contenuto, e come il fotovoltaico aiuta a sostenere il consumo elettrico della PdC.</t>
+        </is>
+      </c>
+      <c r="F133" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G133" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H133" s="31" t="inlineStr"/>
+      <c r="I133" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J133" s="30" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="33" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B134" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C134" s="31" t="inlineStr">
+        <is>
+          <t>Con cosa arriviamo a casa tua: i mezzi della squadra Solare Italiano</t>
+        </is>
+      </c>
+      <c r="D134" s="31" t="inlineStr">
+        <is>
+          <t>Non sa quanta preparazione professionale c'è dietro ogni intervento</t>
+        </is>
+      </c>
+      <c r="E134" s="31" t="inlineStr">
+        <is>
+          <t>Ripresa dei furgoni e della piattaforma aerea per mostrare l'attrezzatura sul campo. Nessuna improvvisazione.</t>
+        </is>
+      </c>
+      <c r="F134" s="30" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G134" s="30" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H134" s="31" t="inlineStr"/>
+      <c r="I134" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J134" s="30" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="33" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B135" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C135" s="31" t="inlineStr">
+        <is>
+          <t>Cosa facciamo prima di venire da te: la preparazione del furgone</t>
+        </is>
+      </c>
+      <c r="D135" s="31" t="inlineStr">
+        <is>
+          <t>Non immagina il lavoro di preparazione dietro ogni uscita — pensa che i tecnici partano senza organizzazione</t>
+        </is>
+      </c>
+      <c r="E135" s="31" t="inlineStr">
+        <is>
+          <t>Il team che carica il furgone, controlla gli strumenti e prepara il materiale prima di partire. Dietro le quinte della professionalità.</t>
+        </is>
+      </c>
+      <c r="F135" s="30" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="G135" s="30" t="inlineStr">
+        <is>
+          <t>Dietro le quinte squadra</t>
+        </is>
+      </c>
+      <c r="H135" s="31" t="inlineStr"/>
+      <c r="I135" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J135" s="30" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="33" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B136" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C136" s="31" t="inlineStr">
+        <is>
+          <t>Chi siamo: la squadra che entra davvero a casa tua</t>
+        </is>
+      </c>
+      <c r="D136" s="31" t="inlineStr">
+        <is>
+          <t>Hanno paura di non sapere chi gli arriva in casa e rimandano il sopralluogo.</t>
+        </is>
+      </c>
+      <c r="E136" s="31" t="inlineStr">
+        <is>
+          <t>Presentiamo i tecnici che fanno installazione e manutenzione: volti, ruoli, da quanti anni lavorano insieme. Niente discorsi aziendali.</t>
+        </is>
+      </c>
+      <c r="F136" s="30" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G136" s="30" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H136" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I136" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J136" s="30" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>
@@ -6725,41 +7119,41 @@
     </row>
     <row r="5" ht="32" customHeight="1" s="20">
       <c r="A5" s="16" t="n">
-        <v>46165</v>
+        <v>46163</v>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>Topic mese</t>
+          <t>Ideazione Claude</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
+          <t>Pompa di calore senza fotovoltaico: si può?</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
+          <t>Pensano che servano per forza insieme — rinviano l'acquisto</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
+          <t>Sì, si può. Ma c'è UN aspetto da considerare prima di partire senza FV.</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Errore comune</t>
+          <t>Confronto con alternative</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>Topic mese: climatizzazione estiva privati</t>
+          <t>Batch 20 idee — 21/05/2026</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
@@ -6768,46 +7162,46 @@
         </is>
       </c>
       <c r="J5" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" s="20">
       <c r="A6" s="16" t="n">
-        <v>46163</v>
+        <v>46165</v>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Ideazione Claude</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Pompa di calore senza fotovoltaico: si può?</t>
+          <t>Fotovoltaico senza batteria nel 2026: ha ancora senso?</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Pensano che servano per forza insieme — rinviano l'acquisto</t>
+          <t>Dopo Superbonus pensano che senza accumulo non valga più</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>Sì, si può. Ma c'è UN aspetto da considerare prima di partire senza FV.</t>
+          <t>Quando la batteria serve davvero, quando puoi aggiungerla dopo senza farti bloccare.</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
+          <t>Come scegliere il modello giusto</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Batch 20 idee — 21/05/2026</t>
+          <t>Generato automaticamente di notte</t>
         </is>
       </c>
       <c r="I6" s="17" t="inlineStr">
@@ -6825,27 +7219,27 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Scheduled Task</t>
+          <t>Topic mese</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Fotovoltaico senza batteria nel 2026: ha ancora senso?</t>
+          <t>Negozio surriscaldato d'estate: la verità sul climatizzatore commerciale</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Dopo Superbonus pensano che senza accumulo non valga più</t>
+          <t>Imprenditori pensano basti un climatizzatore qualsiasi, poi i clienti escono prima dal caldo</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>Quando la batteria serve davvero, quando puoi aggiungerla dopo senza farti bloccare.</t>
+          <t>Perché il climatizzatore commerciale è diverso da quello di casa, e cosa rischi col modello sbagliato.</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Fotovoltaici</t>
+          <t>Prodotto - Climatizzatore</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
@@ -6855,7 +7249,7 @@
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>Generato automaticamente di notte</t>
+          <t>Topic mese: climatizzazione B2B</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
@@ -6878,17 +7272,17 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Negozio surriscaldato d'estate: la verità sul climatizzatore commerciale</t>
+          <t>Climatizzatore in negozio o ufficio: cosa puoi detrarre come azienda?</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Imprenditori pensano basti un climatizzatore qualsiasi, poi i clienti escono prima dal caldo</t>
+          <t>Imprenditori non sanno se possono detrarre l'AC commerciale (e come)</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Perché il climatizzatore commerciale è diverso da quello di casa, e cosa rischi col modello sbagliato.</t>
+          <t>Differenza tra detrazione casa e ammortamento azienda per il climatizzatore commerciale.</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
@@ -6898,12 +7292,12 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Come scegliere il modello giusto</t>
+          <t>Incentivi</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Topic mese: climatizzazione B2B</t>
+          <t>Topic mese: climatizzazione B2B incentivi</t>
         </is>
       </c>
       <c r="I8" s="17" t="inlineStr">
@@ -6926,32 +7320,32 @@
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>Climatizzatore in negozio o ufficio: cosa puoi detrarre come azienda?</t>
+          <t>Pompa di calore: il momento per pensarci è giugno, non ottobre</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Imprenditori non sanno se possono detrarre l'AC commerciale (e come)</t>
+          <t>Aspettano l'autunno e arrivano in coda di stagione: installazione lunga, tempi stretti</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>Differenza tra detrazione casa e ammortamento azienda per il climatizzatore commerciale.</t>
+          <t>Perché chiedere preventivo a giugno per la PdC ti salva da liste d'attesa e installazione in piena stagione fredda.</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Incentivi</t>
+          <t>Quando sostituirlo</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Topic mese: climatizzazione B2B incentivi</t>
+          <t>Topic mese: pompe di calore</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
@@ -6974,27 +7368,27 @@
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>Pompa di calore: il momento per pensarci è giugno, non ottobre</t>
+          <t>Pompa di calore o climatizzatore? Non sono la stessa cosa (anche se si somigliano)</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>Aspettano l'autunno e arrivano in coda di stagione: installazione lunga, tempi stretti</t>
+          <t>Confondono i due prodotti e prendono quello sbagliato per le loro esigenze</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>Perché chiedere preventivo a giugno per la PdC ti salva da liste d'attesa e installazione in piena stagione fredda.</t>
+          <t>Differenza pratica tra PdC aria-acqua e climatizzatore aria-aria — quando ti serve quale.</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Quando sostituirlo</t>
+          <t>Confronto tra prodotti</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
@@ -7022,32 +7416,32 @@
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Pompa di calore o climatizzatore? Non sono la stessa cosa (anche se si somigliano)</t>
+          <t>Fotovoltaico senza batteria: rischi di 'regalare' metà energia alla rete</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>Confondono i due prodotti e prendono quello sbagliato per le loro esigenze</t>
+          <t>Non capiscono come funziona lo scambio sul posto e si perdono valore senza saperlo</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Differenza pratica tra PdC aria-acqua e climatizzatore aria-aria — quando ti serve quale.</t>
+          <t>Cos'è lo scambio sul posto e perché senza batteria una buona parte della produzione finisce alla rete a prezzo basso.</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Confronto tra prodotti</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Topic mese: pompe di calore</t>
+          <t>Topic mese: FV + batterie</t>
         </is>
       </c>
       <c r="I11" s="17" t="inlineStr">
@@ -7070,27 +7464,27 @@
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>Fotovoltaico senza batteria: rischi di 'regalare' metà energia alla rete</t>
+          <t>Batteria di accumulo: quando aggiungerla ha davvero senso (e quando puoi aspettare)</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Non capiscono come funziona lo scambio sul posto e si perdono valore senza saperlo</t>
+          <t>Scelta costosa che blocca l'acquisto del fotovoltaico — paralisi decisionale</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>Cos'è lo scambio sul posto e perché senza batteria una buona parte della produzione finisce alla rete a prezzo basso.</t>
+          <t>3 domande per capire se ti serve la batteria SUBITO o se conviene partire col solo FV e aggiungerla dopo.</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Fotovoltaici</t>
+          <t>Prodotto - Batterie di Accumulo</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Come scegliere il modello giusto</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
@@ -7107,54 +7501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1" s="20">
-      <c r="A13" s="16" t="n">
-        <v>46165</v>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Topic mese</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>Batteria di accumulo: quando aggiungerla ha davvero senso (e quando puoi aspettare)</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Scelta costosa che blocca l'acquisto del fotovoltaico — paralisi decisionale</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>3 domande per capire se ti serve la batteria SUBITO o se conviene partire col solo FV e aggiungerla dopo.</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>Prodotto - Batterie di Accumulo</t>
-        </is>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Come scegliere il modello giusto</t>
-        </is>
-      </c>
-      <c r="H13" s="18" t="inlineStr">
-        <is>
-          <t>Topic mese: FV + batterie</t>
-        </is>
-      </c>
-      <c r="I13" s="17" t="inlineStr">
-        <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J13" s="17" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="13" ht="32" customHeight="1" s="20"/>
     <row r="14" ht="32" customHeight="1" s="20"/>
     <row r="15" ht="32" customHeight="1" s="20"/>
     <row r="16" ht="48" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Shortlist 15 2026-07-15: idee riportate nel Master
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J136"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -6981,6 +6981,400 @@
         </is>
       </c>
       <c r="J136" s="30" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B137" s="30" t="inlineStr">
+        <is>
+          <t>Topic mese</t>
+        </is>
+      </c>
+      <c r="C137" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
+        </is>
+      </c>
+      <c r="D137" s="31" t="inlineStr">
+        <is>
+          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
+        </is>
+      </c>
+      <c r="E137" s="31" t="inlineStr">
+        <is>
+          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
+        </is>
+      </c>
+      <c r="F137" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G137" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H137" s="31" t="inlineStr">
+        <is>
+          <t>Topic mese: climatizzazione estiva privati</t>
+        </is>
+      </c>
+      <c r="I137" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J137" s="30" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B138" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C138" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
+        </is>
+      </c>
+      <c r="D138" s="31" t="inlineStr">
+        <is>
+          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
+        </is>
+      </c>
+      <c r="E138" s="31" t="inlineStr">
+        <is>
+          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
+        </is>
+      </c>
+      <c r="F138" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G138" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H138" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I138" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J138" s="30" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B139" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C139" s="31" t="inlineStr">
+        <is>
+          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
+        </is>
+      </c>
+      <c r="D139" s="31" t="inlineStr">
+        <is>
+          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
+        </is>
+      </c>
+      <c r="E139" s="31" t="inlineStr">
+        <is>
+          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
+        </is>
+      </c>
+      <c r="F139" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G139" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H139" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I139" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J139" s="30" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B140" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C140" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore: come scelgo il modello giusto per casa mia?</t>
+        </is>
+      </c>
+      <c r="D140" s="31" t="inlineStr">
+        <is>
+          <t>Non sa da dove partire nella scelta — marca, BTU, classe energetica gli sembrano tutti uguali</t>
+        </is>
+      </c>
+      <c r="E140" s="31" t="inlineStr">
+        <is>
+          <t>I 3 parametri pratici che fanno la differenza nella scelta di un climatizzatore, spiegati senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F140" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G140" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H140" s="31" t="inlineStr"/>
+      <c r="I140" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J140" s="30" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B141" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C141" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico: copre anche la sostituzione del vecchio condizionatore?</t>
+        </is>
+      </c>
+      <c r="D141" s="31" t="inlineStr">
+        <is>
+          <t>Pensa che il Conto Termico valga solo per caldaie e pompe di calore, non per i climatizzatori</t>
+        </is>
+      </c>
+      <c r="E141" s="31" t="inlineStr">
+        <is>
+          <t>Quando la rottamazione di un vecchio climatizzatore dà diritto al Conto Termico e come richiederlo.</t>
+        </is>
+      </c>
+      <c r="F141" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G141" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica / normativa</t>
+        </is>
+      </c>
+      <c r="H141" s="31" t="inlineStr"/>
+      <c r="I141" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J141" s="30" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B142" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C142" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: non devi rifare tutto l'impianto. E il fotovoltaico può aiutarti.</t>
+        </is>
+      </c>
+      <c r="D142" s="31" t="inlineStr">
+        <is>
+          <t>Rinunciano alla PdC convinti serva un cantiere enorme — non sanno che si può partire in piccolo</t>
+        </is>
+      </c>
+      <c r="E142" s="31" t="inlineStr">
+        <is>
+          <t>Perché in molti casi basta un impianto più contenuto, e come il fotovoltaico aiuta a sostenere il consumo elettrico della PdC.</t>
+        </is>
+      </c>
+      <c r="F142" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G142" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H142" s="31" t="inlineStr"/>
+      <c r="I142" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J142" s="30" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B143" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C143" s="31" t="inlineStr">
+        <is>
+          <t>Con cosa arriviamo a casa tua: i mezzi della squadra Solare Italiano</t>
+        </is>
+      </c>
+      <c r="D143" s="31" t="inlineStr">
+        <is>
+          <t>Non sa quanta preparazione professionale c'è dietro ogni intervento</t>
+        </is>
+      </c>
+      <c r="E143" s="31" t="inlineStr">
+        <is>
+          <t>Ripresa dei furgoni e della piattaforma aerea per mostrare l'attrezzatura sul campo. Nessuna improvvisazione.</t>
+        </is>
+      </c>
+      <c r="F143" s="30" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G143" s="30" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H143" s="31" t="inlineStr"/>
+      <c r="I143" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J143" s="30" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B144" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C144" s="31" t="inlineStr">
+        <is>
+          <t>Cosa facciamo prima di venire da te: la preparazione del furgone</t>
+        </is>
+      </c>
+      <c r="D144" s="31" t="inlineStr">
+        <is>
+          <t>Non immagina il lavoro di preparazione dietro ogni uscita — pensa che i tecnici partano senza organizzazione</t>
+        </is>
+      </c>
+      <c r="E144" s="31" t="inlineStr">
+        <is>
+          <t>Il team che carica il furgone, controlla gli strumenti e prepara il materiale prima di partire. Dietro le quinte della professionalità.</t>
+        </is>
+      </c>
+      <c r="F144" s="30" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="G144" s="30" t="inlineStr">
+        <is>
+          <t>Dietro le quinte squadra</t>
+        </is>
+      </c>
+      <c r="H144" s="31" t="inlineStr"/>
+      <c r="I144" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J144" s="30" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B145" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C145" s="31" t="inlineStr">
+        <is>
+          <t>Chi siamo: la squadra che entra davvero a casa tua</t>
+        </is>
+      </c>
+      <c r="D145" s="31" t="inlineStr">
+        <is>
+          <t>Hanno paura di non sapere chi gli arriva in casa e rimandano il sopralluogo.</t>
+        </is>
+      </c>
+      <c r="E145" s="31" t="inlineStr">
+        <is>
+          <t>Presentiamo i tecnici che fanno installazione e manutenzione: volti, ruoli, da quanti anni lavorano insieme. Niente discorsi aziendali.</t>
+        </is>
+      </c>
+      <c r="F145" s="30" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G145" s="30" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H145" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I145" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J145" s="30" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-15: nuove idee notturne
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -7376,6 +7376,236 @@
       </c>
       <c r="J145" s="30" t="n"/>
     </row>
+    <row r="146">
+      <c r="A146" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B146" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C146" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore ibrida: tiene anche la caldaia? E perché non è un difetto</t>
+        </is>
+      </c>
+      <c r="D146" s="31" t="inlineStr">
+        <is>
+          <t>Non capisco se la pompa di calore ibrida è peggio di una normale</t>
+        </is>
+      </c>
+      <c r="E146" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo cos'è la pompa di calore ibrida (PdC + caldaia nello stesso impianto), quando si usa l'una e quando l'altra, e perché in certe case è la scelta più intelligente — senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F146" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G146" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H146" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I146" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J146" s="30" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B147" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C147" s="31" t="inlineStr">
+        <is>
+          <t>Termostufa a legna: il calore arriva davvero in tutta la casa o rimane nel salotto?</t>
+        </is>
+      </c>
+      <c r="D147" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura che la termostufa scaldi solo dove c'è il fuoco</t>
+        </is>
+      </c>
+      <c r="E147" s="31" t="inlineStr">
+        <is>
+          <t>Mostriamo la differenza tra una stufa normale e una termostufa: i radiatori distribuiscono il calore prodotto dal fuoco in tutti gli ambienti, anche ai piani superiori. Visivo e concreto.</t>
+        </is>
+      </c>
+      <c r="F147" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Termostufe</t>
+        </is>
+      </c>
+      <c r="G147" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H147" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I147" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J147" s="30" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B148" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C148" s="31" t="inlineStr">
+        <is>
+          <t>Incentivi 2026: li gestite voi o devo occuparmi io della burocrazia?</t>
+        </is>
+      </c>
+      <c r="D148" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura di dover fare da solo le domande per i bonus e sbagliare</t>
+        </is>
+      </c>
+      <c r="E148" s="31" t="inlineStr">
+        <is>
+          <t>Risposta diretta e rassicurante: spieghiamo chi fa cosa, dal sopralluogo alla pratica incentivo. Obiettivo: togliere il timore burocratico che blocca la decisione di chiamarci.</t>
+        </is>
+      </c>
+      <c r="F148" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G148" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H148" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I148" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J148" s="30" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B149" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C149" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a legna: ogni quanti anni va pulita la canna fumaria?</t>
+        </is>
+      </c>
+      <c r="D149" s="31" t="inlineStr">
+        <is>
+          <t>Non so se la mia canna fumaria è a rischio e chi dovrei chiamare</t>
+        </is>
+      </c>
+      <c r="E149" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo la regola base sulla pulizia della canna fumaria (almeno una volta l'anno per uso regolare), cosa succede se non si fa, e chi interviene. Utile, pratico, senza allarmismi.</t>
+        </is>
+      </c>
+      <c r="F149" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G149" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H149" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I149" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J149" s="30" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="33" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B150" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C150" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a pellet o pompa di calore: nel 2026 quale ha più senso scegliere?</t>
+        </is>
+      </c>
+      <c r="D150" s="31" t="inlineStr">
+        <is>
+          <t>Non so tra caldaia a pellet e pompa di calore qual è la scelta giusta per me</t>
+        </is>
+      </c>
+      <c r="E150" s="31" t="inlineStr">
+        <is>
+          <t>Confronto diretto, non tecnico: quando la caldaia a pellet è la scelta giusta (casa grande, zona con legna disponibile, impianto a termosifoni esistente) e quando conviene la pompa di calore.</t>
+        </is>
+      </c>
+      <c r="F150" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G150" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H150" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I150" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J150" s="30" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7388,7 +7618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-16: nuove idee notturne
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -7606,6 +7606,1080 @@
       </c>
       <c r="J150" s="30" t="n"/>
     </row>
+    <row r="151">
+      <c r="A151" s="33" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B151" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C151" s="31" t="inlineStr">
+        <is>
+          <t>Ecobonus 2026 per la pompa di calore: chi può richiederlo e cosa serve davvero</t>
+        </is>
+      </c>
+      <c r="D151" s="31" t="inlineStr">
+        <is>
+          <t>Non so se ho diritto all'incentivo e ho paura di perdere soldi per ignoranza burocratica</t>
+        </is>
+      </c>
+      <c r="E151" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo in modo semplice chi può accedere all'Ecobonus per la pompa di calore nel 2026, quali documenti servono e chi gestisce la pratica al posto tuo</t>
+        </is>
+      </c>
+      <c r="F151" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G151" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H151" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I151" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J151" s="30" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="33" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B152" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C152" s="31" t="inlineStr">
+        <is>
+          <t>Termocamino a legna: riscalda solo il salotto o arriva calore anche nelle altre stanze?</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura di installare un termocamino e scoprire che il calore resta tutto in un'unica stanza</t>
+        </is>
+      </c>
+      <c r="E152" s="31" t="inlineStr">
+        <is>
+          <t>Mostriamo come un termocamino si collega all'impianto idraulico esistente e distribuisce calore nei radiatori di tutta la casa, non solo nel locale dove brucia il fuoco</t>
+        </is>
+      </c>
+      <c r="F152" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Termocamini</t>
+        </is>
+      </c>
+      <c r="G152" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H152" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I152" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J152" s="30" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="33" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B153" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C153" s="31" t="inlineStr">
+        <is>
+          <t>Detrazione fiscale o Conto Termico: qual è la differenza e quale spetta a te?</t>
+        </is>
+      </c>
+      <c r="D153" s="31" t="inlineStr">
+        <is>
+          <t>Sento parlare di mille incentivi ma non capisco la differenza e rischio di scegliere quello sbagliato</t>
+        </is>
+      </c>
+      <c r="E153" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo in linguaggio semplice quando si applica la detrazione IRPEF in dichiarazione dei redditi e quando invece si può richiedere il Conto Termico, con gli esempi pratici più comuni</t>
+        </is>
+      </c>
+      <c r="F153" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G153" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H153" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I153" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J153" s="30" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="33" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B154" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C154" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a pellet: l'errore più comune nella scelta della potenza (e come evitarlo)</t>
+        </is>
+      </c>
+      <c r="D154" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura di acquistare una caldaia sbagliata per la mia casa e dover spendere di nuovo dopo poco</t>
+        </is>
+      </c>
+      <c r="E154" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo perché la potenza della caldaia a pellet deve essere calcolata sulla dispersione della casa e non sul prezzo o sulla marca, e cosa succede concretamente se si sbaglia la taglia</t>
+        </is>
+      </c>
+      <c r="F154" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G154" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H154" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I154" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J154" s="30" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="33" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo: quando ha davvero senso installarla insieme al fotovoltaico?</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Non capisco se la batteria è un investimento utile o solo un costo extra che mi propinano</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo in modo pratico come funziona una batteria di accumulo abbinata al fotovoltaico, in quali situazioni domestiche fa la differenza concreta e quando invece non è prioritaria</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-17: 5 nuove idee notturne
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J160"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -7836,850 +7836,236 @@
       </c>
       <c r="J155" s="30" t="n"/>
     </row>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
+    <row r="156">
+      <c r="A156" s="33" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B156" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C156" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: funziona anche quando fa molto freddo fuori?</t>
+        </is>
+      </c>
+      <c r="D156" s="31" t="inlineStr">
+        <is>
+          <t>Il cliente teme che la pompa di calore si blocchi nelle giornate più rigide dell'inverno</t>
+        </is>
+      </c>
+      <c r="E156" s="31" t="inlineStr">
+        <is>
+          <t>Sfatiamo il mito che le pompe di calore si fermino col gelo: spiega come funzionano anche sotto zero, quando serve davvero un'integrazione e perché il 'limite al freddo' è spesso sopravvalutato.</t>
+        </is>
+      </c>
+      <c r="F156" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G156" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H156" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I156" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J156" s="30" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="33" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B157" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C157" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a pellet: dove si installa e quanto spazio serve davvero?</t>
+        </is>
+      </c>
+      <c r="D157" s="31" t="inlineStr">
+        <is>
+          <t>Il cliente non sa se ha lo spazio giusto o dove posizionare la caldaia in casa</t>
+        </is>
+      </c>
+      <c r="E157" s="31" t="inlineStr">
+        <is>
+          <t>Mostra i luoghi tipici di installazione (garage, lavanderia, locale tecnico) e spiega in modo semplice le distanze minime normative, rassicurando chi pensa di non avere abbastanza spazio.</t>
+        </is>
+      </c>
+      <c r="F157" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G157" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H157" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I157" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J157" s="30" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="33" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B158" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C158" s="31" t="inlineStr">
+        <is>
+          <t>Bonus casa 2026: posso richiederlo anche se ho già fatto lavori negli anni scorsi?</t>
+        </is>
+      </c>
+      <c r="D158" s="31" t="inlineStr">
+        <is>
+          <t>Il cliente non sa se può ancora accedere agli incentivi dopo interventi precedenti</t>
+        </is>
+      </c>
+      <c r="E158" s="31" t="inlineStr">
+        <is>
+          <t>Risponde alla domanda frequente su cumulo e accesso agli incentivi per chi ha già detratto in anni passati, con esempi pratici chiari per un proprietario di casa non tecnico.</t>
+        </is>
+      </c>
+      <c r="F158" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G158" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H158" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I158" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J158" s="30" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="33" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B159" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C159" s="31" t="inlineStr">
+        <is>
+          <t>Cucina economica a legna: riscalda solo la cucina o può servire tutta la casa?</t>
+        </is>
+      </c>
+      <c r="D159" s="31" t="inlineStr">
+        <is>
+          <t>Il cliente non conosce la differenza tra cucina economica semplice e termocucina collegata all'impianto</t>
+        </is>
+      </c>
+      <c r="E159" s="31" t="inlineStr">
+        <is>
+          <t>Spiega la distinzione tra cucina economica standalone e termocucina con scambiatore idraulico, mostrando quando la seconda ha senso per distribuire il calore in più ambienti.</t>
+        </is>
+      </c>
+      <c r="F159" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Cucine economiche</t>
+        </is>
+      </c>
+      <c r="G159" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H159" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I159" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J159" s="30" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="33" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B160" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C160" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore e pompa di calore: non sono la stessa cosa — ecco perché</t>
+        </is>
+      </c>
+      <c r="D160" s="31" t="inlineStr">
+        <is>
+          <t>Il cliente confonde i due prodotti e non capisce quale scegliere per riscaldare casa in modo principale</t>
+        </is>
+      </c>
+      <c r="E160" s="31" t="inlineStr">
+        <is>
+          <t>Chiarisce la differenza spesso fraintesa tra un climatizzatore tradizionale e una pompa di calore ad alta efficienza per riscaldamento principale, guidando il cliente verso la scelta giusta per le sue esigenze.</t>
+        </is>
+      </c>
+      <c r="F160" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G160" s="30" t="inlineStr">
+        <is>
+          <t>Confronto tra prodotti</t>
+        </is>
+      </c>
+      <c r="H160" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I160" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J160" s="30" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-18: nuove idee notturne
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J160"/>
+  <dimension ref="A1:J999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="20" min="1" max="1"/>
@@ -8066,6 +8066,1070 @@
       </c>
       <c r="J160" s="30" t="n"/>
     </row>
+    <row r="161">
+      <c r="A161" s="33" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B161" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C161" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: il errore più comune è installarla senza isolare bene la casa</t>
+        </is>
+      </c>
+      <c r="D161" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito dire che la pompa di calore non scalda abbastanza d'inverno — eppure tutti la consigliano</t>
+        </is>
+      </c>
+      <c r="E161" s="31" t="inlineStr">
+        <is>
+          <t>Molti utenti si lamentano del riscaldamento scarso, ma il problema spesso non è la pompa di calore in sé: è la dispersione termica dell'edificio. Il reel spiega perché l'isolamento fa la differenza e cosa chiedere prima dell'installazione.</t>
+        </is>
+      </c>
+      <c r="F161" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G161" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H161" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I161" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J161" s="30" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="33" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B162" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C162" s="31" t="inlineStr">
+        <is>
+          <t>Termostufa a pellet: si può mettere in qualsiasi stanza o ci sono limiti?</t>
+        </is>
+      </c>
+      <c r="D162" s="31" t="inlineStr">
+        <is>
+          <t>Vorrei una termostufa a pellet ma non so se posso metterla dove voglio o se ci sono vincoli di legge</t>
+        </is>
+      </c>
+      <c r="E162" s="31" t="inlineStr">
+        <is>
+          <t>Non tutte le stanze sono adatte: servono scarico fumi, areazione e distanze minime dai materiali combustibili. Il reel guida il proprietario di casa nei criteri di scelta della posizione, in modo semplice e visivo.</t>
+        </is>
+      </c>
+      <c r="F162" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Termostufe</t>
+        </is>
+      </c>
+      <c r="G162" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H162" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I162" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J162" s="30" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="33" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B163" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C163" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 2026: come funziona il rimborso e in quanto tempo arriva?</t>
+        </is>
+      </c>
+      <c r="D163" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito parlare del Conto Termico ma non capisco quando e come mi arrivano i soldi</t>
+        </is>
+      </c>
+      <c r="E163" s="31" t="inlineStr">
+        <is>
+          <t>Il Conto Termico è uno degli incentivi meno conosciuti ma più vantaggiosi per stufe, caldaie e pompe di calore. Il reel spiega in 3 passi: cos'è, chi può richiederlo, in quanto tempo arriva il rimborso — senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F163" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G163" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H163" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I163" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J163" s="30" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="33" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B164" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C164" s="31" t="inlineStr">
+        <is>
+          <t>Fotovoltaico con o senza batteria: come scegliere in base alle tue abitudini di casa</t>
+        </is>
+      </c>
+      <c r="D164" s="31" t="inlineStr">
+        <is>
+          <t>Non so se vale la pena aggiungere la batteria al fotovoltaico o se è solo una spesa in più</t>
+        </is>
+      </c>
+      <c r="E164" s="31" t="inlineStr">
+        <is>
+          <t>La scelta dipende da quando si consuma energia in casa: chi è fuori tutto il giorno trae più vantaggio dalla batteria. Il reel usa esempi pratici di famiglie tipo per aiutare lo spettatore a riconoscersi e capire cosa fa per lui.</t>
+        </is>
+      </c>
+      <c r="F164" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G164" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H164" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I164" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J164" s="30" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="33" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B165" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C165" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a legna al posto del caminetto aperto: cosa cambia davvero in termini di calore e sicurezza</t>
+        </is>
+      </c>
+      <c r="D165" s="31" t="inlineStr">
+        <is>
+          <t>Ho un caminetto aperto che scalda poco e fa fumo — ho sentito che l'inserto è meglio ma non so cosa aspettarmi</t>
+        </is>
+      </c>
+      <c r="E165" s="31" t="inlineStr">
+        <is>
+          <t>Il caminetto aperto disperde fino all'80% del calore. L'inserto a legna trasforma lo stesso vano in una fonte di calore efficiente, con vetro panoramico e meno rischi. Il reel mostra il confronto prima/dopo in modo visivo e immediato.</t>
+        </is>
+      </c>
+      <c r="F165" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G165" s="30" t="inlineStr">
+        <is>
+          <t>A cosa viene sostituito</t>
+        </is>
+      </c>
+      <c r="H165" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I165" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J165" s="30" t="n"/>
+    </row>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Shortlist Luglio 2026: 6 idee spostate su Drive + Shortlist Mensile, 4 idee Scartata spostate in Cimitero Idee
Eseguito manualmente in sostituzione del trigger 1° del mese (bug fix in corso).
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -23,8 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -133,7 +134,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -239,11 +240,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -311,6 +326,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -756,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -5670,27 +5694,27 @@
       </c>
       <c r="C101" s="28" t="inlineStr">
         <is>
-          <t>Pannelli fotovoltaici con neve sopra: si fermano o producono comunque?</t>
+          <t>Conto Termico: il rimborso arriva in conto corrente o è una detrazione in dichiarazione?</t>
         </is>
       </c>
       <c r="D101" s="28" t="inlineStr">
         <is>
-          <t>Paura di perdere produzione in inverno</t>
+          <t>Non capiscono come viene pagato</t>
         </is>
       </c>
       <c r="E101" s="28" t="inlineStr">
         <is>
-          <t>Con 5 cm di neve smettono. Ma la neve scivola da sola in poche ore se i pannelli sono inclinati almeno 15°. E d'inverno con cielo sereno e freddo producono bene (i pannelli rendono meglio al freddo).</t>
+          <t>Differenza fondamentale: il Conto Termico è un rimborso diretto in conto corrente (non detrazione in 730). In 1-2 rate entro 2 anni. Spieghiamo il meccanismo senza burocrazia.</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Fotovoltaici</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Domanda economica</t>
         </is>
       </c>
       <c r="H101" s="28" t="inlineStr">
@@ -5700,7 +5724,7 @@
       </c>
       <c r="I101" s="14" t="inlineStr">
         <is>
-          <t>Scartata</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J101" s="15" t="inlineStr">
@@ -5720,27 +5744,27 @@
       </c>
       <c r="C102" s="28" t="inlineStr">
         <is>
-          <t>Conto Termico: il rimborso arriva in conto corrente o è una detrazione in dichiarazione?</t>
+          <t>Stufa a legna in una casa moderna ben isolata: ha ancora senso?</t>
         </is>
       </c>
       <c r="D102" s="28" t="inlineStr">
         <is>
-          <t>Non capiscono come viene pagato</t>
+          <t>Dubbio se la stufa sia obsoleta nelle case nuove</t>
         </is>
       </c>
       <c r="E102" s="28" t="inlineStr">
         <is>
-          <t>Differenza fondamentale: il Conto Termico è un rimborso diretto in conto corrente (non detrazione in 730). In 1-2 rate entro 2 anni. Spieghiamo il meccanismo senza burocrazia.</t>
+          <t>In una casa ben isolata (A o B) una stufa a legna può essere l'unico riscaldamento necessario nelle mezze stagioni. Ma va dimensionata correttamente. Spieghiamo i parametri giusti.</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Stufe</t>
         </is>
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>Domanda economica</t>
+          <t>Confronto con alternative</t>
         </is>
       </c>
       <c r="H102" s="28" t="inlineStr">
@@ -5770,27 +5794,27 @@
       </c>
       <c r="C103" s="28" t="inlineStr">
         <is>
-          <t>Termocamino ad aria o ad acqua: quale scegliere?</t>
+          <t>Detrazione IRPEF 50%: vale anche se ho pagato poche tasse quell'anno?</t>
         </is>
       </c>
       <c r="D103" s="28" t="inlineStr">
         <is>
-          <t>Non sanno la differenza tra le due versioni</t>
+          <t>Paura di perdere il bonus per reddito basso</t>
         </is>
       </c>
       <c r="E103" s="28" t="inlineStr">
         <is>
-          <t>Ad aria: scalda solo la stanza e le adiacenti. Ad acqua: si collega ai termosifoni e scalda tutta la casa. Mostriamo quando ha senso uno e quando l'altro con esempi pratici.</t>
+          <t>La detrazione si spalma su 10 anni. Se in un anno hai meno capienza, quella quota va persa. Spieghiamo le alternative (cessione del credito dove ancora possibile, Conto Termico).</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Termocamini</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>Come scegliere il modello giusto</t>
+          <t>Domanda burocratica / normativa</t>
         </is>
       </c>
       <c r="H103" s="28" t="inlineStr">
@@ -5800,7 +5824,7 @@
       </c>
       <c r="I103" s="14" t="inlineStr">
         <is>
-          <t>Scartata</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J103" s="15" t="inlineStr">
@@ -5820,27 +5844,27 @@
       </c>
       <c r="C104" s="28" t="inlineStr">
         <is>
-          <t>Stufa a legna in una casa moderna ben isolata: ha ancora senso?</t>
+          <t>Inserto a legna: quanto legna serve per una stagione invernale?</t>
         </is>
       </c>
       <c r="D104" s="28" t="inlineStr">
         <is>
-          <t>Dubbio se la stufa sia obsoleta nelle case nuove</t>
+          <t>Non sanno quanto spazio serve per lo stoccaggio</t>
         </is>
       </c>
       <c r="E104" s="28" t="inlineStr">
         <is>
-          <t>In una casa ben isolata (A o B) una stufa a legna può essere l'unico riscaldamento necessario nelle mezze stagioni. Ma va dimensionata correttamente. Spieghiamo i parametri giusti.</t>
+          <t>Casa di 100 mq ben isolata in pianura padana: circa 2-3 metri steri. Mostriamo come stoccarla correttamente (coperta ma aerata) e perché la legna verde non va bene.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Stufe</t>
+          <t>Prodotto - Inserti e Camini</t>
         </is>
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
+          <t>Manutenzione</t>
         </is>
       </c>
       <c r="H104" s="28" t="inlineStr">
@@ -5870,27 +5894,27 @@
       </c>
       <c r="C105" s="28" t="inlineStr">
         <is>
-          <t>Solare termico sul balcone: si può fare senza tetto di proprietà?</t>
+          <t>Pompa di calore: perché la bolletta elettrica sale il primo mese e poi scende?</t>
         </is>
       </c>
       <c r="D105" s="28" t="inlineStr">
         <is>
-          <t>Vivono in appartamento e credono di non poter installare nulla</t>
+          <t>Si spaventano dopo la prima bolletta</t>
         </is>
       </c>
       <c r="E105" s="28" t="inlineStr">
         <is>
-          <t>Esistono pannelli solari termici balcone (verticali). Non sostituiscono un impianto sul tetto ma riducono del 40-50% il consumo per l'acqua calda sanitaria. Mostriamo l'opzione concreta.</t>
+          <t>Il primo mese l'impianto lavora di più perché deve portare a temperatura una casa che era gestita diversamente. Dal secondo mese si stabilizza. Spieghiamo il fenomeno e i numeri medi.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Solari</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>Dove si può installare</t>
+          <t>Errore comune</t>
         </is>
       </c>
       <c r="H105" s="28" t="inlineStr">
@@ -5900,7 +5924,7 @@
       </c>
       <c r="I105" s="14" t="inlineStr">
         <is>
-          <t>Scartata</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J105" s="15" t="inlineStr">
@@ -5920,27 +5944,27 @@
       </c>
       <c r="C106" s="28" t="inlineStr">
         <is>
-          <t>Detrazione IRPEF 50%: vale anche se ho pagato poche tasse quell'anno?</t>
+          <t>Fotovoltaico su tetto a falde multiple: si installa e quanto rende?</t>
         </is>
       </c>
       <c r="D106" s="28" t="inlineStr">
         <is>
-          <t>Paura di perdere il bonus per reddito basso</t>
+          <t>Credono che il tetto a falde multiple non sia compatibile</t>
         </is>
       </c>
       <c r="E106" s="28" t="inlineStr">
         <is>
-          <t>La detrazione si spalma su 10 anni. Se in un anno hai meno capienza, quella quota va persa. Spieghiamo le alternative (cessione del credito dove ancora possibile, Conto Termico).</t>
+          <t>Si installa su qualsiasi falda purché non in ombra. Le falde a sud-ovest e sud-est rendono solo il 10-15% meno di quella perfettamente a sud. Mostriamo un caso reale.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
         </is>
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica / normativa</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H106" s="28" t="inlineStr">
@@ -5970,27 +5994,27 @@
       </c>
       <c r="C107" s="28" t="inlineStr">
         <is>
-          <t>Inserto a legna: quanto legna serve per una stagione invernale?</t>
+          <t>Caldaia a pellet: si installa anche in appartamento al piano 4°?</t>
         </is>
       </c>
       <c r="D107" s="28" t="inlineStr">
         <is>
-          <t>Non sanno quanto spazio serve per lo stoccaggio</t>
+          <t>Credono che la caldaia a pellet richieda necessariamente un locale grande</t>
         </is>
       </c>
       <c r="E107" s="28" t="inlineStr">
         <is>
-          <t>Casa di 100 mq ben isolata in pianura padana: circa 2-3 metri steri. Mostriamo come stoccarla correttamente (coperta ma aerata) e perché la legna verde non va bene.</t>
+          <t>La caldaia a pellet ha bisogno di: locale tecnico (anche piccolo), silo pellet, canna fumaria. In appartamento il nodo è la canna fumaria condominiale. Spieghiamo i casi possibili.</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Inserti e Camini</t>
+          <t>Prodotto - Caldaie</t>
         </is>
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Dove si può installare</t>
         </is>
       </c>
       <c r="H107" s="28" t="inlineStr">
@@ -6020,27 +6044,27 @@
       </c>
       <c r="C108" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: perché la bolletta elettrica sale il primo mese e poi scende?</t>
+          <t>Ecobonus o Conto Termico: quale conviene di più per la pompa di calore?</t>
         </is>
       </c>
       <c r="D108" s="28" t="inlineStr">
         <is>
-          <t>Si spaventano dopo la prima bolletta</t>
+          <t>Non sanno quale incentivo chiedere</t>
         </is>
       </c>
       <c r="E108" s="28" t="inlineStr">
         <is>
-          <t>Il primo mese l'impianto lavora di più perché deve portare a temperatura una casa che era gestita diversamente. Dal secondo mese si stabilizza. Spieghiamo il fenomeno e i numeri medi.</t>
+          <t>Dipende: Ecobonus 50% spalmato in 10 anni sul 730. Conto Termico rimborso diretto in 2 rate ma ha tetto di spesa. Mostriamo i due scenari con un confronto diretto e semplice.</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
+          <t>Confronto tra prodotti</t>
         </is>
       </c>
       <c r="H108" s="28" t="inlineStr">
@@ -6061,41 +6085,41 @@
     </row>
     <row r="109" ht="45.75" customHeight="1" s="17">
       <c r="A109" s="11" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>Recupero Automatico</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C109" s="28" t="inlineStr">
         <is>
-          <t>Fotovoltaico su tetto a falde multiple: si installa e quanto rende?</t>
+          <t>Pompa di calore: funziona davvero quando fuori ci sono -5°C?</t>
         </is>
       </c>
       <c r="D109" s="28" t="inlineStr">
         <is>
-          <t>Credono che il tetto a falde multiple non sia compatibile</t>
+          <t>Ho sentito che si blocca col gelo — vero o mito?</t>
         </is>
       </c>
       <c r="E109" s="28" t="inlineStr">
         <is>
-          <t>Si installa su qualsiasi falda purché non in ombra. Le falde a sud-ovest e sud-est rendono solo il 10-15% meno di quella perfettamente a sud. Mostriamo un caso reale.</t>
+          <t>Sfatiamo il mito più diffuso: molte pompe di calore moderne lavorano fino a -20°C. Il reel mostra cosa succede realmente all'unità esterna in una notte gelata e perché la casa rimane calda.</t>
         </is>
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Fotovoltaici</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Errore comune</t>
         </is>
       </c>
       <c r="H109" s="28" t="inlineStr">
         <is>
-          <t>Recupero idee lug 2026 — routine fixata</t>
+          <t>Generato automaticamente di notte</t>
         </is>
       </c>
       <c r="I109" s="14" t="inlineStr">
@@ -6111,46 +6135,46 @@
     </row>
     <row r="110" ht="60.75" customHeight="1" s="17">
       <c r="A110" s="11" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B110" s="9" t="inlineStr">
         <is>
-          <t>Recupero Automatico</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C110" s="28" t="inlineStr">
         <is>
-          <t>Colonnina di ricarica: dopo l'installazione come si collega all'app?</t>
+          <t>Conto Termico 2025: chi può richiederlo e per quali prodotti?</t>
         </is>
       </c>
       <c r="D110" s="28" t="inlineStr">
         <is>
-          <t>Non sanno che le wallbox moderne sono smart</t>
+          <t>Sento parlare di Conto Termico ma non so se spetta anche a me</t>
         </is>
       </c>
       <c r="E110" s="28" t="inlineStr">
         <is>
-          <t>Le wallbox moderne hanno app: puoi programmare la ricarica di notte (quando l'energia costa meno), vedere i consumi, bloccarla da remoto. Mostriamo come funziona in 60 secondi.</t>
+          <t>Spiegazione semplice: cos'è il Conto Termico, chi ha diritto (privati inclusi), quali impianti coprono e come si fa domanda senza un commercialista. Pensato per chi ha sentito il nome ma non ha mai capito come funziona.</t>
         </is>
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Colonnine di Ricarica</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G110" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H110" s="28" t="inlineStr">
         <is>
-          <t>Recupero idee lug 2026 — routine fixata</t>
+          <t>Generato automaticamente di notte</t>
         </is>
       </c>
       <c r="I110" s="14" t="inlineStr">
         <is>
-          <t>Scartata</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J110" s="15" t="inlineStr">
@@ -6161,31 +6185,31 @@
     </row>
     <row r="111" ht="45.75" customHeight="1" s="17">
       <c r="A111" s="11" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B111" s="9" t="inlineStr">
         <is>
-          <t>Recupero Automatico</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C111" s="28" t="inlineStr">
         <is>
-          <t>Caldaia a pellet: si installa anche in appartamento al piano 4°?</t>
+          <t>Inserto a legna in condominio: si può installare o è vietato?</t>
         </is>
       </c>
       <c r="D111" s="28" t="inlineStr">
         <is>
-          <t>Credono che la caldaia a pellet richieda necessariamente un locale grande</t>
+          <t>Vogrei il fuoco vero in casa ma abito in un palazzo — è impossibile?</t>
         </is>
       </c>
       <c r="E111" s="28" t="inlineStr">
         <is>
-          <t>La caldaia a pellet ha bisogno di: locale tecnico (anche piccolo), silo pellet, canna fumaria. In appartamento il nodo è la canna fumaria condominiale. Spieghiamo i casi possibili.</t>
+          <t>Moltissimi rinunciano senza nemmeno chiedere. Il reel spiega le condizioni che rendono possibile l'installazione di un inserto in un appartamento (canna fumaria dedicata, regolamento condominiale, norme vigenti) e quando invece non si può.</t>
         </is>
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Caldaie</t>
+          <t>Prodotto - Inserti e Camini</t>
         </is>
       </c>
       <c r="G111" s="9" t="inlineStr">
@@ -6195,7 +6219,7 @@
       </c>
       <c r="H111" s="28" t="inlineStr">
         <is>
-          <t>Recupero idee lug 2026 — routine fixata</t>
+          <t>Generato automaticamente di notte</t>
         </is>
       </c>
       <c r="I111" s="14" t="inlineStr">
@@ -6211,41 +6235,41 @@
     </row>
     <row r="112" ht="45.75" customHeight="1" s="17">
       <c r="A112" s="11" t="n">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="B112" s="9" t="inlineStr">
         <is>
-          <t>Recupero Automatico</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C112" s="28" t="inlineStr">
         <is>
-          <t>Ecobonus o Conto Termico: quale conviene di più per la pompa di calore?</t>
+          <t>Caldaia a gas vs pompa di calore: come scelgo quella giusta per la mia casa?</t>
         </is>
       </c>
       <c r="D112" s="28" t="inlineStr">
         <is>
-          <t>Non sanno quale incentivo chiedere</t>
+          <t>Mi dicono di passare alla pompa di calore ma ho sempre usato il gas — come decido?</t>
         </is>
       </c>
       <c r="E112" s="28" t="inlineStr">
         <is>
-          <t>Dipende: Ecobonus 50% spalmato in 10 anni sul 730. Conto Termico rimborso diretto in 2 rate ma ha tetto di spesa. Mostriamo i due scenari con un confronto diretto e semplice.</t>
+          <t>Non esiste la scelta universalmente migliore. Il reel guida in modo semplice: tipo di abitazione, clima della zona, impianto radiante o termosifoni — un mini-percorso decisionale per il proprietario di casa non tecnico.</t>
         </is>
       </c>
       <c r="F112" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G112" s="9" t="inlineStr">
         <is>
-          <t>Confronto tra prodotti</t>
+          <t>Confronto con alternative</t>
         </is>
       </c>
       <c r="H112" s="28" t="inlineStr">
         <is>
-          <t>Recupero idee lug 2026 — routine fixata</t>
+          <t>Generato automaticamente di notte</t>
         </is>
       </c>
       <c r="I112" s="14" t="inlineStr">
@@ -6261,7 +6285,7 @@
     </row>
     <row r="113" ht="60.75" customHeight="1" s="17">
       <c r="A113" s="11" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="B113" s="9" t="inlineStr">
         <is>
@@ -6270,17 +6294,17 @@
       </c>
       <c r="C113" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: funziona davvero quando fuori ci sono -5°C?</t>
+          <t>Pompa di calore: quanto spazio serve davvero per l'unità esterna?</t>
         </is>
       </c>
       <c r="D113" s="28" t="inlineStr">
         <is>
-          <t>Ho sentito che si blocca col gelo — vero o mito?</t>
+          <t>Voglio la pompa di calore ma ho paura che il motore esterno non ci stia</t>
         </is>
       </c>
       <c r="E113" s="28" t="inlineStr">
         <is>
-          <t>Sfatiamo il mito più diffuso: molte pompe di calore moderne lavorano fino a -20°C. Il reel mostra cosa succede realmente all'unità esterna in una notte gelata e perché la casa rimane calda.</t>
+          <t>Mostriamo con esempi reali quanto spazio occupa un'unità esterna (balcone stretto, nicchia, parete laterale). Sfatiamo la paura che servano grandi spazi.</t>
         </is>
       </c>
       <c r="F113" s="9" t="inlineStr">
@@ -6290,7 +6314,7 @@
       </c>
       <c r="G113" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
+          <t>Dove si può installare</t>
         </is>
       </c>
       <c r="H113" s="28" t="inlineStr">
@@ -6311,7 +6335,7 @@
     </row>
     <row r="114" ht="45.75" customHeight="1" s="17">
       <c r="A114" s="11" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="B114" s="9" t="inlineStr">
         <is>
@@ -6320,27 +6344,27 @@
       </c>
       <c r="C114" s="28" t="inlineStr">
         <is>
-          <t>Stufa a pellet: 3 segnali che ti dice che è ora di cambiarla</t>
+          <t>Conto Termico 2026: dal sopralluogo ai soldi sul conto, quanto tempo passa?</t>
         </is>
       </c>
       <c r="D114" s="28" t="inlineStr">
         <is>
-          <t>La mia stufa ha 8 anni e scalda ancora — la tengo o la cambio?</t>
+          <t>Ho sentito parlare del Conto Termico ma ho paura che i soldi non arrivino mai o che ci voglia un anno</t>
         </is>
       </c>
       <c r="E114" s="28" t="inlineStr">
         <is>
-          <t>Non aspettare il guasto totale. Il reel elenca i tre sintomi che indicano che la stufa sta per cedere e perché intervenire prima conviene in termini di efficienza e incentivi disponibili.</t>
+          <t>Illustriamo passo per passo la tempistica reale: sopralluogo → lavori → domanda GSE → pagamento. Rassicurazione concreta su tempi medi.</t>
         </is>
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Stufe</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G114" s="9" t="inlineStr">
         <is>
-          <t>Quando sostituirlo</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H114" s="28" t="inlineStr">
@@ -6350,16 +6374,18 @@
       </c>
       <c r="I114" s="14" t="inlineStr">
         <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J114" s="15" t="n">
-        <v>1</v>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J114" s="15" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
       </c>
     </row>
     <row r="115" ht="45.75" customHeight="1" s="17">
       <c r="A115" s="11" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="B115" s="9" t="inlineStr">
         <is>
@@ -6368,27 +6394,27 @@
       </c>
       <c r="C115" s="28" t="inlineStr">
         <is>
-          <t>Conto Termico 2025: chi può richiederlo e per quali prodotti?</t>
+          <t>Stufa a pellet rumorosa di notte: è normale o c'è qualcosa che non va?</t>
         </is>
       </c>
       <c r="D115" s="28" t="inlineStr">
         <is>
-          <t>Sento parlare di Conto Termico ma non so se spetta anche a me</t>
+          <t>La mia stufa a pellet fa rumori strani la sera e non so se chiamare il tecnico o se è tutto normale</t>
         </is>
       </c>
       <c r="E115" s="28" t="inlineStr">
         <is>
-          <t>Spiegazione semplice: cos'è il Conto Termico, chi ha diritto (privati inclusi), quali impianti coprono e come si fa domanda senza un commercialista. Pensato per chi ha sentito il nome ma non ha mai capito come funziona.</t>
+          <t>Distinguiamo i rumori normali (coclea, ventola di scarico) da quelli che richiedono assistenza (bruciatore, caricamento irregolare). Regola pratica: quando chiamare vs quando no.</t>
         </is>
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Stufe</t>
         </is>
       </c>
       <c r="G115" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica/normativa</t>
+          <t>Manutenzione</t>
         </is>
       </c>
       <c r="H115" s="28" t="inlineStr">
@@ -6409,46 +6435,46 @@
     </row>
     <row r="116" ht="45.75" customHeight="1" s="17">
       <c r="A116" s="11" t="n">
-        <v>46216</v>
+        <v>46165</v>
       </c>
       <c r="B116" s="9" t="inlineStr">
         <is>
-          <t>Scheduled Task</t>
+          <t>Topic mese</t>
         </is>
       </c>
       <c r="C116" s="28" t="inlineStr">
         <is>
-          <t>Inserto a legna in condominio: si può installare o è vietato?</t>
+          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
         </is>
       </c>
       <c r="D116" s="28" t="inlineStr">
         <is>
-          <t>Vogrei il fuoco vero in casa ma abito in un palazzo — è impossibile?</t>
+          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
         </is>
       </c>
       <c r="E116" s="28" t="inlineStr">
         <is>
-          <t>Moltissimi rinunciano senza nemmeno chiedere. Il reel spiega le condizioni che rendono possibile l'installazione di un inserto in un appartamento (canna fumaria dedicata, regolamento condominiale, norme vigenti) e quando invece non si può.</t>
+          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Inserti e Camini</t>
+          <t>Prodotto - Climatizzatore</t>
         </is>
       </c>
       <c r="G116" s="9" t="inlineStr">
         <is>
-          <t>Dove si può installare</t>
+          <t>Errore comune</t>
         </is>
       </c>
       <c r="H116" s="28" t="inlineStr">
         <is>
-          <t>Generato automaticamente di notte</t>
+          <t>Topic mese: climatizzazione estiva privati</t>
         </is>
       </c>
       <c r="I116" s="14" t="inlineStr">
         <is>
-          <t>Nuova</t>
+          <t>Produzione</t>
         </is>
       </c>
       <c r="J116" s="15" t="inlineStr">
@@ -6459,7 +6485,7 @@
     </row>
     <row r="117" ht="45.75" customHeight="1" s="17">
       <c r="A117" s="11" t="n">
-        <v>46216</v>
+        <v>46170</v>
       </c>
       <c r="B117" s="9" t="inlineStr">
         <is>
@@ -6468,27 +6494,27 @@
       </c>
       <c r="C117" s="28" t="inlineStr">
         <is>
-          <t>Caldaia a gas vs pompa di calore: come scelgo quella giusta per la mia casa?</t>
+          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
         </is>
       </c>
       <c r="D117" s="28" t="inlineStr">
         <is>
-          <t>Mi dicono di passare alla pompa di calore ma ho sempre usato il gas — come decido?</t>
+          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
         </is>
       </c>
       <c r="E117" s="28" t="inlineStr">
         <is>
-          <t>Non esiste la scelta universalmente migliore. Il reel guida in modo semplice: tipo di abitazione, clima della zona, impianto radiante o termosifoni — un mini-percorso decisionale per il proprietario di casa non tecnico.</t>
+          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>Prodotto - Climatizzatore</t>
         </is>
       </c>
       <c r="G117" s="9" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
+          <t>Manutenzione</t>
         </is>
       </c>
       <c r="H117" s="28" t="inlineStr">
@@ -6498,7 +6524,7 @@
       </c>
       <c r="I117" s="14" t="inlineStr">
         <is>
-          <t>Nuova</t>
+          <t>Produzione</t>
         </is>
       </c>
       <c r="J117" s="15" t="inlineStr">
@@ -6509,7 +6535,7 @@
     </row>
     <row r="118" ht="60.75" customHeight="1" s="17">
       <c r="A118" s="11" t="n">
-        <v>46217</v>
+        <v>46171</v>
       </c>
       <c r="B118" s="9" t="inlineStr">
         <is>
@@ -6518,27 +6544,27 @@
       </c>
       <c r="C118" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: quanto spazio serve davvero per l'unità esterna?</t>
+          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
         </is>
       </c>
       <c r="D118" s="28" t="inlineStr">
         <is>
-          <t>Voglio la pompa di calore ma ho paura che il motore esterno non ci stia</t>
+          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
         </is>
       </c>
       <c r="E118" s="28" t="inlineStr">
         <is>
-          <t>Mostriamo con esempi reali quanto spazio occupa un'unità esterna (balcone stretto, nicchia, parete laterale). Sfatiamo la paura che servano grandi spazi.</t>
+          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
         </is>
       </c>
       <c r="G118" s="9" t="inlineStr">
         <is>
-          <t>Dove si può installare</t>
+          <t>Manutenzione</t>
         </is>
       </c>
       <c r="H118" s="28" t="inlineStr">
@@ -6548,7 +6574,7 @@
       </c>
       <c r="I118" s="14" t="inlineStr">
         <is>
-          <t>Nuova</t>
+          <t>Produzione</t>
         </is>
       </c>
       <c r="J118" s="15" t="inlineStr">
@@ -6559,74 +6585,72 @@
     </row>
     <row r="119" ht="45.75" customHeight="1" s="17">
       <c r="A119" s="11" t="n">
-        <v>46217</v>
+        <v>46148</v>
       </c>
       <c r="B119" s="9" t="inlineStr">
         <is>
-          <t>Scheduled Task</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="C119" s="28" t="inlineStr">
         <is>
-          <t>Inserto a pellet: il mio camino è abbastanza grande?</t>
+          <t>Climatizzatore: come scelgo il modello giusto per casa mia?</t>
         </is>
       </c>
       <c r="D119" s="28" t="inlineStr">
         <is>
-          <t>Ho un vecchio camino e non so se posso mettere un inserto a pellet senza demolire tutto</t>
+          <t>Non sa da dove partire nella scelta — marca, BTU, classe energetica gli sembrano tutti uguali</t>
         </is>
       </c>
       <c r="E119" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo le misure di apertura minima e massima per un inserto a pellet. Mostriamo anche cosa controllare sulla canna fumaria prima di chiamarci.</t>
+          <t>I 3 parametri pratici che fanno la differenza nella scelta di un climatizzatore, spiegati senza tecnicismi.</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Inserti e Camini</t>
+          <t>Prodotto - Climatizzatore</t>
         </is>
       </c>
       <c r="G119" s="9" t="inlineStr">
         <is>
-          <t>Dove si può installare</t>
-        </is>
-      </c>
-      <c r="H119" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H119" s="28" t="n"/>
       <c r="I119" s="14" t="inlineStr">
         <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J119" s="15" t="n">
-        <v>1</v>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J119" s="15" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
       </c>
     </row>
     <row r="120" ht="60.75" customHeight="1" s="17">
       <c r="A120" s="11" t="n">
-        <v>46217</v>
+        <v>46148</v>
       </c>
       <c r="B120" s="9" t="inlineStr">
         <is>
-          <t>Scheduled Task</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="C120" s="28" t="inlineStr">
         <is>
-          <t>Conto Termico 2026: dal sopralluogo ai soldi sul conto, quanto tempo passa?</t>
+          <t>Conto Termico: copre anche la sostituzione del vecchio condizionatore?</t>
         </is>
       </c>
       <c r="D120" s="28" t="inlineStr">
         <is>
-          <t>Ho sentito parlare del Conto Termico ma ho paura che i soldi non arrivino mai o che ci voglia un anno</t>
+          <t>Pensa che il Conto Termico valga solo per caldaie e pompe di calore, non per i climatizzatori</t>
         </is>
       </c>
       <c r="E120" s="28" t="inlineStr">
         <is>
-          <t>Illustriamo passo per passo la tempistica reale: sopralluogo → lavori → domanda GSE → pagamento. Rassicurazione concreta su tempi medi.</t>
+          <t>Quando la rottamazione di un vecchio climatizzatore dà diritto al Conto Termico e come richiederlo.</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
@@ -6636,17 +6660,13 @@
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H120" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
+          <t>Domanda burocratica / normativa</t>
+        </is>
+      </c>
+      <c r="H120" s="28" t="n"/>
       <c r="I120" s="14" t="inlineStr">
         <is>
-          <t>Nuova</t>
+          <t>Produzione</t>
         </is>
       </c>
       <c r="J120" s="15" t="inlineStr">
@@ -6657,26 +6677,26 @@
     </row>
     <row r="121" ht="60.75" customHeight="1" s="17">
       <c r="A121" s="11" t="n">
-        <v>46217</v>
+        <v>46148</v>
       </c>
       <c r="B121" s="9" t="inlineStr">
         <is>
-          <t>Scheduled Task</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="C121" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: la lasci accesa la notte o la spegni? L'errore che fa salire la bolletta</t>
+          <t>Pompa di calore: non devi rifare tutto l'impianto. E il fotovoltaico può aiutarti.</t>
         </is>
       </c>
       <c r="D121" s="28" t="inlineStr">
         <is>
-          <t>Uso la pompa di calore da mesi ma non so se sto sbagliando qualcosa nella gestione quotidiana</t>
+          <t>Rinunciano alla PdC convinti serva un cantiere enorme — non sanno che si può partire in piccolo</t>
         </is>
       </c>
       <c r="E121" s="28" t="inlineStr">
         <is>
-          <t>Sveliamo il contro-intuitivo: spegnerla e riaccenderla ogni giorno consuma più di tenerla a temperatura bassa di notte. Concetto di 'inerzia termica' spiegato senza tecnicismi.</t>
+          <t>Perché in molti casi basta un impianto più contenuto, e come il fotovoltaico aiuta a sostenere il consumo elettrico della PdC.</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
@@ -6686,65 +6706,59 @@
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
-        </is>
-      </c>
-      <c r="H121" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H121" s="28" t="n"/>
       <c r="I121" s="14" t="inlineStr">
         <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J121" s="15" t="n">
-        <v>1</v>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J121" s="15" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
       </c>
     </row>
     <row r="122" ht="60.75" customHeight="1" s="17">
       <c r="A122" s="11" t="n">
-        <v>46217</v>
+        <v>46148</v>
       </c>
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>Scheduled Task</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="C122" s="28" t="inlineStr">
         <is>
-          <t>Stufa a pellet rumorosa di notte: è normale o c'è qualcosa che non va?</t>
+          <t>Con cosa arriviamo a casa tua: i mezzi della squadra Solare Italiano</t>
         </is>
       </c>
       <c r="D122" s="28" t="inlineStr">
         <is>
-          <t>La mia stufa a pellet fa rumori strani la sera e non so se chiamare il tecnico o se è tutto normale</t>
+          <t>Non sa quanta preparazione professionale c'è dietro ogni intervento</t>
         </is>
       </c>
       <c r="E122" s="28" t="inlineStr">
         <is>
-          <t>Distinguiamo i rumori normali (coclea, ventola di scarico) da quelli che richiedono assistenza (bruciatore, caricamento irregolare). Regola pratica: quando chiamare vs quando no.</t>
+          <t>Ripresa dei furgoni e della piattaforma aerea per mostrare l'attrezzatura sul campo. Nessuna improvvisazione.</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Stufe</t>
+          <t>Conosci Solare Italiano</t>
         </is>
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
-        </is>
-      </c>
-      <c r="H122" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H122" s="28" t="n"/>
       <c r="I122" s="14" t="inlineStr">
         <is>
-          <t>Nuova</t>
+          <t>Produzione</t>
         </is>
       </c>
       <c r="J122" s="15" t="inlineStr">
@@ -6755,43 +6769,39 @@
     </row>
     <row r="123" ht="45.75" customHeight="1" s="17">
       <c r="A123" s="11" t="n">
-        <v>46165</v>
+        <v>46148</v>
       </c>
       <c r="B123" s="9" t="inlineStr">
         <is>
-          <t>Topic mese</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="C123" s="28" t="inlineStr">
         <is>
-          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
+          <t>Cosa facciamo prima di venire da te: la preparazione del furgone</t>
         </is>
       </c>
       <c r="D123" s="28" t="inlineStr">
         <is>
-          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
+          <t>Non immagina il lavoro di preparazione dietro ogni uscita — pensa che i tecnici partano senza organizzazione</t>
         </is>
       </c>
       <c r="E123" s="28" t="inlineStr">
         <is>
-          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
+          <t>Il team che carica il furgone, controlla gli strumenti e prepara il materiale prima di partire. Dietro le quinte della professionalità.</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Lavori</t>
         </is>
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
-        </is>
-      </c>
-      <c r="H123" s="28" t="inlineStr">
-        <is>
-          <t>Topic mese: climatizzazione estiva privati</t>
-        </is>
-      </c>
+          <t>Dietro le quinte squadra</t>
+        </is>
+      </c>
+      <c r="H123" s="28" t="n"/>
       <c r="I123" s="14" t="inlineStr">
         <is>
           <t>Produzione</t>
@@ -6805,7 +6815,7 @@
     </row>
     <row r="124" ht="45.75" customHeight="1" s="17">
       <c r="A124" s="11" t="n">
-        <v>46170</v>
+        <v>46218</v>
       </c>
       <c r="B124" s="9" t="inlineStr">
         <is>
@@ -6814,27 +6824,27 @@
       </c>
       <c r="C124" s="28" t="inlineStr">
         <is>
-          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
+          <t>Pompa di calore ibrida: tiene anche la caldaia? E perché non è un difetto</t>
         </is>
       </c>
       <c r="D124" s="28" t="inlineStr">
         <is>
-          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
+          <t>Non capisco se la pompa di calore ibrida è peggio di una normale</t>
         </is>
       </c>
       <c r="E124" s="28" t="inlineStr">
         <is>
-          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
+          <t>Spieghiamo cos'è la pompa di calore ibrida (PdC + caldaia nello stesso impianto), quando si usa l'una e quando l'altra, e perché in certe case è la scelta più intelligente — senza tecnicismi.</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H124" s="28" t="inlineStr">
@@ -6844,7 +6854,7 @@
       </c>
       <c r="I124" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J124" s="15" t="inlineStr">
@@ -6855,7 +6865,7 @@
     </row>
     <row r="125" ht="45.75" customHeight="1" s="17">
       <c r="A125" s="11" t="n">
-        <v>46171</v>
+        <v>46218</v>
       </c>
       <c r="B125" s="9" t="inlineStr">
         <is>
@@ -6864,27 +6874,27 @@
       </c>
       <c r="C125" s="28" t="inlineStr">
         <is>
-          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
+          <t>Termostufa a legna: il calore arriva davvero in tutta la casa o rimane nel salotto?</t>
         </is>
       </c>
       <c r="D125" s="28" t="inlineStr">
         <is>
-          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
+          <t>Ho paura che la termostufa scaldi solo dove c'è il fuoco</t>
         </is>
       </c>
       <c r="E125" s="28" t="inlineStr">
         <is>
-          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
+          <t>Mostriamo la differenza tra una stufa normale e una termostufa: i radiatori distribuiscono il calore prodotto dal fuoco in tutti gli ambienti, anche ai piani superiori. Visivo e concreto.</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Fotovoltaici</t>
+          <t>Prodotto - Termostufe</t>
         </is>
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H125" s="28" t="inlineStr">
@@ -6894,7 +6904,7 @@
       </c>
       <c r="I125" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J125" s="15" t="inlineStr">
@@ -6905,42 +6915,46 @@
     </row>
     <row r="126" ht="45.75" customHeight="1" s="17">
       <c r="A126" s="11" t="n">
-        <v>46148</v>
+        <v>46218</v>
       </c>
       <c r="B126" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C126" s="28" t="inlineStr">
         <is>
-          <t>Climatizzatore: come scelgo il modello giusto per casa mia?</t>
+          <t>Incentivi 2026: li gestite voi o devo occuparmi io della burocrazia?</t>
         </is>
       </c>
       <c r="D126" s="28" t="inlineStr">
         <is>
-          <t>Non sa da dove partire nella scelta — marca, BTU, classe energetica gli sembrano tutti uguali</t>
+          <t>Ho paura di dover fare da solo le domande per i bonus e sbagliare</t>
         </is>
       </c>
       <c r="E126" s="28" t="inlineStr">
         <is>
-          <t>I 3 parametri pratici che fanno la differenza nella scelta di un climatizzatore, spiegati senza tecnicismi.</t>
+          <t>Risposta diretta e rassicurante: spieghiamo chi fa cosa, dal sopralluogo alla pratica incentivo. Obiettivo: togliere il timore burocratico che blocca la decisione di chiamarci.</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>Come scegliere il modello giusto</t>
-        </is>
-      </c>
-      <c r="H126" s="28" t="n"/>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H126" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I126" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J126" s="15" t="inlineStr">
@@ -6951,42 +6965,46 @@
     </row>
     <row r="127" ht="45.75" customHeight="1" s="17">
       <c r="A127" s="11" t="n">
-        <v>46148</v>
+        <v>46218</v>
       </c>
       <c r="B127" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C127" s="28" t="inlineStr">
         <is>
-          <t>Conto Termico: copre anche la sostituzione del vecchio condizionatore?</t>
+          <t>Inserto a legna: ogni quanti anni va pulita la canna fumaria?</t>
         </is>
       </c>
       <c r="D127" s="28" t="inlineStr">
         <is>
-          <t>Pensa che il Conto Termico valga solo per caldaie e pompe di calore, non per i climatizzatori</t>
+          <t>Non so se la mia canna fumaria è a rischio e chi dovrei chiamare</t>
         </is>
       </c>
       <c r="E127" s="28" t="inlineStr">
         <is>
-          <t>Quando la rottamazione di un vecchio climatizzatore dà diritto al Conto Termico e come richiederlo.</t>
+          <t>Spieghiamo la regola base sulla pulizia della canna fumaria (almeno una volta l'anno per uso regolare), cosa succede se non si fa, e chi interviene. Utile, pratico, senza allarmismi.</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Inserti e Camini</t>
         </is>
       </c>
       <c r="G127" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica / normativa</t>
-        </is>
-      </c>
-      <c r="H127" s="28" t="n"/>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H127" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I127" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J127" s="15" t="inlineStr">
@@ -6997,26 +7015,26 @@
     </row>
     <row r="128" ht="45.75" customHeight="1" s="17">
       <c r="A128" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B128" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C128" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: non devi rifare tutto l'impianto. E il fotovoltaico può aiutarti.</t>
+          <t>Ecobonus 2026 per la pompa di calore: chi può richiederlo e cosa serve davvero</t>
         </is>
       </c>
       <c r="D128" s="28" t="inlineStr">
         <is>
-          <t>Rinunciano alla PdC convinti serva un cantiere enorme — non sanno che si può partire in piccolo</t>
+          <t>Non so se ho diritto all'incentivo e ho paura di perdere soldi per ignoranza burocratica</t>
         </is>
       </c>
       <c r="E128" s="28" t="inlineStr">
         <is>
-          <t>Perché in molti casi basta un impianto più contenuto, e come il fotovoltaico aiuta a sostenere il consumo elettrico della PdC.</t>
+          <t>Spieghiamo in modo semplice chi può accedere all'Ecobonus per la pompa di calore nel 2026, quali documenti servono e chi gestisce la pratica al posto tuo</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
@@ -7026,13 +7044,17 @@
       </c>
       <c r="G128" s="9" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
-        </is>
-      </c>
-      <c r="H128" s="28" t="n"/>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H128" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I128" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J128" s="15" t="inlineStr">
@@ -7043,42 +7065,46 @@
     </row>
     <row r="129" ht="45.75" customHeight="1" s="17">
       <c r="A129" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B129" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C129" s="28" t="inlineStr">
         <is>
-          <t>Con cosa arriviamo a casa tua: i mezzi della squadra Solare Italiano</t>
+          <t>Termocamino a legna: riscalda solo il salotto o arriva calore anche nelle altre stanze?</t>
         </is>
       </c>
       <c r="D129" s="28" t="inlineStr">
         <is>
-          <t>Non sa quanta preparazione professionale c'è dietro ogni intervento</t>
+          <t>Ho paura di installare un termocamino e scoprire che il calore resta tutto in un'unica stanza</t>
         </is>
       </c>
       <c r="E129" s="28" t="inlineStr">
         <is>
-          <t>Ripresa dei furgoni e della piattaforma aerea per mostrare l'attrezzatura sul campo. Nessuna improvvisazione.</t>
+          <t>Mostriamo come un termocamino si collega all'impianto idraulico esistente e distribuisce calore nei radiatori di tutta la casa, non solo nel locale dove brucia il fuoco</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>Conosci Solare Italiano</t>
+          <t>Prodotto - Termocamini</t>
         </is>
       </c>
       <c r="G129" s="9" t="inlineStr">
         <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="H129" s="28" t="n"/>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H129" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I129" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J129" s="15" t="inlineStr">
@@ -7089,42 +7115,46 @@
     </row>
     <row r="130" ht="45.75" customHeight="1" s="17">
       <c r="A130" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B130" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C130" s="28" t="inlineStr">
         <is>
-          <t>Cosa facciamo prima di venire da te: la preparazione del furgone</t>
+          <t>Detrazione fiscale o Conto Termico: qual è la differenza e quale spetta a te?</t>
         </is>
       </c>
       <c r="D130" s="28" t="inlineStr">
         <is>
-          <t>Non immagina il lavoro di preparazione dietro ogni uscita — pensa che i tecnici partano senza organizzazione</t>
+          <t>Sento parlare di mille incentivi ma non capisco la differenza e rischio di scegliere quello sbagliato</t>
         </is>
       </c>
       <c r="E130" s="28" t="inlineStr">
         <is>
-          <t>Il team che carica il furgone, controlla gli strumenti e prepara il materiale prima di partire. Dietro le quinte della professionalità.</t>
+          <t>Spieghiamo in linguaggio semplice quando si applica la detrazione IRPEF in dichiarazione dei redditi e quando invece si può richiedere il Conto Termico, con gli esempi pratici più comuni</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>Lavori</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G130" s="9" t="inlineStr">
         <is>
-          <t>Dietro le quinte squadra</t>
-        </is>
-      </c>
-      <c r="H130" s="28" t="n"/>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H130" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I130" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J130" s="15" t="inlineStr">
@@ -7135,7 +7165,7 @@
     </row>
     <row r="131" ht="45.75" customHeight="1" s="17">
       <c r="A131" s="11" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="B131" s="9" t="inlineStr">
         <is>
@@ -7144,27 +7174,27 @@
       </c>
       <c r="C131" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore ibrida: tiene anche la caldaia? E perché non è un difetto</t>
+          <t>Caldaia a pellet: l'errore più comune nella scelta della potenza (e come evitarlo)</t>
         </is>
       </c>
       <c r="D131" s="28" t="inlineStr">
         <is>
-          <t>Non capisco se la pompa di calore ibrida è peggio di una normale</t>
+          <t>Ho paura di acquistare una caldaia sbagliata per la mia casa e dover spendere di nuovo dopo poco</t>
         </is>
       </c>
       <c r="E131" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo cos'è la pompa di calore ibrida (PdC + caldaia nello stesso impianto), quando si usa l'una e quando l'altra, e perché in certe case è la scelta più intelligente — senza tecnicismi.</t>
+          <t>Spieghiamo perché la potenza della caldaia a pellet deve essere calcolata sulla dispersione della casa e non sul prezzo o sulla marca, e cosa succede concretamente se si sbaglia la taglia</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>Prodotto - Caldaie</t>
         </is>
       </c>
       <c r="G131" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Errore comune</t>
         </is>
       </c>
       <c r="H131" s="28" t="inlineStr">
@@ -7185,7 +7215,7 @@
     </row>
     <row r="132" ht="45.75" customHeight="1" s="17">
       <c r="A132" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B132" s="9" t="inlineStr">
         <is>
@@ -7194,22 +7224,22 @@
       </c>
       <c r="C132" s="28" t="inlineStr">
         <is>
-          <t>Termostufa a legna: il calore arriva davvero in tutta la casa o rimane nel salotto?</t>
+          <t>Pompa di calore: funziona anche quando fa molto freddo fuori?</t>
         </is>
       </c>
       <c r="D132" s="28" t="inlineStr">
         <is>
-          <t>Ho paura che la termostufa scaldi solo dove c'è il fuoco</t>
+          <t>Il cliente teme che la pompa di calore si blocchi nelle giornate più rigide dell'inverno</t>
         </is>
       </c>
       <c r="E132" s="28" t="inlineStr">
         <is>
-          <t>Mostriamo la differenza tra una stufa normale e una termostufa: i radiatori distribuiscono il calore prodotto dal fuoco in tutti gli ambienti, anche ai piani superiori. Visivo e concreto.</t>
+          <t>Sfatiamo il mito che le pompe di calore si fermino col gelo: spiega come funzionano anche sotto zero, quando serve davvero un'integrazione e perché il 'limite al freddo' è spesso sopravvalutato.</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Termostufe</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G132" s="9" t="inlineStr">
@@ -7235,7 +7265,7 @@
     </row>
     <row r="133" ht="45.75" customHeight="1" s="17">
       <c r="A133" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B133" s="9" t="inlineStr">
         <is>
@@ -7244,27 +7274,27 @@
       </c>
       <c r="C133" s="28" t="inlineStr">
         <is>
-          <t>Incentivi 2026: li gestite voi o devo occuparmi io della burocrazia?</t>
+          <t>Caldaia a pellet: dove si installa e quanto spazio serve davvero?</t>
         </is>
       </c>
       <c r="D133" s="28" t="inlineStr">
         <is>
-          <t>Ho paura di dover fare da solo le domande per i bonus e sbagliare</t>
+          <t>Il cliente non sa se ha lo spazio giusto o dove posizionare la caldaia in casa</t>
         </is>
       </c>
       <c r="E133" s="28" t="inlineStr">
         <is>
-          <t>Risposta diretta e rassicurante: spieghiamo chi fa cosa, dal sopralluogo alla pratica incentivo. Obiettivo: togliere il timore burocratico che blocca la decisione di chiamarci.</t>
+          <t>Mostra i luoghi tipici di installazione (garage, lavanderia, locale tecnico) e spiega in modo semplice le distanze minime normative, rassicurando chi pensa di non avere abbastanza spazio.</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Caldaie</t>
         </is>
       </c>
       <c r="G133" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica/normativa</t>
+          <t>Dove si può installare</t>
         </is>
       </c>
       <c r="H133" s="28" t="inlineStr">
@@ -7285,7 +7315,7 @@
     </row>
     <row r="134" ht="30.75" customHeight="1" s="17">
       <c r="A134" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B134" s="9" t="inlineStr">
         <is>
@@ -7294,27 +7324,27 @@
       </c>
       <c r="C134" s="28" t="inlineStr">
         <is>
-          <t>Inserto a legna: ogni quanti anni va pulita la canna fumaria?</t>
+          <t>Bonus casa 2026: posso richiederlo anche se ho già fatto lavori negli anni scorsi?</t>
         </is>
       </c>
       <c r="D134" s="28" t="inlineStr">
         <is>
-          <t>Non so se la mia canna fumaria è a rischio e chi dovrei chiamare</t>
+          <t>Il cliente non sa se può ancora accedere agli incentivi dopo interventi precedenti</t>
         </is>
       </c>
       <c r="E134" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo la regola base sulla pulizia della canna fumaria (almeno una volta l'anno per uso regolare), cosa succede se non si fa, e chi interviene. Utile, pratico, senza allarmismi.</t>
+          <t>Risponde alla domanda frequente su cumulo e accesso agli incentivi per chi ha già detratto in anni passati, con esempi pratici chiari per un proprietario di casa non tecnico.</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Inserti e Camini</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G134" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H134" s="28" t="inlineStr">
@@ -7335,7 +7365,7 @@
     </row>
     <row r="135" ht="45.75" customHeight="1" s="17">
       <c r="A135" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B135" s="9" t="inlineStr">
         <is>
@@ -7344,27 +7374,27 @@
       </c>
       <c r="C135" s="28" t="inlineStr">
         <is>
-          <t>Caldaia a pellet o pompa di calore: nel 2026 quale ha più senso scegliere?</t>
+          <t>Cucina economica a legna: riscalda solo la cucina o può servire tutta la casa?</t>
         </is>
       </c>
       <c r="D135" s="28" t="inlineStr">
         <is>
-          <t>Non so tra caldaia a pellet e pompa di calore qual è la scelta giusta per me</t>
+          <t>Il cliente non conosce la differenza tra cucina economica semplice e termocucina collegata all'impianto</t>
         </is>
       </c>
       <c r="E135" s="28" t="inlineStr">
         <is>
-          <t>Confronto diretto, non tecnico: quando la caldaia a pellet è la scelta giusta (casa grande, zona con legna disponibile, impianto a termosifoni esistente) e quando conviene la pompa di calore.</t>
+          <t>Spiega la distinzione tra cucina economica standalone e termocucina con scambiatore idraulico, mostrando quando la seconda ha senso per distribuire il calore in più ambienti.</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Caldaie</t>
+          <t>Prodotto - Cucine economiche</t>
         </is>
       </c>
       <c r="G135" s="9" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H135" s="28" t="inlineStr">
@@ -7374,16 +7404,18 @@
       </c>
       <c r="I135" s="14" t="inlineStr">
         <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J135" s="15" t="n">
-        <v>1</v>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J135" s="15" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
       </c>
     </row>
     <row r="136" ht="45.75" customHeight="1" s="17">
       <c r="A136" s="11" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="B136" s="9" t="inlineStr">
         <is>
@@ -7392,27 +7424,27 @@
       </c>
       <c r="C136" s="28" t="inlineStr">
         <is>
-          <t>Ecobonus 2026 per la pompa di calore: chi può richiederlo e cosa serve davvero</t>
+          <t>Climatizzatore e pompa di calore: non sono la stessa cosa — ecco perché</t>
         </is>
       </c>
       <c r="D136" s="28" t="inlineStr">
         <is>
-          <t>Non so se ho diritto all'incentivo e ho paura di perdere soldi per ignoranza burocratica</t>
+          <t>Il cliente confonde i due prodotti e non capisce quale scegliere per riscaldare casa in modo principale</t>
         </is>
       </c>
       <c r="E136" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo in modo semplice chi può accedere all'Ecobonus per la pompa di calore nel 2026, quali documenti servono e chi gestisce la pratica al posto tuo</t>
+          <t>Chiarisce la differenza spesso fraintesa tra un climatizzatore tradizionale e una pompa di calore ad alta efficienza per riscaldamento principale, guidando il cliente verso la scelta giusta per le sue esigenze.</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G136" s="9" t="inlineStr">
         <is>
-          <t>Incentivi</t>
+          <t>Confronto tra prodotti</t>
         </is>
       </c>
       <c r="H136" s="28" t="inlineStr">
@@ -7433,7 +7465,7 @@
     </row>
     <row r="137" ht="45.75" customHeight="1" s="17">
       <c r="A137" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B137" s="9" t="inlineStr">
         <is>
@@ -7442,27 +7474,27 @@
       </c>
       <c r="C137" s="28" t="inlineStr">
         <is>
-          <t>Termocamino a legna: riscalda solo il salotto o arriva calore anche nelle altre stanze?</t>
+          <t>Pompa di calore: il errore più comune è installarla senza isolare bene la casa</t>
         </is>
       </c>
       <c r="D137" s="28" t="inlineStr">
         <is>
-          <t>Ho paura di installare un termocamino e scoprire che il calore resta tutto in un'unica stanza</t>
+          <t>Ho sentito dire che la pompa di calore non scalda abbastanza d'inverno — eppure tutti la consigliano</t>
         </is>
       </c>
       <c r="E137" s="28" t="inlineStr">
         <is>
-          <t>Mostriamo come un termocamino si collega all'impianto idraulico esistente e distribuisce calore nei radiatori di tutta la casa, non solo nel locale dove brucia il fuoco</t>
+          <t>Molti utenti si lamentano del riscaldamento scarso, ma il problema spesso non è la pompa di calore in sé: è la dispersione termica dell'edificio. Il reel spiega perché l'isolamento fa la differenza e cosa chiedere prima dell'installazione.</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Termocamini</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G137" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Errore comune</t>
         </is>
       </c>
       <c r="H137" s="28" t="inlineStr">
@@ -7483,7 +7515,7 @@
     </row>
     <row r="138" ht="45.75" customHeight="1" s="17">
       <c r="A138" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B138" s="9" t="inlineStr">
         <is>
@@ -7492,27 +7524,27 @@
       </c>
       <c r="C138" s="28" t="inlineStr">
         <is>
-          <t>Detrazione fiscale o Conto Termico: qual è la differenza e quale spetta a te?</t>
+          <t>Termostufa a pellet: si può mettere in qualsiasi stanza o ci sono limiti?</t>
         </is>
       </c>
       <c r="D138" s="28" t="inlineStr">
         <is>
-          <t>Sento parlare di mille incentivi ma non capisco la differenza e rischio di scegliere quello sbagliato</t>
+          <t>Vorrei una termostufa a pellet ma non so se posso metterla dove voglio o se ci sono vincoli di legge</t>
         </is>
       </c>
       <c r="E138" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo in linguaggio semplice quando si applica la detrazione IRPEF in dichiarazione dei redditi e quando invece si può richiedere il Conto Termico, con gli esempi pratici più comuni</t>
+          <t>Non tutte le stanze sono adatte: servono scarico fumi, areazione e distanze minime dai materiali combustibili. Il reel guida il proprietario di casa nei criteri di scelta della posizione, in modo semplice e visivo.</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Termostufe</t>
         </is>
       </c>
       <c r="G138" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica/normativa</t>
+          <t>Dove si può installare</t>
         </is>
       </c>
       <c r="H138" s="28" t="inlineStr">
@@ -7533,7 +7565,7 @@
     </row>
     <row r="139" ht="45.75" customHeight="1" s="17">
       <c r="A139" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B139" s="9" t="inlineStr">
         <is>
@@ -7542,27 +7574,27 @@
       </c>
       <c r="C139" s="28" t="inlineStr">
         <is>
-          <t>Caldaia a pellet: l'errore più comune nella scelta della potenza (e come evitarlo)</t>
+          <t>Conto Termico 2026: come funziona il rimborso e in quanto tempo arriva?</t>
         </is>
       </c>
       <c r="D139" s="28" t="inlineStr">
         <is>
-          <t>Ho paura di acquistare una caldaia sbagliata per la mia casa e dover spendere di nuovo dopo poco</t>
+          <t>Ho sentito parlare del Conto Termico ma non capisco quando e come mi arrivano i soldi</t>
         </is>
       </c>
       <c r="E139" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo perché la potenza della caldaia a pellet deve essere calcolata sulla dispersione della casa e non sul prezzo o sulla marca, e cosa succede concretamente se si sbaglia la taglia</t>
+          <t>Il Conto Termico è uno degli incentivi meno conosciuti ma più vantaggiosi per stufe, caldaie e pompe di calore. Il reel spiega in 3 passi: cos'è, chi può richiederlo, in quanto tempo arriva il rimborso — senza tecnicismi.</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Caldaie</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G139" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H139" s="28" t="inlineStr">
@@ -7583,7 +7615,7 @@
     </row>
     <row r="140" ht="45.75" customHeight="1" s="17">
       <c r="A140" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B140" s="9" t="inlineStr">
         <is>
@@ -7592,27 +7624,27 @@
       </c>
       <c r="C140" s="28" t="inlineStr">
         <is>
-          <t>Batteria di accumulo: quando ha davvero senso installarla insieme al fotovoltaico?</t>
+          <t>Inserto a legna al posto del caminetto aperto: cosa cambia davvero in termini di calore e sicurezza</t>
         </is>
       </c>
       <c r="D140" s="28" t="inlineStr">
         <is>
-          <t>Non capisco se la batteria è un investimento utile o solo un costo extra che mi propinano</t>
+          <t>Ho un caminetto aperto che scalda poco e fa fumo — ho sentito che l'inserto è meglio ma non so cosa aspettarmi</t>
         </is>
       </c>
       <c r="E140" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo in modo pratico come funziona una batteria di accumulo abbinata al fotovoltaico, in quali situazioni domestiche fa la differenza concreta e quando invece non è prioritaria</t>
+          <t>Il caminetto aperto disperde fino all'80% del calore. L'inserto a legna trasforma lo stesso vano in una fonte di calore efficiente, con vetro panoramico e meno rischi. Il reel mostra il confronto prima/dopo in modo visivo e immediato.</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Batterie di Accumulo</t>
+          <t>Prodotto - Inserti e Camini</t>
         </is>
       </c>
       <c r="G140" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>A cosa viene sostituito</t>
         </is>
       </c>
       <c r="H140" s="28" t="inlineStr">
@@ -7622,511 +7654,25 @@
       </c>
       <c r="I140" s="14" t="inlineStr">
         <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J140" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="141" ht="45.75" customHeight="1" s="17">
-      <c r="A141" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B141" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C141" s="28" t="inlineStr">
-        <is>
-          <t>Pompa di calore: funziona anche quando fa molto freddo fuori?</t>
-        </is>
-      </c>
-      <c r="D141" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente teme che la pompa di calore si blocchi nelle giornate più rigide dell'inverno</t>
-        </is>
-      </c>
-      <c r="E141" s="28" t="inlineStr">
-        <is>
-          <t>Sfatiamo il mito che le pompe di calore si fermino col gelo: spiega come funzionano anche sotto zero, quando serve davvero un'integrazione e perché il 'limite al freddo' è spesso sopravvalutato.</t>
-        </is>
-      </c>
-      <c r="F141" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Pompe di Calore</t>
-        </is>
-      </c>
-      <c r="G141" s="9" t="inlineStr">
-        <is>
-          <t>Come funziona</t>
-        </is>
-      </c>
-      <c r="H141" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I141" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J141" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="45.75" customHeight="1" s="17">
-      <c r="A142" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B142" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C142" s="28" t="inlineStr">
-        <is>
-          <t>Caldaia a pellet: dove si installa e quanto spazio serve davvero?</t>
-        </is>
-      </c>
-      <c r="D142" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente non sa se ha lo spazio giusto o dove posizionare la caldaia in casa</t>
-        </is>
-      </c>
-      <c r="E142" s="28" t="inlineStr">
-        <is>
-          <t>Mostra i luoghi tipici di installazione (garage, lavanderia, locale tecnico) e spiega in modo semplice le distanze minime normative, rassicurando chi pensa di non avere abbastanza spazio.</t>
-        </is>
-      </c>
-      <c r="F142" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Caldaie</t>
-        </is>
-      </c>
-      <c r="G142" s="9" t="inlineStr">
-        <is>
-          <t>Dove si può installare</t>
-        </is>
-      </c>
-      <c r="H142" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I142" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J142" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="30.75" customHeight="1" s="17">
-      <c r="A143" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B143" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C143" s="28" t="inlineStr">
-        <is>
-          <t>Bonus casa 2026: posso richiederlo anche se ho già fatto lavori negli anni scorsi?</t>
-        </is>
-      </c>
-      <c r="D143" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente non sa se può ancora accedere agli incentivi dopo interventi precedenti</t>
-        </is>
-      </c>
-      <c r="E143" s="28" t="inlineStr">
-        <is>
-          <t>Risponde alla domanda frequente su cumulo e accesso agli incentivi per chi ha già detratto in anni passati, con esempi pratici chiari per un proprietario di casa non tecnico.</t>
-        </is>
-      </c>
-      <c r="F143" s="9" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G143" s="9" t="inlineStr">
-        <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H143" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I143" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J143" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="45.75" customHeight="1" s="17">
-      <c r="A144" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B144" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C144" s="28" t="inlineStr">
-        <is>
-          <t>Cucina economica a legna: riscalda solo la cucina o può servire tutta la casa?</t>
-        </is>
-      </c>
-      <c r="D144" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente non conosce la differenza tra cucina economica semplice e termocucina collegata all'impianto</t>
-        </is>
-      </c>
-      <c r="E144" s="28" t="inlineStr">
-        <is>
-          <t>Spiega la distinzione tra cucina economica standalone e termocucina con scambiatore idraulico, mostrando quando la seconda ha senso per distribuire il calore in più ambienti.</t>
-        </is>
-      </c>
-      <c r="F144" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Cucine economiche</t>
-        </is>
-      </c>
-      <c r="G144" s="9" t="inlineStr">
-        <is>
-          <t>Come funziona</t>
-        </is>
-      </c>
-      <c r="H144" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I144" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J144" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="45.75" customHeight="1" s="17">
-      <c r="A145" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B145" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C145" s="28" t="inlineStr">
-        <is>
-          <t>Climatizzatore e pompa di calore: non sono la stessa cosa — ecco perché</t>
-        </is>
-      </c>
-      <c r="D145" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente confonde i due prodotti e non capisce quale scegliere per riscaldare casa in modo principale</t>
-        </is>
-      </c>
-      <c r="E145" s="28" t="inlineStr">
-        <is>
-          <t>Chiarisce la differenza spesso fraintesa tra un climatizzatore tradizionale e una pompa di calore ad alta efficienza per riscaldamento principale, guidando il cliente verso la scelta giusta per le sue esigenze.</t>
-        </is>
-      </c>
-      <c r="F145" s="9" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G145" s="9" t="inlineStr">
-        <is>
-          <t>Confronto tra prodotti</t>
-        </is>
-      </c>
-      <c r="H145" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I145" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J145" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="60.75" customHeight="1" s="17">
-      <c r="A146" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B146" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C146" s="28" t="inlineStr">
-        <is>
-          <t>Pompa di calore: il errore più comune è installarla senza isolare bene la casa</t>
-        </is>
-      </c>
-      <c r="D146" s="28" t="inlineStr">
-        <is>
-          <t>Ho sentito dire che la pompa di calore non scalda abbastanza d'inverno — eppure tutti la consigliano</t>
-        </is>
-      </c>
-      <c r="E146" s="28" t="inlineStr">
-        <is>
-          <t>Molti utenti si lamentano del riscaldamento scarso, ma il problema spesso non è la pompa di calore in sé: è la dispersione termica dell'edificio. Il reel spiega perché l'isolamento fa la differenza e cosa chiedere prima dell'installazione.</t>
-        </is>
-      </c>
-      <c r="F146" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Pompe di Calore</t>
-        </is>
-      </c>
-      <c r="G146" s="9" t="inlineStr">
-        <is>
-          <t>Errore comune</t>
-        </is>
-      </c>
-      <c r="H146" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I146" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J146" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="60.75" customHeight="1" s="17">
-      <c r="A147" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B147" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C147" s="28" t="inlineStr">
-        <is>
-          <t>Termostufa a pellet: si può mettere in qualsiasi stanza o ci sono limiti?</t>
-        </is>
-      </c>
-      <c r="D147" s="28" t="inlineStr">
-        <is>
-          <t>Vorrei una termostufa a pellet ma non so se posso metterla dove voglio o se ci sono vincoli di legge</t>
-        </is>
-      </c>
-      <c r="E147" s="28" t="inlineStr">
-        <is>
-          <t>Non tutte le stanze sono adatte: servono scarico fumi, areazione e distanze minime dai materiali combustibili. Il reel guida il proprietario di casa nei criteri di scelta della posizione, in modo semplice e visivo.</t>
-        </is>
-      </c>
-      <c r="F147" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Termostufe</t>
-        </is>
-      </c>
-      <c r="G147" s="9" t="inlineStr">
-        <is>
-          <t>Dove si può installare</t>
-        </is>
-      </c>
-      <c r="H147" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I147" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J147" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="45.75" customHeight="1" s="17">
-      <c r="A148" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B148" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C148" s="28" t="inlineStr">
-        <is>
-          <t>Conto Termico 2026: come funziona il rimborso e in quanto tempo arriva?</t>
-        </is>
-      </c>
-      <c r="D148" s="28" t="inlineStr">
-        <is>
-          <t>Ho sentito parlare del Conto Termico ma non capisco quando e come mi arrivano i soldi</t>
-        </is>
-      </c>
-      <c r="E148" s="28" t="inlineStr">
-        <is>
-          <t>Il Conto Termico è uno degli incentivi meno conosciuti ma più vantaggiosi per stufe, caldaie e pompe di calore. Il reel spiega in 3 passi: cos'è, chi può richiederlo, in quanto tempo arriva il rimborso — senza tecnicismi.</t>
-        </is>
-      </c>
-      <c r="F148" s="9" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G148" s="9" t="inlineStr">
-        <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H148" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I148" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J148" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="45.75" customHeight="1" s="17">
-      <c r="A149" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B149" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C149" s="28" t="inlineStr">
-        <is>
-          <t>Fotovoltaico con o senza batteria: come scegliere in base alle tue abitudini di casa</t>
-        </is>
-      </c>
-      <c r="D149" s="28" t="inlineStr">
-        <is>
-          <t>Non so se vale la pena aggiungere la batteria al fotovoltaico o se è solo una spesa in più</t>
-        </is>
-      </c>
-      <c r="E149" s="28" t="inlineStr">
-        <is>
-          <t>La scelta dipende da quando si consuma energia in casa: chi è fuori tutto il giorno trae più vantaggio dalla batteria. Il reel usa esempi pratici di famiglie tipo per aiutare lo spettatore a riconoscersi e capire cosa fa per lui.</t>
-        </is>
-      </c>
-      <c r="F149" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Batterie di Accumulo</t>
-        </is>
-      </c>
-      <c r="G149" s="9" t="inlineStr">
-        <is>
-          <t>Come scegliere il modello giusto</t>
-        </is>
-      </c>
-      <c r="H149" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I149" s="14" t="inlineStr">
-        <is>
-          <t>Shortlist</t>
-        </is>
-      </c>
-      <c r="J149" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="150" ht="60.75" customHeight="1" s="17">
-      <c r="A150" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B150" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C150" s="28" t="inlineStr">
-        <is>
-          <t>Inserto a legna al posto del caminetto aperto: cosa cambia davvero in termini di calore e sicurezza</t>
-        </is>
-      </c>
-      <c r="D150" s="28" t="inlineStr">
-        <is>
-          <t>Ho un caminetto aperto che scalda poco e fa fumo — ho sentito che l'inserto è meglio ma non so cosa aspettarmi</t>
-        </is>
-      </c>
-      <c r="E150" s="28" t="inlineStr">
-        <is>
-          <t>Il caminetto aperto disperde fino all'80% del calore. L'inserto a legna trasforma lo stesso vano in una fonte di calore efficiente, con vetro panoramico e meno rischi. Il reel mostra il confronto prima/dopo in modo visivo e immediato.</t>
-        </is>
-      </c>
-      <c r="F150" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Inserti e Camini</t>
-        </is>
-      </c>
-      <c r="G150" s="9" t="inlineStr">
-        <is>
-          <t>A cosa viene sostituito</t>
-        </is>
-      </c>
-      <c r="H150" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I150" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J150" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J140" s="15" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="45.75" customHeight="1" s="17"/>
+    <row r="142" ht="45.75" customHeight="1" s="17"/>
+    <row r="143" ht="30.75" customHeight="1" s="17"/>
+    <row r="144" ht="45.75" customHeight="1" s="17"/>
+    <row r="145" ht="45.75" customHeight="1" s="17"/>
+    <row r="146" ht="60.75" customHeight="1" s="17"/>
+    <row r="147" ht="60.75" customHeight="1" s="17"/>
+    <row r="148" ht="45.75" customHeight="1" s="17"/>
+    <row r="149" ht="45.75" customHeight="1" s="17"/>
+    <row r="150" ht="60.75" customHeight="1" s="17"/>
     <row r="151" ht="45.75" customHeight="1" s="17"/>
     <row r="152" ht="45.75" customHeight="1" s="17"/>
     <row r="153" ht="60.75" customHeight="1" s="17"/>
@@ -8154,7 +7700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8661,12 +8207,294 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" ht="32.1" customHeight="1" s="17"/>
-    <row r="14" ht="32.1" customHeight="1" s="17"/>
-    <row r="15" ht="32.1" customHeight="1" s="17"/>
-    <row r="16" ht="48" customHeight="1" s="17"/>
-    <row r="17" ht="32.1" customHeight="1" s="17"/>
-    <row r="18" ht="32.1" customHeight="1" s="17"/>
+    <row r="13" ht="32.1" customHeight="1" s="17">
+      <c r="A13" s="29" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>Stufa a pellet: 3 segnali che ti dice che è ora di cambiarla</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>La mia stufa ha 8 anni e scalda ancora — la tengo o la cambio?</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Non aspettare il guasto totale. Il reel elenca i tre sintomi che indicano che la stufa sta per cedere e perché intervenire prima conviene in termini di efficienza e incentivi disponibili.</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Stufe</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="inlineStr">
+        <is>
+          <t>Quando sostituirlo</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I13" s="30" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+      <c r="J13" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="32.1" customHeight="1" s="17">
+      <c r="A14" s="29" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a pellet: il mio camino è abbastanza grande?</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>Ho un vecchio camino e non so se posso mettere un inserto a pellet senza demolire tutto</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo le misure di apertura minima e massima per un inserto a pellet. Mostriamo anche cosa controllare sulla canna fumaria prima di chiamarci.</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H14" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+      <c r="J14" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="32.1" customHeight="1" s="17">
+      <c r="A15" s="29" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: la lasci accesa la notte o la spegni? L'errore che fa salire la bolletta</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>Uso la pompa di calore da mesi ma non so se sto sbagliando qualcosa nella gestione quotidiana</t>
+        </is>
+      </c>
+      <c r="E15" s="31" t="inlineStr">
+        <is>
+          <t>Sveliamo il contro-intuitivo: spegnerla e riaccenderla ogni giorno consuma più di tenerla a temperatura bassa di notte. Concetto di 'inerzia termica' spiegato senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I15" s="30" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+      <c r="J15" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" s="17">
+      <c r="A16" s="29" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a pellet o pompa di calore: nel 2026 quale ha più senso scegliere?</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>Non so tra caldaia a pellet e pompa di calore qual è la scelta giusta per me</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>Confronto diretto, non tecnico: quando la caldaia a pellet è la scelta giusta (casa grande, zona con legna disponibile, impianto a termosifoni esistente) e quando conviene la pompa di calore.</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G16" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H16" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I16" s="30" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+      <c r="J16" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="32.1" customHeight="1" s="17">
+      <c r="A17" s="29" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo: quando ha davvero senso installarla insieme al fotovoltaico?</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>Non capisco se la batteria è un investimento utile o solo un costo extra che mi propinano</t>
+        </is>
+      </c>
+      <c r="E17" s="31" t="inlineStr">
+        <is>
+          <t>Spieghiamo in modo pratico come funziona una batteria di accumulo abbinata al fotovoltaico, in quali situazioni domestiche fa la differenza concreta e quando invece non è prioritaria</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G17" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H17" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I17" s="30" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+      <c r="J17" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" ht="32.1" customHeight="1" s="17">
+      <c r="A18" s="29" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>Fotovoltaico con o senza batteria: come scegliere in base alle tue abitudini di casa</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>Non so se vale la pena aggiungere la batteria al fotovoltaico o se è solo una spesa in più</t>
+        </is>
+      </c>
+      <c r="E18" s="31" t="inlineStr">
+        <is>
+          <t>La scelta dipende da quando si consuma energia in casa: chi è fuori tutto il giorno trae più vantaggio dalla batteria. Il reel usa esempi pratici di famiglie tipo per aiutare lo spettatore a riconoscersi e capire cosa fa per lui.</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G18" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H18" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I18" s="30" t="inlineStr">
+        <is>
+          <t>Shortlist</t>
+        </is>
+      </c>
+      <c r="J18" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
     <row r="19" ht="48" customHeight="1" s="17"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9005,7 +8833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9079,6 +8907,206 @@
       <c r="J3" s="20" t="inlineStr">
         <is>
           <t>Priorità</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Recupero Automatico</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>Pannelli fotovoltaici con neve sopra: si fermano o producono comunque?</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Paura di perdere produzione in inverno</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Con 5 cm di neve smettono. Ma la neve scivola da sola in poche ore se i pannelli sono inclinati almeno 15°. E d'inverno con cielo sereno e freddo producono bene (i pannelli rendono meglio al freddo).</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>Recupero idee lug 2026 — routine fixata</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="inlineStr">
+        <is>
+          <t>Scartata</t>
+        </is>
+      </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Recupero Automatico</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>Termocamino ad aria o ad acqua: quale scegliere?</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Non sanno la differenza tra le due versioni</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>Ad aria: scalda solo la stanza e le adiacenti. Ad acqua: si collega ai termosifoni e scalda tutta la casa. Mostriamo quando ha senso uno e quando l'altro con esempi pratici.</t>
+        </is>
+      </c>
+      <c r="F5" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Termocamini</t>
+        </is>
+      </c>
+      <c r="G5" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H5" s="31" t="inlineStr">
+        <is>
+          <t>Recupero idee lug 2026 — routine fixata</t>
+        </is>
+      </c>
+      <c r="I5" s="30" t="inlineStr">
+        <is>
+          <t>Scartata</t>
+        </is>
+      </c>
+      <c r="J5" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Recupero Automatico</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>Solare termico sul balcone: si può fare senza tetto di proprietà?</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>Vivono in appartamento e credono di non poter installare nulla</t>
+        </is>
+      </c>
+      <c r="E6" s="31" t="inlineStr">
+        <is>
+          <t>Esistono pannelli solari termici balcone (verticali). Non sostituiscono un impianto sul tetto ma riducono del 40-50% il consumo per l'acqua calda sanitaria. Mostriamo l'opzione concreta.</t>
+        </is>
+      </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Solari</t>
+        </is>
+      </c>
+      <c r="G6" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H6" s="31" t="inlineStr">
+        <is>
+          <t>Recupero idee lug 2026 — routine fixata</t>
+        </is>
+      </c>
+      <c r="I6" s="30" t="inlineStr">
+        <is>
+          <t>Scartata</t>
+        </is>
+      </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Recupero Automatico</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>Colonnina di ricarica: dopo l'installazione come si collega all'app?</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>Non sanno che le wallbox moderne sono smart</t>
+        </is>
+      </c>
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>Le wallbox moderne hanno app: puoi programmare la ricarica di notte (quando l'energia costa meno), vedere i consumi, bloccarla da remoto. Mostriamo come funziona in 60 secondi.</t>
+        </is>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G7" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>Recupero idee lug 2026 — routine fixata</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="inlineStr">
+        <is>
+          <t>Scartata</t>
+        </is>
+      </c>
+      <c r="J7" s="30" t="inlineStr">
+        <is>
+          <t> </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master Idee 2026-07-19: 5 idee news-informed + news brief Case Green/APE/bonus
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -25,7 +25,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -7663,11 +7663,236 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="45.75" customHeight="1" s="17"/>
-    <row r="142" ht="45.75" customHeight="1" s="17"/>
-    <row r="143" ht="30.75" customHeight="1" s="17"/>
-    <row r="144" ht="45.75" customHeight="1" s="17"/>
-    <row r="145" ht="45.75" customHeight="1" s="17"/>
+    <row r="141" ht="45.75" customHeight="1" s="17">
+      <c r="A141" s="29" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B141" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C141" s="31" t="inlineStr">
+        <is>
+          <t>L'UE ha aperto la procedura d'infrazione contro l'Italia per le case green: cosa cambia davvero per la tua casa?</t>
+        </is>
+      </c>
+      <c r="D141" s="31" t="inlineStr">
+        <is>
+          <t>Paura di sanzioni imminenti o obbligo di ristrutturare dopo la notizia dell'infrazione UE, senza capire cosa si applica davvero alla propria abitazione</t>
+        </is>
+      </c>
+      <c r="E141" s="31" t="inlineStr">
+        <is>
+          <t>La Commissione europea ha aperto l'infrazione contro l'Italia per le Case Green il 15 luglio 2026. Il reel spiega cosa significa concretamente per un proprietario di prima casa: nessuna sanzione diretta, ma il tempo per adeguarsi e usare i bonus si sta accorciando. Reel di risposta immediata alla notizia del giorno.</t>
+        </is>
+      </c>
+      <c r="F141" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G141" s="30" t="inlineStr">
+        <is>
+          <t>Paura</t>
+        </is>
+      </c>
+      <c r="H141" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I141" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J141" s="30" t="n"/>
+    </row>
+    <row r="142" ht="45.75" customHeight="1" s="17">
+      <c r="A142" s="29" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B142" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C142" s="31" t="inlineStr">
+        <is>
+          <t>Dicembre 2026: perché è l'ultimo anno per installare la pompa di calore con il bonus al 50%</t>
+        </is>
+      </c>
+      <c r="D142" s="31" t="inlineStr">
+        <is>
+          <t>Non sapere se è meglio agire subito o aspettare, rischiando di perdere la percentuale di detrazione più alta della storia</t>
+        </is>
+      </c>
+      <c r="E142" s="31" t="inlineStr">
+        <is>
+          <t>Dal 2027 la detrazione scende al 36% per la prima casa. Il reel spiega chiaramente cosa cambia, quando decorre e perché chi sta valutando la pompa di calore ha convenienza ad agire entro fine anno. Nessun calcolo numerico — solo la logica della scadenza spiegata con parole semplici.</t>
+        </is>
+      </c>
+      <c r="F142" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G142" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H142" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I142" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J142" s="30" t="n"/>
+    </row>
+    <row r="143" ht="30.75" customHeight="1" s="17">
+      <c r="A143" s="29" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B143" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C143" s="31" t="inlineStr">
+        <is>
+          <t>La tua casa ha cambiato classe energetica da giugno 2026: cosa significa e cosa fare</t>
+        </is>
+      </c>
+      <c r="D143" s="31" t="inlineStr">
+        <is>
+          <t>Ricevere una valutazione APE diversa da quella di pochi anni fa senza capire se è un errore, cosa implica per vendere o affittare, e se bisogna fare lavori</t>
+        </is>
+      </c>
+      <c r="E143" s="31" t="inlineStr">
+        <is>
+          <t>Dal 29 maggio 2026 è in vigore la nuova scala di classificazione APE. Molti proprietari si ritrovano in una classe diversa rispetto a prima senza aver fatto nulla. Il reel spiega il cambio, cosa implica (vendita, bonus, locazione) e quando è il momento di intervenire.</t>
+        </is>
+      </c>
+      <c r="F143" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G143" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H143" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I143" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J143" s="30" t="n"/>
+    </row>
+    <row r="144" ht="45.75" customHeight="1" s="17">
+      <c r="A144" s="29" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B144" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C144" s="31" t="inlineStr">
+        <is>
+          <t>Hai già il fotovoltaico? Le batterie di accumulo si possono aggiungere dopo (e il bonus c'è ancora)</t>
+        </is>
+      </c>
+      <c r="D144" s="31" t="inlineStr">
+        <is>
+          <t>Credere che per avere il bonus sulle batterie bisogna installarle insieme ai pannelli, perdendo l'opportunità di potenziare un impianto già esistente</t>
+        </is>
+      </c>
+      <c r="E144" s="31" t="inlineStr">
+        <is>
+          <t>Molti proprietari con fotovoltaico già installato pensano di non avere più accesso agli incentivi per le batterie. Il reel chiarisce che le batterie sono detraibili al 50% anche in un secondo momento, indipendentemente da quando sono stati installati i pannelli. Notizia: la Legge di Bilancio 2026 ha confermato la detrazione.</t>
+        </is>
+      </c>
+      <c r="F144" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G144" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H144" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I144" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J144" s="30" t="n"/>
+    </row>
+    <row r="145" ht="45.75" customHeight="1" s="17">
+      <c r="A145" s="29" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B145" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C145" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a pellet nel caminetto che hai già: si può fare o devi rifare tutto?</t>
+        </is>
+      </c>
+      <c r="D145" s="31" t="inlineStr">
+        <is>
+          <t>Non sapere se il caminetto esistente può ospitare un inserto a pellet o se la canna fumaria è incompatibile, bloccandosi prima ancora di chiedere un preventivo</t>
+        </is>
+      </c>
+      <c r="E145" s="31" t="inlineStr">
+        <is>
+          <t>Un pain frequentissimo: chi ha già un caminetto aperto (o a legna) vorrebbe passare al pellet ma teme che la canna fumaria non vada bene o che bisogna abbattere tutto. Il reel spiega cosa si verifica in sopralluogo e in quali casi l'inserto a pellet si installa senza interventi strutturali.</t>
+        </is>
+      </c>
+      <c r="F145" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G145" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H145" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I145" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J145" s="30" t="n"/>
+    </row>
     <row r="146" ht="60.75" customHeight="1" s="17"/>
     <row r="147" ht="60.75" customHeight="1" s="17"/>
     <row r="148" ht="45.75" customHeight="1" s="17"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-20: 5 idee notturne news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -25,7 +25,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -7663,11 +7663,236 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="45.75" customHeight="1" s="17"/>
-    <row r="142" ht="45.75" customHeight="1" s="17"/>
-    <row r="143" ht="30.75" customHeight="1" s="17"/>
-    <row r="144" ht="45.75" customHeight="1" s="17"/>
-    <row r="145" ht="45.75" customHeight="1" s="17"/>
+    <row r="141" ht="45.75" customHeight="1" s="17">
+      <c r="A141" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B141" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C141" s="31" t="inlineStr">
+        <is>
+          <t>Vuoi cambiare la caldaia? Ecco perché il bonus che ti aspettavi non esiste più</t>
+        </is>
+      </c>
+      <c r="D141" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario vuole cambiare la vecchia caldaia a gas e dà per scontato di avere l'Ecobonus, poi scopre che le caldaie a gas sono ora escluse</t>
+        </is>
+      </c>
+      <c r="E141" s="31" t="inlineStr">
+        <is>
+          <t>Reel che chiarisce la svolta del 2026: le caldaie a gas non sono più coperte dall'Ecobonus. Spiega le alternative (pompa di calore, impianto ibrido, biomassa) che invece danno diritto a incentivi fino al 65% con il Conto Termico 3.0. Collegato a notizia Ecobonus luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F141" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G141" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H141" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I141" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J141" s="30" t="n"/>
+    </row>
+    <row r="142" ht="45.75" customHeight="1" s="17">
+      <c r="A142" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B142" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C142" s="31" t="inlineStr">
+        <is>
+          <t>Le classi energetiche sono cambiate a giugno 2026: cosa significa davvero per la tua casa?</t>
+        </is>
+      </c>
+      <c r="D142" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario ha sentito delle nuove classi energetiche e teme di dover fare lavori obbligatori o che la casa abbia perso valore</t>
+        </is>
+      </c>
+      <c r="E142" s="31" t="inlineStr">
+        <is>
+          <t>Reel che demistifica il nuovo APE entrato in vigore il 3 giugno 2026: nessun obbligo individuale sui privati, ma capire la classe della propria casa aiuta a scegliere i lavori giusti per risparmiare e valorizzare l'immobile. Soft CTA: valutazione energetica gratuita. Collegato a notizia Direttiva Case Green / nuovo APE luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F142" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G142" s="30" t="inlineStr">
+        <is>
+          <t>Paura</t>
+        </is>
+      </c>
+      <c r="H142" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I142" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J142" s="30" t="n"/>
+    </row>
+    <row r="143" ht="30.75" customHeight="1" s="17">
+      <c r="A143" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B143" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C143" s="31" t="inlineStr">
+        <is>
+          <t>Fotovoltaico e colonnina di ricarica insieme: l'agevolazione IVA che in pochi conoscono</t>
+        </is>
+      </c>
+      <c r="D143" s="31" t="inlineStr">
+        <is>
+          <t>Chi vuole installare il fotovoltaico e la colonnina non sa che farli insieme dà l'IVA al 10% sulla colonnina, mentre installarli separati costa il 22%</t>
+        </is>
+      </c>
+      <c r="E143" s="31" t="inlineStr">
+        <is>
+          <t>Reel pratico che spiega il vantaggio dell'installazione combinata fotovoltaico + colonnina di ricarica nello stesso cantiere: IVA al 10% invece del 22% ordinario. Posizionamento: Solare Italiano installa entrambi e conviene farlo in un unico intervento. Collegato a notizia incentivi fotovoltaico/colonnine 2026.</t>
+        </is>
+      </c>
+      <c r="F143" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G143" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H143" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I143" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J143" s="30" t="n"/>
+    </row>
+    <row r="144" ht="45.75" customHeight="1" s="17">
+      <c r="A144" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B144" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C144" s="31" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo: a cosa serve davvero e quando conviene aggiungerla al fotovoltaico</t>
+        </is>
+      </c>
+      <c r="D144" s="31" t="inlineStr">
+        <is>
+          <t>Chi ha il fotovoltaico o sta per installarlo non capisce se la batteria di accumulo è davvero utile o solo un costo aggiuntivo</t>
+        </is>
+      </c>
+      <c r="E144" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega in modo semplice cos'è una batteria di accumulo: di notte usi l'energia che hai prodotto di giorno invece di prenderla dalla rete. Senza numeri, con la logica dell'autonomia energetica. Quando aggiungerla subito e quando aspettare. Collegato a notizia detrazione 50% batterie confermata 2026.</t>
+        </is>
+      </c>
+      <c r="F144" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G144" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H144" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I144" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J144" s="30" t="n"/>
+    </row>
+    <row r="145" ht="45.75" customHeight="1" s="17">
+      <c r="A145" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B145" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C145" s="31" t="inlineStr">
+        <is>
+          <t>Termocamino a pellet o a legna: qual è la differenza e come scegliere quello giusto per la tua casa?</t>
+        </is>
+      </c>
+      <c r="D145" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario vuole un termocamino ma non sa se preferire il modello a pellet o a legna — sembrano simili ma funzionano in modo molto diverso nella vita quotidiana</t>
+        </is>
+      </c>
+      <c r="E145" s="31" t="inlineStr">
+        <is>
+          <t>Confronto diretto termocamino a pellet vs a legna: autonomia, comodità d'uso, spazio necessario per lo stoccaggio del combustibile, adattabilità alla casa. Chiusura: la scelta dipende dal tuo stile di vita, non dalla tecnologia in sé. Solare Italiano installa entrambi.</t>
+        </is>
+      </c>
+      <c r="F145" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Termocamini</t>
+        </is>
+      </c>
+      <c r="G145" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H145" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I145" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J145" s="30" t="n"/>
+    </row>
     <row r="146" ht="60.75" customHeight="1" s="17"/>
     <row r="147" ht="60.75" customHeight="1" s="17"/>
     <row r="148" ht="45.75" customHeight="1" s="17"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-21: idee notturne news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -7893,11 +7893,236 @@
       </c>
       <c r="J145" s="30" t="n"/>
     </row>
-    <row r="146" ht="60.75" customHeight="1" s="17"/>
-    <row r="147" ht="60.75" customHeight="1" s="17"/>
-    <row r="148" ht="45.75" customHeight="1" s="17"/>
-    <row r="149" ht="45.75" customHeight="1" s="17"/>
-    <row r="150" ht="60.75" customHeight="1" s="17"/>
+    <row r="146" ht="60.75" customHeight="1" s="17">
+      <c r="A146" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B146" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C146" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0 o Ecobonus: non puoi averli entrambi — qual è quello giusto per la tua pompa di calore?</t>
+        </is>
+      </c>
+      <c r="D146" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito parlare di vari bonus e non capisco quale scegliere: non voglio sbagliare e perdere soldi</t>
+        </is>
+      </c>
+      <c r="E146" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega in modo semplice la differenza pratica tra CT 3.0 (soldi subito, fondo perduto) ed Ecobonus (detrazione in 10 anni): quando conviene l'uno e quando l'altro. Ispirato da news: CT 3.0 e Ecobonus non sono cumulabili.</t>
+        </is>
+      </c>
+      <c r="F146" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G146" s="30" t="inlineStr">
+        <is>
+          <t>Confronto tra prodotti</t>
+        </is>
+      </c>
+      <c r="H146" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I146" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J146" s="30" t="n"/>
+    </row>
+    <row r="147" ht="60.75" customHeight="1" s="17">
+      <c r="A147" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B147" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C147" s="31" t="inlineStr">
+        <is>
+          <t>La tua casa è in classe F o G? Ecco cosa ti chiede davvero la Direttiva Case Green adesso (e cosa no)</t>
+        </is>
+      </c>
+      <c r="D147" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura che l'Europa mi obblighi a fare lavori costosi subito — non so se devo fare qualcosa</t>
+        </is>
+      </c>
+      <c r="E147" s="31" t="inlineStr">
+        <is>
+          <t>Reel che chiarisce: la Direttiva Case Green è in vigore ma NON obbliga interventi immediati al singolo proprietario. Spiega cosa è già cambiato (scala APE, requisiti minimi giugno 2026) e cosa arriverà nel medio periodo per le classi basse. Ispirato da news: procedura infrazione UE, EPBD in vigore.</t>
+        </is>
+      </c>
+      <c r="F147" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G147" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H147" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I147" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J147" s="30" t="n"/>
+    </row>
+    <row r="148" ht="45.75" customHeight="1" s="17">
+      <c r="A148" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B148" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C148" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore affiancata alla caldaia: esiste davvero e funziona meglio di quanto pensi</t>
+        </is>
+      </c>
+      <c r="D148" s="31" t="inlineStr">
+        <is>
+          <t>Vorrei una pompa di calore ma ho già una caldaia che funziona e temo di dover buttare via tutto</t>
+        </is>
+      </c>
+      <c r="E148" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega il sistema bivalente (pompa di calore + caldaia esistente): come si integrano, chi fa cosa al variare della temperatura esterna, e che ora è ammesso anche dal Conto Termico 3.0. Risolve il blocco psicologico 'devo rifare tutto'.</t>
+        </is>
+      </c>
+      <c r="F148" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G148" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H148" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I148" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J148" s="30" t="n"/>
+    </row>
+    <row r="149" ht="45.75" customHeight="1" s="17">
+      <c r="A149" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B149" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C149" s="31" t="inlineStr">
+        <is>
+          <t>Detrazioni al 50%: il 31 dicembre 2026 non è solo una scadenza — è un bivio che non puoi ignorare</t>
+        </is>
+      </c>
+      <c r="D149" s="31" t="inlineStr">
+        <is>
+          <t>Non so se fare i lavori adesso o aspettare — ho paura di sbagliare i tempi</t>
+        </is>
+      </c>
+      <c r="E149" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega con chiarezza: bonus edilizi confermati al 50% prima casa solo fino al 31/12/2026, dal 2027 scendono al 36%. Nessun calcolo di risparmio, solo il meccanismo normativo e la domanda semplice: 'I lavori li vuoi fare entro fine anno o aspetti?'. Ispirato da news: Bonus edilizi 2026 ultima finestra.</t>
+        </is>
+      </c>
+      <c r="F149" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G149" s="30" t="inlineStr">
+        <is>
+          <t>Domanda economica</t>
+        </is>
+      </c>
+      <c r="H149" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I149" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J149" s="30" t="n"/>
+    </row>
+    <row r="150" ht="60.75" customHeight="1" s="17">
+      <c r="A150" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B150" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C150" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore che fatica a raffreddare: lo ripari ancora o è il momento di cambiarlo?</t>
+        </is>
+      </c>
+      <c r="D150" s="31" t="inlineStr">
+        <is>
+          <t>Il mio climatizzatore non funziona più bene — non so se spendere per ripararlo o comprarne uno nuovo</t>
+        </is>
+      </c>
+      <c r="E150" s="31" t="inlineStr">
+        <is>
+          <t>Reel evergreen perfetto per luglio: segnali chiari che indicano quando ha senso riparare (guasto isolato, impianto giovane) vs quando conviene sostituire (più di 10-12 anni, gas fuori produzione, consumi alti). Nessuna cifra, solo criteri pratici da capire al volo.</t>
+        </is>
+      </c>
+      <c r="F150" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G150" s="30" t="inlineStr">
+        <is>
+          <t>Quando sostituirlo</t>
+        </is>
+      </c>
+      <c r="H150" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I150" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J150" s="30" t="n"/>
+    </row>
     <row r="151" ht="45.75" customHeight="1" s="17"/>
     <row r="152" ht="45.75" customHeight="1" s="17"/>
     <row r="153" ht="60.75" customHeight="1" s="17"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-22: 4 idee notturne news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J154"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8123,10 +8123,190 @@
       </c>
       <c r="J150" s="30" t="n"/>
     </row>
-    <row r="151" ht="45.75" customHeight="1" s="17"/>
-    <row r="152" ht="45.75" customHeight="1" s="17"/>
-    <row r="153" ht="60.75" customHeight="1" s="17"/>
-    <row r="154" ht="60.75" customHeight="1" s="17"/>
+    <row r="151" ht="45.75" customHeight="1" s="17">
+      <c r="A151" s="29" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B151" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C151" s="31" t="inlineStr">
+        <is>
+          <t>Hai installato la pompa di calore? C'è una comunicazione ENEA che devi fare entro 90 giorni — o perdi la detrazione</t>
+        </is>
+      </c>
+      <c r="D151" s="31" t="inlineStr">
+        <is>
+          <t>Ho finito i lavori, ho la fattura, ma non sapevo che bisognasse mandare qualcosa all'ENEA entro 90 giorni dalla fine cantiere</t>
+        </is>
+      </c>
+      <c r="E151" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega l'obbligo di comunicazione ENEA per ottenere la detrazione 50% su pompa di calore, climatizzatore o caldaia. Cosa succede se si supera i 90 giorni (sanzione 250€ + rimedio 'remissione in bonis'), come si invia la comunicazione. Collegato a notizia Ecobonus luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F151" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G151" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H151" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I151" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J151" s="30" t="n"/>
+    </row>
+    <row r="152" ht="45.75" customHeight="1" s="17">
+      <c r="A152" s="29" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B152" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C152" s="31" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo senza fotovoltaico: il bonus 50% vale anche in questo caso?</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="inlineStr">
+        <is>
+          <t>Voglio solo la batteria per non buttar via l'energia — non so se ho diritto al bonus senza installare anche i pannelli solari</t>
+        </is>
+      </c>
+      <c r="E152" s="31" t="inlineStr">
+        <is>
+          <t>Chiarisce la distinzione: detrazione 50% spetta per accumulo aggiunto a impianto FV (nuovo o esistente); per batteria standalone senza FV si applica solo IVA agevolata al 10%. Spiega quando conviene e quale incentivo spetta davvero nel 2026. Collegato a notizia Bonus accumulo luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F152" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G152" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H152" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I152" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J152" s="30" t="n"/>
+    </row>
+    <row r="153" ht="60.75" customHeight="1" s="17">
+      <c r="A153" s="29" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B153" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C153" s="31" t="inlineStr">
+        <is>
+          <t>Colonnina di ricarica in condominio: hai il diritto di installarla anche se il condominio dice no?</t>
+        </is>
+      </c>
+      <c r="D153" s="31" t="inlineStr">
+        <is>
+          <t>Voglio la colonnina per l'auto elettrica ma in assemblea mi hanno detto di no — non so se possono vietarmela o se ho un diritto</t>
+        </is>
+      </c>
+      <c r="E153" s="31" t="inlineStr">
+        <is>
+          <t>Spiega il diritto del singolo condomino di installare la colonnina nel proprio posto auto (D.Lgs. 48/2020), cosa può e non può decidere l'assemblea, e se la detrazione 50% vale anche per installazioni in condominio. Pain molto comune con crescita auto elettriche.</t>
+        </is>
+      </c>
+      <c r="F153" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G153" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H153" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I153" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J153" s="30" t="n"/>
+    </row>
+    <row r="154" ht="60.75" customHeight="1" s="17">
+      <c r="A154" s="29" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B154" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C154" s="31" t="inlineStr">
+        <is>
+          <t>Pannelli solari termici e pannelli fotovoltaici: non sono la stessa cosa — quale dei due fa per te?</t>
+        </is>
+      </c>
+      <c r="D154" s="31" t="inlineStr">
+        <is>
+          <t>Quando sento 'solare' non capisco se mi stanno parlando di quello per l'acqua calda o di quello per l'elettricità — e non so quale mi serve</t>
+        </is>
+      </c>
+      <c r="E154" s="31" t="inlineStr">
+        <is>
+          <t>Reel che distingue chiaramente i pannelli solari termici (producono acqua calda sanitaria e/o calore per riscaldamento) dai fotovoltaici (producono elettricità). Spiega in che caso conviene il termico (consumi alti di acqua calda, integrazione con caldaia), bonus applicabili a ciascuno, e se si possono combinare.</t>
+        </is>
+      </c>
+      <c r="F154" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Solari</t>
+        </is>
+      </c>
+      <c r="G154" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H154" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I154" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J154" s="30" t="n"/>
+    </row>
     <row r="155" ht="60.75" customHeight="1" s="17"/>
     <row r="156" ht="60.75" customHeight="1" s="17"/>
     <row r="157" ht="60.75" customHeight="1" s="17"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-23: 5 idee news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J999"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8123,11 +8123,236 @@
       </c>
       <c r="J150" s="30" t="n"/>
     </row>
-    <row r="151" ht="45.75" customHeight="1" s="17"/>
-    <row r="152" ht="45.75" customHeight="1" s="17"/>
-    <row r="153" ht="60.75" customHeight="1" s="17"/>
-    <row r="154" ht="60.75" customHeight="1" s="17"/>
-    <row r="155" ht="60.75" customHeight="1" s="17"/>
+    <row r="151" ht="45.75" customHeight="1" s="17">
+      <c r="A151" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B151" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C151" s="31" t="inlineStr">
+        <is>
+          <t>L'Europa mette l'Italia sotto infrazione per le Case Green: cosa cambia davvero per chi ha casa</t>
+        </is>
+      </c>
+      <c r="D151" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito la notizia al TG ma non capisco se devo fare qualcosa alla mia casa</t>
+        </is>
+      </c>
+      <c r="E151" s="31" t="inlineStr">
+        <is>
+          <t>Reel chiarificatore post-notizia del 15 luglio: spiega in termini semplici cosa significa procedura d'infrazione UE, che non ci sono obblighi immediati per i privati, ma che il tema è destinato a diventare sempre più concreto. Smonta la paura, orienta verso la riqualificazione come scelta proattiva.</t>
+        </is>
+      </c>
+      <c r="F151" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G151" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H151" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I151" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J151" s="30" t="n"/>
+    </row>
+    <row r="152" ht="45.75" customHeight="1" s="17">
+      <c r="A152" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B152" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C152" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0: non è solo per i Comuni — ecco chi può davvero fare domanda</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="inlineStr">
+        <is>
+          <t>Pensavo che il Conto Termico fosse roba da PA o grandi imprese, non per me</t>
+        </is>
+      </c>
+      <c r="E152" s="31" t="inlineStr">
+        <is>
+          <t>Reel che chiarisce la platea del CT 3.0: privati, condomini, imprese, enti terzo settore. Smonta il mito che sia riservato agli enti pubblici. Concretizza: 'Se stai mettendo una pompa di calore o sostituendo la caldaia, puoi fare domanda anche tu'. Collegato alla riapertura del portale aprile 2026.</t>
+        </is>
+      </c>
+      <c r="F152" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G152" s="30" t="inlineStr">
+        <is>
+          <t>Scetticismo</t>
+        </is>
+      </c>
+      <c r="H152" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I152" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J152" s="30" t="n"/>
+    </row>
+    <row r="153" ht="60.75" customHeight="1" s="17">
+      <c r="A153" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B153" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C153" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: ogni quanto si fa la manutenzione e quanto dura davvero</t>
+        </is>
+      </c>
+      <c r="D153" s="31" t="inlineStr">
+        <is>
+          <t>Ho installato (o sto valutando) la pompa di calore ma non so se richiede manutenzione e quanto mi costerà nel tempo</t>
+        </is>
+      </c>
+      <c r="E153" s="31" t="inlineStr">
+        <is>
+          <t>Reel pratico: manutenzione annuale consigliata, cosa controlla il tecnico, costi medi, aspettativa di vita 15-20 anni. Rassicura chi ha già comprato e aiuta chi deve decidere confrontandola con la caldaia tradizionale.</t>
+        </is>
+      </c>
+      <c r="F153" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G153" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H153" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I153" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J153" s="30" t="n"/>
+    </row>
+    <row r="154" ht="60.75" customHeight="1" s="17">
+      <c r="A154" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B154" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C154" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a pellet: ogni quanto va pulito e cosa rischi se lo trascuri</t>
+        </is>
+      </c>
+      <c r="D154" s="31" t="inlineStr">
+        <is>
+          <t>Ho l'inserto a pellet ma nessuno mi ha mai spiegato chiaramente ogni quanto pulirlo e cosa succede se non lo faccio</t>
+        </is>
+      </c>
+      <c r="E154" s="31" t="inlineStr">
+        <is>
+          <t>Reel in 3 step: pulizia quotidiana (cenere braciere), mensile (vetrino, deflettore), annuale da tecnico (canna fumaria, scambiatore). Mostra in modo visivo le conseguenze della mancata manutenzione: perdita di efficienza, guasti, rischi. Tono pratico, non allarmista.</t>
+        </is>
+      </c>
+      <c r="F154" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G154" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H154" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I154" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J154" s="30" t="n"/>
+    </row>
+    <row r="155" ht="60.75" customHeight="1" s="17">
+      <c r="A155" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Fotovoltaico con batteria: l'IVA agevolata al 10% che puoi avere (ma pochissimi sanno di chiedere)</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito che c'è qualche agevolazione IVA sul fotovoltaico ma non so se vale per me o come ottenerla</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega l'IVA al 10% (vs 22% standard) per impianti fotovoltaici con batterie installati in contesto di ristrutturazione. Chi la ottiene, quando spetta, cosa chiedere esplicitamente all'installatore prima di firmare il preventivo. Concreta e azionabile.</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
     <row r="156" ht="60.75" customHeight="1" s="17"/>
     <row r="157" ht="60.75" customHeight="1" s="17"/>
     <row r="158" ht="45.75" customHeight="1" s="17"/>
@@ -8138,6 +8363,840 @@
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-24: 5 idee news-informed + news brief luglio 2026
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J155"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8123,11 +8123,236 @@
       </c>
       <c r="J150" s="30" t="n"/>
     </row>
-    <row r="151" ht="45.75" customHeight="1" s="17"/>
-    <row r="152" ht="45.75" customHeight="1" s="17"/>
-    <row r="153" ht="60.75" customHeight="1" s="17"/>
-    <row r="154" ht="60.75" customHeight="1" s="17"/>
-    <row r="155" ht="60.75" customHeight="1" s="17"/>
+    <row r="151" ht="45.75" customHeight="1" s="17">
+      <c r="A151" s="29" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B151" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C151" s="31" t="inlineStr">
+        <is>
+          <t>Bonus colonnina di ricarica 2026: ti rimborsano l'80% del costo — ma devi fare domanda nel modo giusto</t>
+        </is>
+      </c>
+      <c r="D151" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito che c'è un bonus per installare la colonnina a casa, ma non so se mi spetta, quanti soldi prendo e come chiederlo</t>
+        </is>
+      </c>
+      <c r="E151" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega il nuovo bonus colonnine domestiche (DPCM Automotive giugno 2026): 80% rimborsato, max 1.500€ per privati e 8.000€ per condomini, accessibile solo a privati (no partita IVA), domanda da fare tramite portale MIMIT. Collegato a notizia reale luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F151" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G151" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H151" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I151" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J151" s="30" t="n"/>
+    </row>
+    <row r="152" ht="45.75" customHeight="1" s="17">
+      <c r="A152" s="29" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B152" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C152" s="31" t="inlineStr">
+        <is>
+          <t>L'UE ha messo sotto infrazione l'Italia sulla Direttiva Case Green: cosa devi fare tu adesso (e cosa no)</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito che l'Europa ha aperto una procedura contro l'Italia sulle case — non so se devo fare qualcosa subito o aspettare</t>
+        </is>
+      </c>
+      <c r="E152" s="31" t="inlineStr">
+        <is>
+          <t>Reel che demistifica la notizia del 15 luglio 2026 (infrazione UE per mancato recepimento EPBD): spiegare cosa è successo davvero, che scadenze contano per i proprietari di casa, se conviene agire adesso o aspettare la normativa italiana, e cosa fa cambiare l'APE aggiornato dal 3 giugno 2026. Collegato a notizia reale luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F152" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G152" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H152" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I152" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J152" s="30" t="n"/>
+    </row>
+    <row r="153" ht="60.75" customHeight="1" s="17">
+      <c r="A153" s="29" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B153" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C153" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0: puoi aggiungere una pompa di calore senza smontare la caldaia — e lo Stato ti rimborsa il 65%</t>
+        </is>
+      </c>
+      <c r="D153" s="31" t="inlineStr">
+        <is>
+          <t>Ho già una caldaia e vorrei la pompa di calore, ma pensavo di dover buttare tutto e non me lo posso permettere</t>
+        </is>
+      </c>
+      <c r="E153" s="31" t="inlineStr">
+        <is>
+          <t>Reel su una delle novità più concrete del Conto Termico 3.0 (DM agosto 2025, in vigore 2026): i sistemi ibridi/bivalenti e le pompe di calore add-on sono ora ammesse al rimborso. Non serve demolire l'impianto esistente. Si può integrare e ricevere fino al 65% dalla spesa. Chiarire anche che il Portaltermico 3.0 è attivo dal febbraio 2026. Collegato a notizia reale.</t>
+        </is>
+      </c>
+      <c r="F153" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G153" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H153" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I153" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J153" s="30" t="n"/>
+    </row>
+    <row r="154" ht="60.75" customHeight="1" s="17">
+      <c r="A154" s="29" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B154" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C154" s="31" t="inlineStr">
+        <is>
+          <t>Hai già il fotovoltaico? Ecco come recuperare il 50% aggiungendo una batteria di accumulo nel 2026</t>
+        </is>
+      </c>
+      <c r="D154" s="31" t="inlineStr">
+        <is>
+          <t>Ho già i pannelli fotovoltaici ma non ho la batteria — non so se ho ancora diritto al bonus o se era solo per chi parte da zero</t>
+        </is>
+      </c>
+      <c r="E154" s="31" t="inlineStr">
+        <is>
+          <t>Reel che risponde a un dubbio concreto e frequente: la detrazione del 50% per le batterie di accumulo vale anche per chi ha già l'impianto fotovoltaico installato (non solo per chi lo installa nuovo). Spiegare il massimale di spesa (96.000€), le 10 rate annuali IRPEF, e la differenza prima/seconda casa (50% vs 36%). Collegato a notizia reale (conferma Legge di Bilancio 2026).</t>
+        </is>
+      </c>
+      <c r="F154" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G154" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H154" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I154" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J154" s="30" t="n"/>
+    </row>
+    <row r="155" ht="60.75" customHeight="1" s="17">
+      <c r="A155" s="29" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Ecobonus 2026: sconto in fattura e cessione del credito non esistono più — adesso come recuperi i soldi</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Pensavo di poter fare la detrazione senza tirar fuori i soldi subito — mi hanno detto che non si può più fare: e allora come funziona adesso?</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Reel che affronta uno dei malintesi più comuni del 2026: molti ancora si aspettano lo sconto in fattura o la cessione del credito per i lavori di efficienza (pompa di calore, solare, caldaia). Chiarire che dal 2023 questi strumenti sono stati eliminati per i privati, e che adesso la detrazione si recupera solo in dichiarazione dei redditi in 10 rate. Collegato a notizia reale (Ecobonus 2026).</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Domanda economica</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
     <row r="156" ht="60.75" customHeight="1" s="17"/>
     <row r="157" ht="60.75" customHeight="1" s="17"/>
     <row r="158" ht="45.75" customHeight="1" s="17"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-25: 4 idee news-informed + news brief
- FAQ: infrazione UE Case Green (notizia 15 luglio 2026)
- Pompa di calore: portale CT3.0 riaperto dopo blocco marzo
- Pompa di calore: doppia funzione riscaldamento+raffrescamento
- Caldaie: scadenza detrazione 50% fine 2026
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J999"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8123,10 +8123,190 @@
       </c>
       <c r="J150" s="30" t="n"/>
     </row>
-    <row r="151" ht="45.75" customHeight="1" s="17"/>
-    <row r="152" ht="45.75" customHeight="1" s="17"/>
-    <row r="153" ht="60.75" customHeight="1" s="17"/>
-    <row r="154" ht="60.75" customHeight="1" s="17"/>
+    <row r="151" ht="45.75" customHeight="1" s="17">
+      <c r="A151" s="29" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B151" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C151" s="31" t="inlineStr">
+        <is>
+          <t>L'Europa ha aperto una procedura d'infrazione sull'Italia per la Direttiva Case Green: cosa cambia davvero per chi ha una casa?</t>
+        </is>
+      </c>
+      <c r="D151" s="31" t="inlineStr">
+        <is>
+          <t>Paura di obbligo immediato di ristrutturare dopo la notizia dell'infrazione UE</t>
+        </is>
+      </c>
+      <c r="E151" s="31" t="inlineStr">
+        <is>
+          <t>Il reel spiega che la procedura d'infrazione riguarda lo Stato italiano, non il singolo proprietario. Nessun obbligo immediato di ristrutturare. Significa però che il recepimento della direttiva accelererà e i requisiti minimi arriveranno. Meglio conoscere già la classe energetica della propria casa e sapere che esistono incentivi attivi oggi.</t>
+        </is>
+      </c>
+      <c r="F151" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G151" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H151" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I151" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J151" s="30" t="n"/>
+    </row>
+    <row r="152" ht="45.75" customHeight="1" s="17">
+      <c r="A152" s="29" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B152" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C152" s="31" t="inlineStr">
+        <is>
+          <t>Il portale Conto Termico 3.0 era bloccato a marzo — ma ha riaperto: puoi ancora fare domanda per la pompa di calore</t>
+        </is>
+      </c>
+      <c r="D152" s="31" t="inlineStr">
+        <is>
+          <t>Non sa che dopo il blocco del portale si può ancora accedere all'incentivo CT3.0</t>
+        </is>
+      </c>
+      <c r="E152" s="31" t="inlineStr">
+        <is>
+          <t>Il reel racconta cosa è successo: il portale GSE ha aperto a febbraio, poi si è bloccato a marzo per eccesso di domande, ed è riaperto ad aprile con proroga dei termini. Chi vuole installare una pompa di calore può ancora presentare domanda nel 2026. Spiega i tre passi essenziali: preventivo tecnico, tecnico abilitato, IBAN per il rimborso diretto.</t>
+        </is>
+      </c>
+      <c r="F152" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G152" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H152" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I152" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J152" s="30" t="n"/>
+    </row>
+    <row r="153" ht="60.75" customHeight="1" s="17">
+      <c r="A153" s="29" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B153" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C153" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: in tanti pensano serva solo per riscaldare — ma fa anche il lavoro del climatizzatore. Ecco come funziona</t>
+        </is>
+      </c>
+      <c r="D153" s="31" t="inlineStr">
+        <is>
+          <t>Ha caldaia e climatizzatore separati e non sa che potrebbe avere un unico sistema</t>
+        </is>
+      </c>
+      <c r="E153" s="31" t="inlineStr">
+        <is>
+          <t>Il reel spiega la doppia funzione della pompa di calore: riscalda d'inverno, raffredda d'estate. È un sostituto sia della caldaia che del climatizzatore. Un solo impianto, meno manutenzione, meno spazio. Con gli incentivi 2026 (CT3.0 o Ecobonus) il momento è favorevole.</t>
+        </is>
+      </c>
+      <c r="F153" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G153" s="30" t="inlineStr">
+        <is>
+          <t>A cosa viene sostituito</t>
+        </is>
+      </c>
+      <c r="H153" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I153" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J153" s="30" t="n"/>
+    </row>
+    <row r="154" ht="60.75" customHeight="1" s="17">
+      <c r="A154" s="29" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B154" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C154" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia nuova nel 2026 o nel 2027? C'è una differenza che vale — e non è il prezzo della caldaia</t>
+        </is>
+      </c>
+      <c r="D154" s="31" t="inlineStr">
+        <is>
+          <t>Non sa che la detrazione per la sostituzione della caldaia scende dal 50% al 36% a gennaio 2027</t>
+        </is>
+      </c>
+      <c r="E154" s="31" t="inlineStr">
+        <is>
+          <t>Il reel spiega in modo semplice: chi sostituisce la caldaia entro il 31 dicembre 2026 ha la detrazione al 50% (prima casa). Dal 1° gennaio 2027 scende al 36%. Non è un invito a decidere in fretta — è un'informazione che molti non hanno e che può influenzare la pianificazione dei lavori.</t>
+        </is>
+      </c>
+      <c r="F154" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G154" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H154" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I154" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J154" s="30" t="n"/>
+    </row>
     <row r="155" ht="60.75" customHeight="1" s="17"/>
     <row r="156" ht="60.75" customHeight="1" s="17"/>
     <row r="157" ht="60.75" customHeight="1" s="17"/>
@@ -8138,6 +8318,840 @@
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-26: 4 idee news-informed + news brief luglio 2026
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8307,10 +8307,190 @@
       </c>
       <c r="J154" s="30" t="n"/>
     </row>
-    <row r="155" ht="60.75" customHeight="1" s="17"/>
-    <row r="156" ht="60.75" customHeight="1" s="17"/>
-    <row r="157" ht="60.75" customHeight="1" s="17"/>
-    <row r="158" ht="45.75" customHeight="1" s="17"/>
+    <row r="155" ht="60.75" customHeight="1" s="17">
+      <c r="A155" s="29" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore add-on: si aggancia alla caldaia che hai già e accede agli incentivi del Conto Termico 3.0</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Voglio passare alla pompa di calore ma non voglio (o non posso) rifare tutto l'impianto di riscaldamento</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Spiega cos'è la pompa di calore add-on (o bivalente), introdotta come tecnologia incentivata nel Conto Termico 3.0. Si affianca alla caldaia esistente senza smontarla: gestisce il riscaldamento quando fa meno freddo, lascia lavorare la caldaia nei picchi di freddo. Ideale per chi ha radiatori e non vuole un'installazione invasiva.</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
+    <row r="156" ht="60.75" customHeight="1" s="17">
+      <c r="A156" s="29" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B156" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C156" s="31" t="inlineStr">
+        <is>
+          <t>Pannello solare termico o fotovoltaico: non sono la stessa cosa — quale fa al caso tuo?</t>
+        </is>
+      </c>
+      <c r="D156" s="31" t="inlineStr">
+        <is>
+          <t>Sento sempre parlare di solare ma non capisco se fa l'acqua calda o la corrente elettrica</t>
+        </is>
+      </c>
+      <c r="E156" s="31" t="inlineStr">
+        <is>
+          <t>Chiarisce la differenza fondamentale: il solare termico scalda l'acqua (doccia, cucina) riducendo la bolletta del gas, il fotovoltaico produce elettricità. Spiega i casi d'uso tipici, chi è il candidato ideale per il solare termico (chi spende molto per l'acqua calda, ha già una caldaia), e gli incentivi disponibili per ciascuno.</t>
+        </is>
+      </c>
+      <c r="F156" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Solari</t>
+        </is>
+      </c>
+      <c r="G156" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H156" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I156" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J156" s="30" t="n"/>
+    </row>
+    <row r="157" ht="60.75" customHeight="1" s="17">
+      <c r="A157" s="29" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B157" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C157" s="31" t="inlineStr">
+        <is>
+          <t>Colonnina di ricarica in condominio: il condominio può impedirti di installarla?</t>
+        </is>
+      </c>
+      <c r="D157" s="31" t="inlineStr">
+        <is>
+          <t>Ho un'auto elettrica (o ci sto pensando) ma non so se il condominio può bloccarmi l'installazione della colonnina</t>
+        </is>
+      </c>
+      <c r="E157" s="31" t="inlineStr">
+        <is>
+          <t>Spiega la normativa italiana che tutela il diritto del condomino di installare la colonnina a proprie spese nel proprio posto auto senza bisogno del voto dell'assemblea (basta una comunicazione). Chiarisce i limiti pratici (impianto condominiale comune, potenza disponibile) e quando invece è necessario un accordo. Reel rassicurante e concreto.</t>
+        </is>
+      </c>
+      <c r="F157" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G157" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H157" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I157" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J157" s="30" t="n"/>
+    </row>
+    <row r="158" ht="45.75" customHeight="1" s="17">
+      <c r="A158" s="29" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B158" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C158" s="31" t="inlineStr">
+        <is>
+          <t>La Direttiva Case Green: l'UE ha aperto la procedura d'infrazione contro tutti e 27 i paesi — cosa cambia davvero per chi ha casa in Italia</t>
+        </is>
+      </c>
+      <c r="D158" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura di dover ristrutturare casa per forza e non so se ho scadenze immediate da rispettare</t>
+        </is>
+      </c>
+      <c r="E158" s="31" t="inlineStr">
+        <is>
+          <t>Aggiornamento luglio 2026: la Commissione ha aperto la procedura contro tutti i 27 Stati (non solo Italia) per mancato recepimento EPBD entro maggio 2026. Messaggio rassicurante: nessun obbligo retroattivo per i privati, il recepimento italiano è atteso entro dicembre 2026. Spiega cosa succederà nei prossimi mesi e perché conviene comunque non aspettare se stai già pensando a efficienza energetica.</t>
+        </is>
+      </c>
+      <c r="F158" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G158" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H158" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I158" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J158" s="30" t="n"/>
+    </row>
     <row r="159" ht="45.75" customHeight="1" s="17"/>
     <row r="160" ht="60.75" customHeight="1" s="17"/>
     <row r="161" ht="76.5" customHeight="1" s="17"/>
@@ -8318,840 +8498,6 @@
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-27: 5 idee news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J159"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8307,851 +8307,242 @@
       </c>
       <c r="J154" s="30" t="n"/>
     </row>
-    <row r="155" ht="60.75" customHeight="1" s="17"/>
-    <row r="156" ht="60.75" customHeight="1" s="17"/>
-    <row r="157" ht="60.75" customHeight="1" s="17"/>
-    <row r="158" ht="45.75" customHeight="1" s="17"/>
-    <row r="159" ht="45.75" customHeight="1" s="17"/>
+    <row r="155" ht="60.75" customHeight="1" s="17">
+      <c r="A155" s="29" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a pellet nel 2026: il Conto Termico 3.0 la finanzia ancora o è esclusa come quella a gas?</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario pensa che 'le caldaie non hanno più incentivi' senza sapere che la biomassa/pellet è trattata diversamente dalla caldaia a gas</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Reel che chiarisce: caldaie a gas escluse da tutti gli incentivi dal 2025, ma le caldaie a biomassa/pellet sono ancora incentivate con Conto Termico 3.0 (rimborso diretto fino al 65%). Call to action: 'Stai valutando di sostituire la caldaia? Chiedici un preventivo — l'incentivo c'è ancora.'</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
+    <row r="156" ht="60.75" customHeight="1" s="17">
+      <c r="A156" s="29" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B156" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C156" s="31" t="inlineStr">
+        <is>
+          <t>Ho già il fotovoltaico: se aggiungo la batteria di accumulo adesso, ho ancora l'IVA al 10%?</t>
+        </is>
+      </c>
+      <c r="D156" s="31" t="inlineStr">
+        <is>
+          <t>Chi ha installato il fotovoltaico anni fa pensa che l'IVA ridotta al 10% valga solo se si installano pannelli e batteria nello stesso momento</t>
+        </is>
+      </c>
+      <c r="E156" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega: l'IVA al 10% si applica all'installazione della batteria di accumulo anche aggiunta in un secondo momento a un impianto fotovoltaico esistente. Si abbina anche la detrazione 50% (prima casa). Call to action: 'Hai il fotovoltaico e pensi alla batteria? Vediamo insieme cosa ti spetta.'</t>
+        </is>
+      </c>
+      <c r="F156" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G156" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H156" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I156" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J156" s="30" t="n"/>
+    </row>
+    <row r="157" ht="60.75" customHeight="1" s="17">
+      <c r="A157" s="29" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B157" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C157" s="31" t="inlineStr">
+        <is>
+          <t>Stufa a legna o a pellet in appartamento: si può installare o ci sono divieti automatici?</t>
+        </is>
+      </c>
+      <c r="D157" s="31" t="inlineStr">
+        <is>
+          <t>Chi vive in appartamento o condominio dà per scontato di non poter installare una stufa e rinuncia senza nemmeno chiedere</t>
+        </is>
+      </c>
+      <c r="E157" s="31" t="inlineStr">
+        <is>
+          <t>Reel che sfata il mito: dipende dalla canna fumaria condominiale disponibile, dalle normative locali e dall'approvazione del condominio. Con la canna fumaria giusta e la stufa certificata, in molti casi si può. Call to action: 'Chiedi un sopralluogo — valutiamo insieme se è fattibile nel tuo appartamento.'</t>
+        </is>
+      </c>
+      <c r="F157" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Stufe</t>
+        </is>
+      </c>
+      <c r="G157" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H157" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I157" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J157" s="30" t="n"/>
+    </row>
+    <row r="158" ht="45.75" customHeight="1" s="17">
+      <c r="A158" s="29" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B158" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C158" s="31" t="inlineStr">
+        <is>
+          <t>Il Piano Nazionale di Ristrutturazione arriva entro fine 2026: cosa cambia davvero per chi ha una casa in classe E?</t>
+        </is>
+      </c>
+      <c r="D158" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario con casa in classe E teme di ricevere obblighi improvvisi — non sa che il piano non è ancora vigente e che gli obblighi arriveranno gradualmente</t>
+        </is>
+      </c>
+      <c r="E158" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega la sequenza: l'Italia deve presentare il Piano entro dicembre 2026, ma gli obblighi concreti per i privati scatteranno solo dopo il recepimento con scadenze graduate (classe E residenziale: 2033). Nessun panico — ma conviene informarsi e pianificare adesso. Agganciato alla notizia: procedura infrazione UE del 15/07/2026.</t>
+        </is>
+      </c>
+      <c r="F158" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G158" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H158" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I158" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J158" s="30" t="n"/>
+    </row>
+    <row r="159" ht="45.75" customHeight="1" s="17">
+      <c r="A159" s="29" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B159" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C159" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore aria-acqua con i radiatori che ho già: funziona davvero o devo rifare tutto l'impianto?</t>
+        </is>
+      </c>
+      <c r="D159" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario con riscaldamento a radiatori tradizionali pensa di non poter installare una pompa di calore senza rifare completamente l'impianto idraulico</t>
+        </is>
+      </c>
+      <c r="E159" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega due soluzioni concrete: 1) pompe di calore a bassa temperatura di nuova generazione compatibili con radiatori esistenti (se dimensionamento corretto); 2) sistema ibrido PdC + caldaia esistente che non richiede di toccare i radiatori. Call to action: 'Hai i radiatori? Vieni a sentirti dire se la pompa di calore è compatibile.'</t>
+        </is>
+      </c>
+      <c r="F159" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G159" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H159" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I159" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J159" s="30" t="n"/>
+    </row>
     <row r="160" ht="60.75" customHeight="1" s="17"/>
     <row r="161" ht="76.5" customHeight="1" s="17"/>
     <row r="162" ht="60.75" customHeight="1" s="17"/>
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-28: 4 idee news-informed + news brief
- 4 nuove idee in Master Idee (righe 155-158)
- News brief: 5 notizie rilevanti (APE nuovi criteri, CT3.0 regola fotovoltaico, ENEA 90gg, batterie accumulo)
- Categorie: FAQ x2, Pompe di Calore, Batterie di Accumulo
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8307,10 +8307,190 @@
       </c>
       <c r="J154" s="30" t="n"/>
     </row>
-    <row r="155" ht="60.75" customHeight="1" s="17"/>
-    <row r="156" ht="60.75" customHeight="1" s="17"/>
-    <row r="157" ht="60.75" customHeight="1" s="17"/>
-    <row r="158" ht="45.75" customHeight="1" s="17"/>
+    <row r="155" ht="60.75" customHeight="1" s="17">
+      <c r="A155" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Il nuovo APE può abbassarti la classe energetica senza che tu abbia fatto nulla — e cosa puoi fare adesso</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Devo richiedere un nuovo APE e temo di scoprire una classe energetica peggiore rispetto a quella attuale, senza aver fatto lavori</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Dal 3 giugno 2026 i criteri di valutazione dell'APE sono cambiati (metodi più rigorosi, analisi dei ponti termici). Un APE rifatto oggi potrebbe certificare una classe più bassa rispetto a uno vecchio. Ma la soluzione esiste: interventi mirati (pompa di calore, nuova caldaia, pannelli) possono far risalire la classe. Reel fear → soluzione.</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Paura</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
+    <row r="156" ht="60.75" customHeight="1" s="17">
+      <c r="A156" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B156" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C156" s="31" t="inlineStr">
+        <is>
+          <t>Vuoi il Conto Termico per la pompa di calore e anche il fotovoltaico? C'è una regola che devi sapere prima</t>
+        </is>
+      </c>
+      <c r="D156" s="31" t="inlineStr">
+        <is>
+          <t>Sto valutando pompa di calore + fotovoltaico e non so se posso usare il Conto Termico 3.0 per entrambi o solo per uno</t>
+        </is>
+      </c>
+      <c r="E156" s="31" t="inlineStr">
+        <is>
+          <t>Spiegare la regola specifica del CT3.0: il fotovoltaico viene incentivato SOLO come intervento accessorio a una pompa di calore installata nello stesso intervento — non da solo. Se installi i due prodotti in momenti diversi, il fotovoltaico non rientra nel CT3. Reel pratico 'prima di firmare, guarda questo'.</t>
+        </is>
+      </c>
+      <c r="F156" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G156" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H156" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I156" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J156" s="30" t="n"/>
+    </row>
+    <row r="157" ht="60.75" customHeight="1" s="17">
+      <c r="A157" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B157" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C157" s="31" t="inlineStr">
+        <is>
+          <t>Hai finito i lavori con l'Ecobonus — ma se non mandi questo documento all'ENEA entro 90 giorni, perdi tutto</t>
+        </is>
+      </c>
+      <c r="D157" s="31" t="inlineStr">
+        <is>
+          <t>Ho terminato i lavori e preso l'Ecobonus, ma non sapevo dell'obbligo di comunicazione ENEA — rischio di perdere la detrazione</t>
+        </is>
+      </c>
+      <c r="E157" s="31" t="inlineStr">
+        <is>
+          <t>Spiegare l'obbligo di trasmissione telematica all'ENEA entro 90 giorni dal termine lavori, pena la decadenza della detrazione del 50%. Molti lo scoprono solo in fase di dichiarazione dei redditi. Reel urgente e pratico: 'controlla la data, poi fai questo'. Applicabile a pompe di calore, caldaie, fotovoltaico, climatizzatori.</t>
+        </is>
+      </c>
+      <c r="F157" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G157" s="30" t="inlineStr">
+        <is>
+          <t>Paura</t>
+        </is>
+      </c>
+      <c r="H157" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I157" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J157" s="30" t="n"/>
+    </row>
+    <row r="158" ht="45.75" customHeight="1" s="17">
+      <c r="A158" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B158" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C158" s="31" t="inlineStr">
+        <is>
+          <t>Hai già il fotovoltaico da anni? La batteria di accumulo si aggiunge dopo — e il bonus del 50% vale uguale</t>
+        </is>
+      </c>
+      <c r="D158" s="31" t="inlineStr">
+        <is>
+          <t>Penso che il bonus per le batterie di accumulo valga solo se installo fotovoltaico e batteria insieme, non se ho già i pannelli</t>
+        </is>
+      </c>
+      <c r="E158" s="31" t="inlineStr">
+        <is>
+          <t>Sfatare il mito che la detrazione del 50% per le batterie di accumulo sia riservata a chi installa tutto insieme. Chi ha già il fotovoltaico da 2, 5 o 10 anni può aggiungere la batteria in un secondo momento e accedere al bonus normalmente. Reel diretto: 'hai i pannelli? Il bonus batteria è tuo anche adesso'.</t>
+        </is>
+      </c>
+      <c r="F158" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G158" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H158" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I158" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J158" s="30" t="n"/>
+    </row>
     <row r="159" ht="45.75" customHeight="1" s="17"/>
     <row r="160" ht="60.75" customHeight="1" s="17"/>
     <row r="161" ht="76.5" customHeight="1" s="17"/>
@@ -8318,840 +8498,6 @@
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Archivio 2026-07-28: 8 idee in Produzione spostate in Libreria Contenuti
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P542iGw78tuf7xgmGVUjFd
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -6435,46 +6435,46 @@
     </row>
     <row r="116" ht="45.75" customHeight="1" s="17">
       <c r="A116" s="11" t="n">
-        <v>46165</v>
+        <v>46218</v>
       </c>
       <c r="B116" s="9" t="inlineStr">
         <is>
-          <t>Topic mese</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C116" s="28" t="inlineStr">
         <is>
-          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
+          <t>Pompa di calore ibrida: tiene anche la caldaia? E perché non è un difetto</t>
         </is>
       </c>
       <c r="D116" s="28" t="inlineStr">
         <is>
-          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
+          <t>Non capisco se la pompa di calore ibrida è peggio di una normale</t>
         </is>
       </c>
       <c r="E116" s="28" t="inlineStr">
         <is>
-          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
+          <t>Spieghiamo cos'è la pompa di calore ibrida (PdC + caldaia nello stesso impianto), quando si usa l'una e quando l'altra, e perché in certe case è la scelta più intelligente — senza tecnicismi.</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G116" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H116" s="28" t="inlineStr">
         <is>
-          <t>Topic mese: climatizzazione estiva privati</t>
+          <t>Generato automaticamente di notte</t>
         </is>
       </c>
       <c r="I116" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J116" s="15" t="inlineStr">
@@ -6485,7 +6485,7 @@
     </row>
     <row r="117" ht="45.75" customHeight="1" s="17">
       <c r="A117" s="11" t="n">
-        <v>46170</v>
+        <v>46218</v>
       </c>
       <c r="B117" s="9" t="inlineStr">
         <is>
@@ -6494,27 +6494,27 @@
       </c>
       <c r="C117" s="28" t="inlineStr">
         <is>
-          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
+          <t>Termostufa a legna: il calore arriva davvero in tutta la casa o rimane nel salotto?</t>
         </is>
       </c>
       <c r="D117" s="28" t="inlineStr">
         <is>
-          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
+          <t>Ho paura che la termostufa scaldi solo dove c'è il fuoco</t>
         </is>
       </c>
       <c r="E117" s="28" t="inlineStr">
         <is>
-          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
+          <t>Mostriamo la differenza tra una stufa normale e una termostufa: i radiatori distribuiscono il calore prodotto dal fuoco in tutti gli ambienti, anche ai piani superiori. Visivo e concreto.</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Prodotto - Termostufe</t>
         </is>
       </c>
       <c r="G117" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H117" s="28" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="I117" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J117" s="15" t="inlineStr">
@@ -6535,7 +6535,7 @@
     </row>
     <row r="118" ht="60.75" customHeight="1" s="17">
       <c r="A118" s="11" t="n">
-        <v>46171</v>
+        <v>46218</v>
       </c>
       <c r="B118" s="9" t="inlineStr">
         <is>
@@ -6544,27 +6544,27 @@
       </c>
       <c r="C118" s="28" t="inlineStr">
         <is>
-          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
+          <t>Incentivi 2026: li gestite voi o devo occuparmi io della burocrazia?</t>
         </is>
       </c>
       <c r="D118" s="28" t="inlineStr">
         <is>
-          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
+          <t>Ho paura di dover fare da solo le domande per i bonus e sbagliare</t>
         </is>
       </c>
       <c r="E118" s="28" t="inlineStr">
         <is>
-          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
+          <t>Risposta diretta e rassicurante: spieghiamo chi fa cosa, dal sopralluogo alla pratica incentivo. Obiettivo: togliere il timore burocratico che blocca la decisione di chiamarci.</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pannelli Fotovoltaici</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G118" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H118" s="28" t="inlineStr">
@@ -6574,7 +6574,7 @@
       </c>
       <c r="I118" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J118" s="15" t="inlineStr">
@@ -6585,42 +6585,46 @@
     </row>
     <row r="119" ht="45.75" customHeight="1" s="17">
       <c r="A119" s="11" t="n">
-        <v>46148</v>
+        <v>46218</v>
       </c>
       <c r="B119" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C119" s="28" t="inlineStr">
         <is>
-          <t>Climatizzatore: come scelgo il modello giusto per casa mia?</t>
+          <t>Inserto a legna: ogni quanti anni va pulita la canna fumaria?</t>
         </is>
       </c>
       <c r="D119" s="28" t="inlineStr">
         <is>
-          <t>Non sa da dove partire nella scelta — marca, BTU, classe energetica gli sembrano tutti uguali</t>
+          <t>Non so se la mia canna fumaria è a rischio e chi dovrei chiamare</t>
         </is>
       </c>
       <c r="E119" s="28" t="inlineStr">
         <is>
-          <t>I 3 parametri pratici che fanno la differenza nella scelta di un climatizzatore, spiegati senza tecnicismi.</t>
+          <t>Spieghiamo la regola base sulla pulizia della canna fumaria (almeno una volta l'anno per uso regolare), cosa succede se non si fa, e chi interviene. Utile, pratico, senza allarmismi.</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Climatizzatore</t>
+          <t>Prodotto - Inserti e Camini</t>
         </is>
       </c>
       <c r="G119" s="9" t="inlineStr">
         <is>
-          <t>Come scegliere il modello giusto</t>
-        </is>
-      </c>
-      <c r="H119" s="28" t="n"/>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H119" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I119" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J119" s="15" t="inlineStr">
@@ -6631,42 +6635,46 @@
     </row>
     <row r="120" ht="60.75" customHeight="1" s="17">
       <c r="A120" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B120" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C120" s="28" t="inlineStr">
         <is>
-          <t>Conto Termico: copre anche la sostituzione del vecchio condizionatore?</t>
+          <t>Ecobonus 2026 per la pompa di calore: chi può richiederlo e cosa serve davvero</t>
         </is>
       </c>
       <c r="D120" s="28" t="inlineStr">
         <is>
-          <t>Pensa che il Conto Termico valga solo per caldaie e pompe di calore, non per i climatizzatori</t>
+          <t>Non so se ho diritto all'incentivo e ho paura di perdere soldi per ignoranza burocratica</t>
         </is>
       </c>
       <c r="E120" s="28" t="inlineStr">
         <is>
-          <t>Quando la rottamazione di un vecchio climatizzatore dà diritto al Conto Termico e come richiederlo.</t>
+          <t>Spieghiamo in modo semplice chi può accedere all'Ecobonus per la pompa di calore nel 2026, quali documenti servono e chi gestisce la pratica al posto tuo</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica / normativa</t>
-        </is>
-      </c>
-      <c r="H120" s="28" t="n"/>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H120" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I120" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J120" s="15" t="inlineStr">
@@ -6677,42 +6685,46 @@
     </row>
     <row r="121" ht="60.75" customHeight="1" s="17">
       <c r="A121" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B121" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C121" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: non devi rifare tutto l'impianto. E il fotovoltaico può aiutarti.</t>
+          <t>Termocamino a legna: riscalda solo il salotto o arriva calore anche nelle altre stanze?</t>
         </is>
       </c>
       <c r="D121" s="28" t="inlineStr">
         <is>
-          <t>Rinunciano alla PdC convinti serva un cantiere enorme — non sanno che si può partire in piccolo</t>
+          <t>Ho paura di installare un termocamino e scoprire che il calore resta tutto in un'unica stanza</t>
         </is>
       </c>
       <c r="E121" s="28" t="inlineStr">
         <is>
-          <t>Perché in molti casi basta un impianto più contenuto, e come il fotovoltaico aiuta a sostenere il consumo elettrico della PdC.</t>
+          <t>Mostriamo come un termocamino si collega all'impianto idraulico esistente e distribuisce calore nei radiatori di tutta la casa, non solo nel locale dove brucia il fuoco</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>Prodotto - Termocamini</t>
         </is>
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
-        </is>
-      </c>
-      <c r="H121" s="28" t="n"/>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H121" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I121" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J121" s="15" t="inlineStr">
@@ -6723,42 +6735,46 @@
     </row>
     <row r="122" ht="60.75" customHeight="1" s="17">
       <c r="A122" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C122" s="28" t="inlineStr">
         <is>
-          <t>Con cosa arriviamo a casa tua: i mezzi della squadra Solare Italiano</t>
+          <t>Detrazione fiscale o Conto Termico: qual è la differenza e quale spetta a te?</t>
         </is>
       </c>
       <c r="D122" s="28" t="inlineStr">
         <is>
-          <t>Non sa quanta preparazione professionale c'è dietro ogni intervento</t>
+          <t>Sento parlare di mille incentivi ma non capisco la differenza e rischio di scegliere quello sbagliato</t>
         </is>
       </c>
       <c r="E122" s="28" t="inlineStr">
         <is>
-          <t>Ripresa dei furgoni e della piattaforma aerea per mostrare l'attrezzatura sul campo. Nessuna improvvisazione.</t>
+          <t>Spieghiamo in linguaggio semplice quando si applica la detrazione IRPEF in dichiarazione dei redditi e quando invece si può richiedere il Conto Termico, con gli esempi pratici più comuni</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>Conosci Solare Italiano</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="H122" s="28" t="n"/>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H122" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I122" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J122" s="15" t="inlineStr">
@@ -6769,42 +6785,46 @@
     </row>
     <row r="123" ht="45.75" customHeight="1" s="17">
       <c r="A123" s="11" t="n">
-        <v>46148</v>
+        <v>46219</v>
       </c>
       <c r="B123" s="9" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Scheduled Task</t>
         </is>
       </c>
       <c r="C123" s="28" t="inlineStr">
         <is>
-          <t>Cosa facciamo prima di venire da te: la preparazione del furgone</t>
+          <t>Caldaia a pellet: l'errore più comune nella scelta della potenza (e come evitarlo)</t>
         </is>
       </c>
       <c r="D123" s="28" t="inlineStr">
         <is>
-          <t>Non immagina il lavoro di preparazione dietro ogni uscita — pensa che i tecnici partano senza organizzazione</t>
+          <t>Ho paura di acquistare una caldaia sbagliata per la mia casa e dover spendere di nuovo dopo poco</t>
         </is>
       </c>
       <c r="E123" s="28" t="inlineStr">
         <is>
-          <t>Il team che carica il furgone, controlla gli strumenti e prepara il materiale prima di partire. Dietro le quinte della professionalità.</t>
+          <t>Spieghiamo perché la potenza della caldaia a pellet deve essere calcolata sulla dispersione della casa e non sul prezzo o sulla marca, e cosa succede concretamente se si sbaglia la taglia</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>Lavori</t>
+          <t>Prodotto - Caldaie</t>
         </is>
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>Dietro le quinte squadra</t>
-        </is>
-      </c>
-      <c r="H123" s="28" t="n"/>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H123" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
       <c r="I123" s="14" t="inlineStr">
         <is>
-          <t>Produzione</t>
+          <t>Nuova</t>
         </is>
       </c>
       <c r="J123" s="15" t="inlineStr">
@@ -6815,7 +6835,7 @@
     </row>
     <row r="124" ht="45.75" customHeight="1" s="17">
       <c r="A124" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B124" s="9" t="inlineStr">
         <is>
@@ -6824,17 +6844,17 @@
       </c>
       <c r="C124" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore ibrida: tiene anche la caldaia? E perché non è un difetto</t>
+          <t>Pompa di calore: funziona anche quando fa molto freddo fuori?</t>
         </is>
       </c>
       <c r="D124" s="28" t="inlineStr">
         <is>
-          <t>Non capisco se la pompa di calore ibrida è peggio di una normale</t>
+          <t>Il cliente teme che la pompa di calore si blocchi nelle giornate più rigide dell'inverno</t>
         </is>
       </c>
       <c r="E124" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo cos'è la pompa di calore ibrida (PdC + caldaia nello stesso impianto), quando si usa l'una e quando l'altra, e perché in certe case è la scelta più intelligente — senza tecnicismi.</t>
+          <t>Sfatiamo il mito che le pompe di calore si fermino col gelo: spiega come funzionano anche sotto zero, quando serve davvero un'integrazione e perché il 'limite al freddo' è spesso sopravvalutato.</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
@@ -6865,7 +6885,7 @@
     </row>
     <row r="125" ht="45.75" customHeight="1" s="17">
       <c r="A125" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B125" s="9" t="inlineStr">
         <is>
@@ -6874,27 +6894,27 @@
       </c>
       <c r="C125" s="28" t="inlineStr">
         <is>
-          <t>Termostufa a legna: il calore arriva davvero in tutta la casa o rimane nel salotto?</t>
+          <t>Caldaia a pellet: dove si installa e quanto spazio serve davvero?</t>
         </is>
       </c>
       <c r="D125" s="28" t="inlineStr">
         <is>
-          <t>Ho paura che la termostufa scaldi solo dove c'è il fuoco</t>
+          <t>Il cliente non sa se ha lo spazio giusto o dove posizionare la caldaia in casa</t>
         </is>
       </c>
       <c r="E125" s="28" t="inlineStr">
         <is>
-          <t>Mostriamo la differenza tra una stufa normale e una termostufa: i radiatori distribuiscono il calore prodotto dal fuoco in tutti gli ambienti, anche ai piani superiori. Visivo e concreto.</t>
+          <t>Mostra i luoghi tipici di installazione (garage, lavanderia, locale tecnico) e spiega in modo semplice le distanze minime normative, rassicurando chi pensa di non avere abbastanza spazio.</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Termostufe</t>
+          <t>Prodotto - Caldaie</t>
         </is>
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Dove si può installare</t>
         </is>
       </c>
       <c r="H125" s="28" t="inlineStr">
@@ -6915,7 +6935,7 @@
     </row>
     <row r="126" ht="45.75" customHeight="1" s="17">
       <c r="A126" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B126" s="9" t="inlineStr">
         <is>
@@ -6924,17 +6944,17 @@
       </c>
       <c r="C126" s="28" t="inlineStr">
         <is>
-          <t>Incentivi 2026: li gestite voi o devo occuparmi io della burocrazia?</t>
+          <t>Bonus casa 2026: posso richiederlo anche se ho già fatto lavori negli anni scorsi?</t>
         </is>
       </c>
       <c r="D126" s="28" t="inlineStr">
         <is>
-          <t>Ho paura di dover fare da solo le domande per i bonus e sbagliare</t>
+          <t>Il cliente non sa se può ancora accedere agli incentivi dopo interventi precedenti</t>
         </is>
       </c>
       <c r="E126" s="28" t="inlineStr">
         <is>
-          <t>Risposta diretta e rassicurante: spieghiamo chi fa cosa, dal sopralluogo alla pratica incentivo. Obiettivo: togliere il timore burocratico che blocca la decisione di chiamarci.</t>
+          <t>Risponde alla domanda frequente su cumulo e accesso agli incentivi per chi ha già detratto in anni passati, con esempi pratici chiari per un proprietario di casa non tecnico.</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
@@ -6965,7 +6985,7 @@
     </row>
     <row r="127" ht="45.75" customHeight="1" s="17">
       <c r="A127" s="11" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="B127" s="9" t="inlineStr">
         <is>
@@ -6974,27 +6994,27 @@
       </c>
       <c r="C127" s="28" t="inlineStr">
         <is>
-          <t>Inserto a legna: ogni quanti anni va pulita la canna fumaria?</t>
+          <t>Cucina economica a legna: riscalda solo la cucina o può servire tutta la casa?</t>
         </is>
       </c>
       <c r="D127" s="28" t="inlineStr">
         <is>
-          <t>Non so se la mia canna fumaria è a rischio e chi dovrei chiamare</t>
+          <t>Il cliente non conosce la differenza tra cucina economica semplice e termocucina collegata all'impianto</t>
         </is>
       </c>
       <c r="E127" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo la regola base sulla pulizia della canna fumaria (almeno una volta l'anno per uso regolare), cosa succede se non si fa, e chi interviene. Utile, pratico, senza allarmismi.</t>
+          <t>Spiega la distinzione tra cucina economica standalone e termocucina con scambiatore idraulico, mostrando quando la seconda ha senso per distribuire il calore in più ambienti.</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Inserti e Camini</t>
+          <t>Prodotto - Cucine economiche</t>
         </is>
       </c>
       <c r="G127" s="9" t="inlineStr">
         <is>
-          <t>Manutenzione</t>
+          <t>Come funziona</t>
         </is>
       </c>
       <c r="H127" s="28" t="inlineStr">
@@ -7015,7 +7035,7 @@
     </row>
     <row r="128" ht="45.75" customHeight="1" s="17">
       <c r="A128" s="11" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="B128" s="9" t="inlineStr">
         <is>
@@ -7024,27 +7044,27 @@
       </c>
       <c r="C128" s="28" t="inlineStr">
         <is>
-          <t>Ecobonus 2026 per la pompa di calore: chi può richiederlo e cosa serve davvero</t>
+          <t>Climatizzatore e pompa di calore: non sono la stessa cosa — ecco perché</t>
         </is>
       </c>
       <c r="D128" s="28" t="inlineStr">
         <is>
-          <t>Non so se ho diritto all'incentivo e ho paura di perdere soldi per ignoranza burocratica</t>
+          <t>Il cliente confonde i due prodotti e non capisce quale scegliere per riscaldare casa in modo principale</t>
         </is>
       </c>
       <c r="E128" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo in modo semplice chi può accedere all'Ecobonus per la pompa di calore nel 2026, quali documenti servono e chi gestisce la pratica al posto tuo</t>
+          <t>Chiarisce la differenza spesso fraintesa tra un climatizzatore tradizionale e una pompa di calore ad alta efficienza per riscaldamento principale, guidando il cliente verso la scelta giusta per le sue esigenze.</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Pompe di Calore</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G128" s="9" t="inlineStr">
         <is>
-          <t>Incentivi</t>
+          <t>Confronto tra prodotti</t>
         </is>
       </c>
       <c r="H128" s="28" t="inlineStr">
@@ -7065,7 +7085,7 @@
     </row>
     <row r="129" ht="45.75" customHeight="1" s="17">
       <c r="A129" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B129" s="9" t="inlineStr">
         <is>
@@ -7074,27 +7094,27 @@
       </c>
       <c r="C129" s="28" t="inlineStr">
         <is>
-          <t>Termocamino a legna: riscalda solo il salotto o arriva calore anche nelle altre stanze?</t>
+          <t>Pompa di calore: il errore più comune è installarla senza isolare bene la casa</t>
         </is>
       </c>
       <c r="D129" s="28" t="inlineStr">
         <is>
-          <t>Ho paura di installare un termocamino e scoprire che il calore resta tutto in un'unica stanza</t>
+          <t>Ho sentito dire che la pompa di calore non scalda abbastanza d'inverno — eppure tutti la consigliano</t>
         </is>
       </c>
       <c r="E129" s="28" t="inlineStr">
         <is>
-          <t>Mostriamo come un termocamino si collega all'impianto idraulico esistente e distribuisce calore nei radiatori di tutta la casa, non solo nel locale dove brucia il fuoco</t>
+          <t>Molti utenti si lamentano del riscaldamento scarso, ma il problema spesso non è la pompa di calore in sé: è la dispersione termica dell'edificio. Il reel spiega perché l'isolamento fa la differenza e cosa chiedere prima dell'installazione.</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Termocamini</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G129" s="9" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Errore comune</t>
         </is>
       </c>
       <c r="H129" s="28" t="inlineStr">
@@ -7115,7 +7135,7 @@
     </row>
     <row r="130" ht="45.75" customHeight="1" s="17">
       <c r="A130" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B130" s="9" t="inlineStr">
         <is>
@@ -7124,27 +7144,27 @@
       </c>
       <c r="C130" s="28" t="inlineStr">
         <is>
-          <t>Detrazione fiscale o Conto Termico: qual è la differenza e quale spetta a te?</t>
+          <t>Termostufa a pellet: si può mettere in qualsiasi stanza o ci sono limiti?</t>
         </is>
       </c>
       <c r="D130" s="28" t="inlineStr">
         <is>
-          <t>Sento parlare di mille incentivi ma non capisco la differenza e rischio di scegliere quello sbagliato</t>
+          <t>Vorrei una termostufa a pellet ma non so se posso metterla dove voglio o se ci sono vincoli di legge</t>
         </is>
       </c>
       <c r="E130" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo in linguaggio semplice quando si applica la detrazione IRPEF in dichiarazione dei redditi e quando invece si può richiedere il Conto Termico, con gli esempi pratici più comuni</t>
+          <t>Non tutte le stanze sono adatte: servono scarico fumi, areazione e distanze minime dai materiali combustibili. Il reel guida il proprietario di casa nei criteri di scelta della posizione, in modo semplice e visivo.</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Termostufe</t>
         </is>
       </c>
       <c r="G130" s="9" t="inlineStr">
         <is>
-          <t>Domanda burocratica/normativa</t>
+          <t>Dove si può installare</t>
         </is>
       </c>
       <c r="H130" s="28" t="inlineStr">
@@ -7165,7 +7185,7 @@
     </row>
     <row r="131" ht="45.75" customHeight="1" s="17">
       <c r="A131" s="11" t="n">
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="B131" s="9" t="inlineStr">
         <is>
@@ -7174,27 +7194,27 @@
       </c>
       <c r="C131" s="28" t="inlineStr">
         <is>
-          <t>Caldaia a pellet: l'errore più comune nella scelta della potenza (e come evitarlo)</t>
+          <t>Conto Termico 2026: come funziona il rimborso e in quanto tempo arriva?</t>
         </is>
       </c>
       <c r="D131" s="28" t="inlineStr">
         <is>
-          <t>Ho paura di acquistare una caldaia sbagliata per la mia casa e dover spendere di nuovo dopo poco</t>
+          <t>Ho sentito parlare del Conto Termico ma non capisco quando e come mi arrivano i soldi</t>
         </is>
       </c>
       <c r="E131" s="28" t="inlineStr">
         <is>
-          <t>Spieghiamo perché la potenza della caldaia a pellet deve essere calcolata sulla dispersione della casa e non sul prezzo o sulla marca, e cosa succede concretamente se si sbaglia la taglia</t>
+          <t>Il Conto Termico è uno degli incentivi meno conosciuti ma più vantaggiosi per stufe, caldaie e pompe di calore. Il reel spiega in 3 passi: cos'è, chi può richiederlo, in quanto tempo arriva il rimborso — senza tecnicismi.</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>Prodotto - Caldaie</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G131" s="9" t="inlineStr">
         <is>
-          <t>Errore comune</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H131" s="28" t="inlineStr">
@@ -7215,7 +7235,7 @@
     </row>
     <row r="132" ht="45.75" customHeight="1" s="17">
       <c r="A132" s="11" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="B132" s="9" t="inlineStr">
         <is>
@@ -7224,448 +7244,416 @@
       </c>
       <c r="C132" s="28" t="inlineStr">
         <is>
-          <t>Pompa di calore: funziona anche quando fa molto freddo fuori?</t>
+          <t>Inserto a legna al posto del caminetto aperto: cosa cambia davvero in termini di calore e sicurezza</t>
         </is>
       </c>
       <c r="D132" s="28" t="inlineStr">
         <is>
-          <t>Il cliente teme che la pompa di calore si blocchi nelle giornate più rigide dell'inverno</t>
+          <t>Ho un caminetto aperto che scalda poco e fa fumo — ho sentito che l'inserto è meglio ma non so cosa aspettarmi</t>
         </is>
       </c>
       <c r="E132" s="28" t="inlineStr">
         <is>
-          <t>Sfatiamo il mito che le pompe di calore si fermino col gelo: spiega come funzionano anche sotto zero, quando serve davvero un'integrazione e perché il 'limite al freddo' è spesso sopravvalutato.</t>
+          <t>Il caminetto aperto disperde fino all'80% del calore. L'inserto a legna trasforma lo stesso vano in una fonte di calore efficiente, con vetro panoramico e meno rischi. Il reel mostra il confronto prima/dopo in modo visivo e immediato.</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>A cosa viene sostituito</t>
+        </is>
+      </c>
+      <c r="H132" s="28" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I132" s="14" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J132" s="15" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="45.75" customHeight="1" s="17">
+      <c r="A133" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B133" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C133" s="31" t="inlineStr">
+        <is>
+          <t>Vuoi cambiare la caldaia? Ecco perché il bonus che ti aspettavi non esiste più</t>
+        </is>
+      </c>
+      <c r="D133" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario vuole cambiare la vecchia caldaia a gas e dà per scontato di avere l'Ecobonus, poi scopre che le caldaie a gas sono ora escluse</t>
+        </is>
+      </c>
+      <c r="E133" s="31" t="inlineStr">
+        <is>
+          <t>Reel che chiarisce la svolta del 2026: le caldaie a gas non sono più coperte dall'Ecobonus. Spiega le alternative (pompa di calore, impianto ibrido, biomassa) che invece danno diritto a incentivi fino al 65% con il Conto Termico 3.0. Collegato a notizia Ecobonus luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F133" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G133" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H133" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I133" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J133" s="30" t="n"/>
+    </row>
+    <row r="134" ht="30.75" customHeight="1" s="17">
+      <c r="A134" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B134" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C134" s="31" t="inlineStr">
+        <is>
+          <t>Le classi energetiche sono cambiate a giugno 2026: cosa significa davvero per la tua casa?</t>
+        </is>
+      </c>
+      <c r="D134" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario ha sentito delle nuove classi energetiche e teme di dover fare lavori obbligatori o che la casa abbia perso valore</t>
+        </is>
+      </c>
+      <c r="E134" s="31" t="inlineStr">
+        <is>
+          <t>Reel che demistifica il nuovo APE entrato in vigore il 3 giugno 2026: nessun obbligo individuale sui privati, ma capire la classe della propria casa aiuta a scegliere i lavori giusti per risparmiare e valorizzare l'immobile. Soft CTA: valutazione energetica gratuita. Collegato a notizia Direttiva Case Green / nuovo APE luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F134" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G134" s="30" t="inlineStr">
+        <is>
+          <t>Paura</t>
+        </is>
+      </c>
+      <c r="H134" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I134" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J134" s="30" t="n"/>
+    </row>
+    <row r="135" ht="45.75" customHeight="1" s="17">
+      <c r="A135" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B135" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C135" s="31" t="inlineStr">
+        <is>
+          <t>Fotovoltaico e colonnina di ricarica insieme: l'agevolazione IVA che in pochi conoscono</t>
+        </is>
+      </c>
+      <c r="D135" s="31" t="inlineStr">
+        <is>
+          <t>Chi vuole installare il fotovoltaico e la colonnina non sa che farli insieme dà l'IVA al 10% sulla colonnina, mentre installarli separati costa il 22%</t>
+        </is>
+      </c>
+      <c r="E135" s="31" t="inlineStr">
+        <is>
+          <t>Reel pratico che spiega il vantaggio dell'installazione combinata fotovoltaico + colonnina di ricarica nello stesso cantiere: IVA al 10% invece del 22% ordinario. Posizionamento: Solare Italiano installa entrambi e conviene farlo in un unico intervento. Collegato a notizia incentivi fotovoltaico/colonnine 2026.</t>
+        </is>
+      </c>
+      <c r="F135" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G135" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H135" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I135" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J135" s="30" t="n"/>
+    </row>
+    <row r="136" ht="45.75" customHeight="1" s="17">
+      <c r="A136" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B136" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C136" s="31" t="inlineStr">
+        <is>
+          <t>Batteria di accumulo: a cosa serve davvero e quando conviene aggiungerla al fotovoltaico</t>
+        </is>
+      </c>
+      <c r="D136" s="31" t="inlineStr">
+        <is>
+          <t>Chi ha il fotovoltaico o sta per installarlo non capisce se la batteria di accumulo è davvero utile o solo un costo aggiuntivo</t>
+        </is>
+      </c>
+      <c r="E136" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega in modo semplice cos'è una batteria di accumulo: di notte usi l'energia che hai prodotto di giorno invece di prenderla dalla rete. Senza numeri, con la logica dell'autonomia energetica. Quando aggiungerla subito e quando aspettare. Collegato a notizia detrazione 50% batterie confermata 2026.</t>
+        </is>
+      </c>
+      <c r="F136" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G136" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H136" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I136" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J136" s="30" t="n"/>
+    </row>
+    <row r="137" ht="45.75" customHeight="1" s="17">
+      <c r="A137" s="29" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B137" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C137" s="31" t="inlineStr">
+        <is>
+          <t>Termocamino a pellet o a legna: qual è la differenza e come scegliere quello giusto per la tua casa?</t>
+        </is>
+      </c>
+      <c r="D137" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario vuole un termocamino ma non sa se preferire il modello a pellet o a legna — sembrano simili ma funzionano in modo molto diverso nella vita quotidiana</t>
+        </is>
+      </c>
+      <c r="E137" s="31" t="inlineStr">
+        <is>
+          <t>Confronto diretto termocamino a pellet vs a legna: autonomia, comodità d'uso, spazio necessario per lo stoccaggio del combustibile, adattabilità alla casa. Chiusura: la scelta dipende dal tuo stile di vita, non dalla tecnologia in sé. Solare Italiano installa entrambi.</t>
+        </is>
+      </c>
+      <c r="F137" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Termocamini</t>
+        </is>
+      </c>
+      <c r="G137" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H137" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I137" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J137" s="30" t="n"/>
+    </row>
+    <row r="138" ht="45.75" customHeight="1" s="17">
+      <c r="A138" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B138" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C138" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0 o Ecobonus: non puoi averli entrambi — qual è quello giusto per la tua pompa di calore?</t>
+        </is>
+      </c>
+      <c r="D138" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito parlare di vari bonus e non capisco quale scegliere: non voglio sbagliare e perdere soldi</t>
+        </is>
+      </c>
+      <c r="E138" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega in modo semplice la differenza pratica tra CT 3.0 (soldi subito, fondo perduto) ed Ecobonus (detrazione in 10 anni): quando conviene l'uno e quando l'altro. Ispirato da news: CT 3.0 e Ecobonus non sono cumulabili.</t>
+        </is>
+      </c>
+      <c r="F138" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G138" s="30" t="inlineStr">
+        <is>
+          <t>Confronto tra prodotti</t>
+        </is>
+      </c>
+      <c r="H138" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I138" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J138" s="30" t="n"/>
+    </row>
+    <row r="139" ht="45.75" customHeight="1" s="17">
+      <c r="A139" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B139" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C139" s="31" t="inlineStr">
+        <is>
+          <t>La tua casa è in classe F o G? Ecco cosa ti chiede davvero la Direttiva Case Green adesso (e cosa no)</t>
+        </is>
+      </c>
+      <c r="D139" s="31" t="inlineStr">
+        <is>
+          <t>Ho paura che l'Europa mi obblighi a fare lavori costosi subito — non so se devo fare qualcosa</t>
+        </is>
+      </c>
+      <c r="E139" s="31" t="inlineStr">
+        <is>
+          <t>Reel che chiarisce: la Direttiva Case Green è in vigore ma NON obbliga interventi immediati al singolo proprietario. Spiega cosa è già cambiato (scala APE, requisiti minimi giugno 2026) e cosa arriverà nel medio periodo per le classi basse. Ispirato da news: procedura infrazione UE, EPBD in vigore.</t>
+        </is>
+      </c>
+      <c r="F139" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G139" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H139" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I139" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J139" s="30" t="n"/>
+    </row>
+    <row r="140" ht="45.75" customHeight="1" s="17">
+      <c r="A140" s="29" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B140" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C140" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore affiancata alla caldaia: esiste davvero e funziona meglio di quanto pensi</t>
+        </is>
+      </c>
+      <c r="D140" s="31" t="inlineStr">
+        <is>
+          <t>Vorrei una pompa di calore ma ho già una caldaia che funziona e temo di dover buttare via tutto</t>
+        </is>
+      </c>
+      <c r="E140" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega il sistema bivalente (pompa di calore + caldaia esistente): come si integrano, chi fa cosa al variare della temperatura esterna, e che ora è ammesso anche dal Conto Termico 3.0. Risolve il blocco psicologico 'devo rifare tutto'.</t>
+        </is>
+      </c>
+      <c r="F140" s="30" t="inlineStr">
+        <is>
           <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
-      <c r="G132" s="9" t="inlineStr">
+      <c r="G140" s="30" t="inlineStr">
         <is>
           <t>Come funziona</t>
         </is>
       </c>
-      <c r="H132" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I132" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J132" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="45.75" customHeight="1" s="17">
-      <c r="A133" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B133" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C133" s="28" t="inlineStr">
-        <is>
-          <t>Caldaia a pellet: dove si installa e quanto spazio serve davvero?</t>
-        </is>
-      </c>
-      <c r="D133" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente non sa se ha lo spazio giusto o dove posizionare la caldaia in casa</t>
-        </is>
-      </c>
-      <c r="E133" s="28" t="inlineStr">
-        <is>
-          <t>Mostra i luoghi tipici di installazione (garage, lavanderia, locale tecnico) e spiega in modo semplice le distanze minime normative, rassicurando chi pensa di non avere abbastanza spazio.</t>
-        </is>
-      </c>
-      <c r="F133" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Caldaie</t>
-        </is>
-      </c>
-      <c r="G133" s="9" t="inlineStr">
-        <is>
-          <t>Dove si può installare</t>
-        </is>
-      </c>
-      <c r="H133" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I133" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J133" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="30.75" customHeight="1" s="17">
-      <c r="A134" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B134" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C134" s="28" t="inlineStr">
-        <is>
-          <t>Bonus casa 2026: posso richiederlo anche se ho già fatto lavori negli anni scorsi?</t>
-        </is>
-      </c>
-      <c r="D134" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente non sa se può ancora accedere agli incentivi dopo interventi precedenti</t>
-        </is>
-      </c>
-      <c r="E134" s="28" t="inlineStr">
-        <is>
-          <t>Risponde alla domanda frequente su cumulo e accesso agli incentivi per chi ha già detratto in anni passati, con esempi pratici chiari per un proprietario di casa non tecnico.</t>
-        </is>
-      </c>
-      <c r="F134" s="9" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G134" s="9" t="inlineStr">
-        <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H134" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I134" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J134" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="45.75" customHeight="1" s="17">
-      <c r="A135" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B135" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C135" s="28" t="inlineStr">
-        <is>
-          <t>Cucina economica a legna: riscalda solo la cucina o può servire tutta la casa?</t>
-        </is>
-      </c>
-      <c r="D135" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente non conosce la differenza tra cucina economica semplice e termocucina collegata all'impianto</t>
-        </is>
-      </c>
-      <c r="E135" s="28" t="inlineStr">
-        <is>
-          <t>Spiega la distinzione tra cucina economica standalone e termocucina con scambiatore idraulico, mostrando quando la seconda ha senso per distribuire il calore in più ambienti.</t>
-        </is>
-      </c>
-      <c r="F135" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Cucine economiche</t>
-        </is>
-      </c>
-      <c r="G135" s="9" t="inlineStr">
-        <is>
-          <t>Come funziona</t>
-        </is>
-      </c>
-      <c r="H135" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I135" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J135" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="136" ht="45.75" customHeight="1" s="17">
-      <c r="A136" s="11" t="n">
-        <v>46220</v>
-      </c>
-      <c r="B136" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C136" s="28" t="inlineStr">
-        <is>
-          <t>Climatizzatore e pompa di calore: non sono la stessa cosa — ecco perché</t>
-        </is>
-      </c>
-      <c r="D136" s="28" t="inlineStr">
-        <is>
-          <t>Il cliente confonde i due prodotti e non capisce quale scegliere per riscaldare casa in modo principale</t>
-        </is>
-      </c>
-      <c r="E136" s="28" t="inlineStr">
-        <is>
-          <t>Chiarisce la differenza spesso fraintesa tra un climatizzatore tradizionale e una pompa di calore ad alta efficienza per riscaldamento principale, guidando il cliente verso la scelta giusta per le sue esigenze.</t>
-        </is>
-      </c>
-      <c r="F136" s="9" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G136" s="9" t="inlineStr">
-        <is>
-          <t>Confronto tra prodotti</t>
-        </is>
-      </c>
-      <c r="H136" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I136" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J136" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="45.75" customHeight="1" s="17">
-      <c r="A137" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B137" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C137" s="28" t="inlineStr">
-        <is>
-          <t>Pompa di calore: il errore più comune è installarla senza isolare bene la casa</t>
-        </is>
-      </c>
-      <c r="D137" s="28" t="inlineStr">
-        <is>
-          <t>Ho sentito dire che la pompa di calore non scalda abbastanza d'inverno — eppure tutti la consigliano</t>
-        </is>
-      </c>
-      <c r="E137" s="28" t="inlineStr">
-        <is>
-          <t>Molti utenti si lamentano del riscaldamento scarso, ma il problema spesso non è la pompa di calore in sé: è la dispersione termica dell'edificio. Il reel spiega perché l'isolamento fa la differenza e cosa chiedere prima dell'installazione.</t>
-        </is>
-      </c>
-      <c r="F137" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Pompe di Calore</t>
-        </is>
-      </c>
-      <c r="G137" s="9" t="inlineStr">
-        <is>
-          <t>Errore comune</t>
-        </is>
-      </c>
-      <c r="H137" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I137" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J137" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="45.75" customHeight="1" s="17">
-      <c r="A138" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B138" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C138" s="28" t="inlineStr">
-        <is>
-          <t>Termostufa a pellet: si può mettere in qualsiasi stanza o ci sono limiti?</t>
-        </is>
-      </c>
-      <c r="D138" s="28" t="inlineStr">
-        <is>
-          <t>Vorrei una termostufa a pellet ma non so se posso metterla dove voglio o se ci sono vincoli di legge</t>
-        </is>
-      </c>
-      <c r="E138" s="28" t="inlineStr">
-        <is>
-          <t>Non tutte le stanze sono adatte: servono scarico fumi, areazione e distanze minime dai materiali combustibili. Il reel guida il proprietario di casa nei criteri di scelta della posizione, in modo semplice e visivo.</t>
-        </is>
-      </c>
-      <c r="F138" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Termostufe</t>
-        </is>
-      </c>
-      <c r="G138" s="9" t="inlineStr">
-        <is>
-          <t>Dove si può installare</t>
-        </is>
-      </c>
-      <c r="H138" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I138" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J138" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="45.75" customHeight="1" s="17">
-      <c r="A139" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B139" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C139" s="28" t="inlineStr">
-        <is>
-          <t>Conto Termico 2026: come funziona il rimborso e in quanto tempo arriva?</t>
-        </is>
-      </c>
-      <c r="D139" s="28" t="inlineStr">
-        <is>
-          <t>Ho sentito parlare del Conto Termico ma non capisco quando e come mi arrivano i soldi</t>
-        </is>
-      </c>
-      <c r="E139" s="28" t="inlineStr">
-        <is>
-          <t>Il Conto Termico è uno degli incentivi meno conosciuti ma più vantaggiosi per stufe, caldaie e pompe di calore. Il reel spiega in 3 passi: cos'è, chi può richiederlo, in quanto tempo arriva il rimborso — senza tecnicismi.</t>
-        </is>
-      </c>
-      <c r="F139" s="9" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G139" s="9" t="inlineStr">
-        <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H139" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I139" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J139" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="45.75" customHeight="1" s="17">
-      <c r="A140" s="11" t="n">
-        <v>46221</v>
-      </c>
-      <c r="B140" s="9" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C140" s="28" t="inlineStr">
-        <is>
-          <t>Inserto a legna al posto del caminetto aperto: cosa cambia davvero in termini di calore e sicurezza</t>
-        </is>
-      </c>
-      <c r="D140" s="28" t="inlineStr">
-        <is>
-          <t>Ho un caminetto aperto che scalda poco e fa fumo — ho sentito che l'inserto è meglio ma non so cosa aspettarmi</t>
-        </is>
-      </c>
-      <c r="E140" s="28" t="inlineStr">
-        <is>
-          <t>Il caminetto aperto disperde fino all'80% del calore. L'inserto a legna trasforma lo stesso vano in una fonte di calore efficiente, con vetro panoramico e meno rischi. Il reel mostra il confronto prima/dopo in modo visivo e immediato.</t>
-        </is>
-      </c>
-      <c r="F140" s="9" t="inlineStr">
-        <is>
-          <t>Prodotto - Inserti e Camini</t>
-        </is>
-      </c>
-      <c r="G140" s="9" t="inlineStr">
-        <is>
-          <t>A cosa viene sostituito</t>
-        </is>
-      </c>
-      <c r="H140" s="28" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte</t>
-        </is>
-      </c>
-      <c r="I140" s="14" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J140" s="15" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
+      <c r="H140" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I140" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J140" s="30" t="n"/>
     </row>
     <row r="141" ht="45.75" customHeight="1" s="17">
       <c r="A141" s="29" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B141" s="30" t="inlineStr">
         <is>
@@ -7674,27 +7662,27 @@
       </c>
       <c r="C141" s="31" t="inlineStr">
         <is>
-          <t>Vuoi cambiare la caldaia? Ecco perché il bonus che ti aspettavi non esiste più</t>
+          <t>Detrazioni al 50%: il 31 dicembre 2026 non è solo una scadenza — è un bivio che non puoi ignorare</t>
         </is>
       </c>
       <c r="D141" s="31" t="inlineStr">
         <is>
-          <t>Il proprietario vuole cambiare la vecchia caldaia a gas e dà per scontato di avere l'Ecobonus, poi scopre che le caldaie a gas sono ora escluse</t>
+          <t>Non so se fare i lavori adesso o aspettare — ho paura di sbagliare i tempi</t>
         </is>
       </c>
       <c r="E141" s="31" t="inlineStr">
         <is>
-          <t>Reel che chiarisce la svolta del 2026: le caldaie a gas non sono più coperte dall'Ecobonus. Spiega le alternative (pompa di calore, impianto ibrido, biomassa) che invece danno diritto a incentivi fino al 65% con il Conto Termico 3.0. Collegato a notizia Ecobonus luglio 2026.</t>
+          <t>Reel che spiega con chiarezza: bonus edilizi confermati al 50% prima casa solo fino al 31/12/2026, dal 2027 scendono al 36%. Nessun calcolo di risparmio, solo il meccanismo normativo e la domanda semplice: 'I lavori li vuoi fare entro fine anno o aspetti?'. Ispirato da news: Bonus edilizi 2026 ultima finestra.</t>
         </is>
       </c>
       <c r="F141" s="30" t="inlineStr">
         <is>
-          <t>Prodotto - Caldaie</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G141" s="30" t="inlineStr">
         <is>
-          <t>Incentivi</t>
+          <t>Domanda economica</t>
         </is>
       </c>
       <c r="H141" s="31" t="inlineStr">
@@ -7711,7 +7699,7 @@
     </row>
     <row r="142" ht="45.75" customHeight="1" s="17">
       <c r="A142" s="29" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B142" s="30" t="inlineStr">
         <is>
@@ -7720,27 +7708,27 @@
       </c>
       <c r="C142" s="31" t="inlineStr">
         <is>
-          <t>Le classi energetiche sono cambiate a giugno 2026: cosa significa davvero per la tua casa?</t>
+          <t>Climatizzatore che fatica a raffreddare: lo ripari ancora o è il momento di cambiarlo?</t>
         </is>
       </c>
       <c r="D142" s="31" t="inlineStr">
         <is>
-          <t>Il proprietario ha sentito delle nuove classi energetiche e teme di dover fare lavori obbligatori o che la casa abbia perso valore</t>
+          <t>Il mio climatizzatore non funziona più bene — non so se spendere per ripararlo o comprarne uno nuovo</t>
         </is>
       </c>
       <c r="E142" s="31" t="inlineStr">
         <is>
-          <t>Reel che demistifica il nuovo APE entrato in vigore il 3 giugno 2026: nessun obbligo individuale sui privati, ma capire la classe della propria casa aiuta a scegliere i lavori giusti per risparmiare e valorizzare l'immobile. Soft CTA: valutazione energetica gratuita. Collegato a notizia Direttiva Case Green / nuovo APE luglio 2026.</t>
+          <t>Reel evergreen perfetto per luglio: segnali chiari che indicano quando ha senso riparare (guasto isolato, impianto giovane) vs quando conviene sostituire (più di 10-12 anni, gas fuori produzione, consumi alti). Nessuna cifra, solo criteri pratici da capire al volo.</t>
         </is>
       </c>
       <c r="F142" s="30" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Climatizzatore</t>
         </is>
       </c>
       <c r="G142" s="30" t="inlineStr">
         <is>
-          <t>Paura</t>
+          <t>Quando sostituirlo</t>
         </is>
       </c>
       <c r="H142" s="31" t="inlineStr">
@@ -7757,7 +7745,7 @@
     </row>
     <row r="143" ht="30.75" customHeight="1" s="17">
       <c r="A143" s="29" t="n">
-        <v>46223</v>
+        <v>46228</v>
       </c>
       <c r="B143" s="30" t="inlineStr">
         <is>
@@ -7766,27 +7754,27 @@
       </c>
       <c r="C143" s="31" t="inlineStr">
         <is>
-          <t>Fotovoltaico e colonnina di ricarica insieme: l'agevolazione IVA che in pochi conoscono</t>
+          <t>L'Europa ha aperto una procedura d'infrazione sull'Italia per la Direttiva Case Green: cosa cambia davvero per chi ha una casa?</t>
         </is>
       </c>
       <c r="D143" s="31" t="inlineStr">
         <is>
-          <t>Chi vuole installare il fotovoltaico e la colonnina non sa che farli insieme dà l'IVA al 10% sulla colonnina, mentre installarli separati costa il 22%</t>
+          <t>Paura di obbligo immediato di ristrutturare dopo la notizia dell'infrazione UE</t>
         </is>
       </c>
       <c r="E143" s="31" t="inlineStr">
         <is>
-          <t>Reel pratico che spiega il vantaggio dell'installazione combinata fotovoltaico + colonnina di ricarica nello stesso cantiere: IVA al 10% invece del 22% ordinario. Posizionamento: Solare Italiano installa entrambi e conviene farlo in un unico intervento. Collegato a notizia incentivi fotovoltaico/colonnine 2026.</t>
+          <t>Il reel spiega che la procedura d'infrazione riguarda lo Stato italiano, non il singolo proprietario. Nessun obbligo immediato di ristrutturare. Significa però che il recepimento della direttiva accelererà e i requisiti minimi arriveranno. Meglio conoscere già la classe energetica della propria casa e sapere che esistono incentivi attivi oggi.</t>
         </is>
       </c>
       <c r="F143" s="30" t="inlineStr">
         <is>
-          <t>Prodotto - Colonnine di Ricarica</t>
+          <t>FAQ</t>
         </is>
       </c>
       <c r="G143" s="30" t="inlineStr">
         <is>
-          <t>Incentivi</t>
+          <t>Domanda burocratica/normativa</t>
         </is>
       </c>
       <c r="H143" s="31" t="inlineStr">
@@ -7803,7 +7791,7 @@
     </row>
     <row r="144" ht="45.75" customHeight="1" s="17">
       <c r="A144" s="29" t="n">
-        <v>46223</v>
+        <v>46228</v>
       </c>
       <c r="B144" s="30" t="inlineStr">
         <is>
@@ -7812,27 +7800,27 @@
       </c>
       <c r="C144" s="31" t="inlineStr">
         <is>
-          <t>Batteria di accumulo: a cosa serve davvero e quando conviene aggiungerla al fotovoltaico</t>
+          <t>Il portale Conto Termico 3.0 era bloccato a marzo — ma ha riaperto: puoi ancora fare domanda per la pompa di calore</t>
         </is>
       </c>
       <c r="D144" s="31" t="inlineStr">
         <is>
-          <t>Chi ha il fotovoltaico o sta per installarlo non capisce se la batteria di accumulo è davvero utile o solo un costo aggiuntivo</t>
+          <t>Non sa che dopo il blocco del portale si può ancora accedere all'incentivo CT3.0</t>
         </is>
       </c>
       <c r="E144" s="31" t="inlineStr">
         <is>
-          <t>Reel che spiega in modo semplice cos'è una batteria di accumulo: di notte usi l'energia che hai prodotto di giorno invece di prenderla dalla rete. Senza numeri, con la logica dell'autonomia energetica. Quando aggiungerla subito e quando aspettare. Collegato a notizia detrazione 50% batterie confermata 2026.</t>
+          <t>Il reel racconta cosa è successo: il portale GSE ha aperto a febbraio, poi si è bloccato a marzo per eccesso di domande, ed è riaperto ad aprile con proroga dei termini. Chi vuole installare una pompa di calore può ancora presentare domanda nel 2026. Spiega i tre passi essenziali: preventivo tecnico, tecnico abilitato, IBAN per il rimborso diretto.</t>
         </is>
       </c>
       <c r="F144" s="30" t="inlineStr">
         <is>
-          <t>Prodotto - Batterie di Accumulo</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G144" s="30" t="inlineStr">
         <is>
-          <t>Come funziona</t>
+          <t>Incentivi</t>
         </is>
       </c>
       <c r="H144" s="31" t="inlineStr">
@@ -7849,7 +7837,7 @@
     </row>
     <row r="145" ht="45.75" customHeight="1" s="17">
       <c r="A145" s="29" t="n">
-        <v>46223</v>
+        <v>46228</v>
       </c>
       <c r="B145" s="30" t="inlineStr">
         <is>
@@ -7858,27 +7846,27 @@
       </c>
       <c r="C145" s="31" t="inlineStr">
         <is>
-          <t>Termocamino a pellet o a legna: qual è la differenza e come scegliere quello giusto per la tua casa?</t>
+          <t>Pompa di calore: in tanti pensano serva solo per riscaldare — ma fa anche il lavoro del climatizzatore. Ecco come funziona</t>
         </is>
       </c>
       <c r="D145" s="31" t="inlineStr">
         <is>
-          <t>Il proprietario vuole un termocamino ma non sa se preferire il modello a pellet o a legna — sembrano simili ma funzionano in modo molto diverso nella vita quotidiana</t>
+          <t>Ha caldaia e climatizzatore separati e non sa che potrebbe avere un unico sistema</t>
         </is>
       </c>
       <c r="E145" s="31" t="inlineStr">
         <is>
-          <t>Confronto diretto termocamino a pellet vs a legna: autonomia, comodità d'uso, spazio necessario per lo stoccaggio del combustibile, adattabilità alla casa. Chiusura: la scelta dipende dal tuo stile di vita, non dalla tecnologia in sé. Solare Italiano installa entrambi.</t>
+          <t>Il reel spiega la doppia funzione della pompa di calore: riscalda d'inverno, raffredda d'estate. È un sostituto sia della caldaia che del climatizzatore. Un solo impianto, meno manutenzione, meno spazio. Con gli incentivi 2026 (CT3.0 o Ecobonus) il momento è favorevole.</t>
         </is>
       </c>
       <c r="F145" s="30" t="inlineStr">
         <is>
-          <t>Prodotto - Termocamini</t>
+          <t>Prodotto - Pompe di Calore</t>
         </is>
       </c>
       <c r="G145" s="30" t="inlineStr">
         <is>
-          <t>Confronto con alternative</t>
+          <t>A cosa viene sostituito</t>
         </is>
       </c>
       <c r="H145" s="31" t="inlineStr">
@@ -7895,7 +7883,7 @@
     </row>
     <row r="146" ht="60.75" customHeight="1" s="17">
       <c r="A146" s="29" t="n">
-        <v>46224</v>
+        <v>46228</v>
       </c>
       <c r="B146" s="30" t="inlineStr">
         <is>
@@ -7904,27 +7892,27 @@
       </c>
       <c r="C146" s="31" t="inlineStr">
         <is>
-          <t>Conto Termico 3.0 o Ecobonus: non puoi averli entrambi — qual è quello giusto per la tua pompa di calore?</t>
+          <t>Caldaia nuova nel 2026 o nel 2027? C'è una differenza che vale — e non è il prezzo della caldaia</t>
         </is>
       </c>
       <c r="D146" s="31" t="inlineStr">
         <is>
-          <t>Ho sentito parlare di vari bonus e non capisco quale scegliere: non voglio sbagliare e perdere soldi</t>
+          <t>Non sa che la detrazione per la sostituzione della caldaia scende dal 50% al 36% a gennaio 2027</t>
         </is>
       </c>
       <c r="E146" s="31" t="inlineStr">
         <is>
-          <t>Reel che spiega in modo semplice la differenza pratica tra CT 3.0 (soldi subito, fondo perduto) ed Ecobonus (detrazione in 10 anni): quando conviene l'uno e quando l'altro. Ispirato da news: CT 3.0 e Ecobonus non sono cumulabili.</t>
+          <t>Il reel spiega in modo semplice: chi sostituisce la caldaia entro il 31 dicembre 2026 ha la detrazione al 50% (prima casa). Dal 1° gennaio 2027 scende al 36%. Non è un invito a decidere in fretta — è un'informazione che molti non hanno e che può influenzare la pianificazione dei lavori.</t>
         </is>
       </c>
       <c r="F146" s="30" t="inlineStr">
         <is>
-          <t>FAQ</t>
+          <t>Prodotto - Caldaie</t>
         </is>
       </c>
       <c r="G146" s="30" t="inlineStr">
         <is>
-          <t>Confronto tra prodotti</t>
+          <t>Incentivi</t>
         </is>
       </c>
       <c r="H146" s="31" t="inlineStr">
@@ -7939,374 +7927,14 @@
       </c>
       <c r="J146" s="30" t="n"/>
     </row>
-    <row r="147" ht="60.75" customHeight="1" s="17">
-      <c r="A147" s="29" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B147" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C147" s="31" t="inlineStr">
-        <is>
-          <t>La tua casa è in classe F o G? Ecco cosa ti chiede davvero la Direttiva Case Green adesso (e cosa no)</t>
-        </is>
-      </c>
-      <c r="D147" s="31" t="inlineStr">
-        <is>
-          <t>Ho paura che l'Europa mi obblighi a fare lavori costosi subito — non so se devo fare qualcosa</t>
-        </is>
-      </c>
-      <c r="E147" s="31" t="inlineStr">
-        <is>
-          <t>Reel che chiarisce: la Direttiva Case Green è in vigore ma NON obbliga interventi immediati al singolo proprietario. Spiega cosa è già cambiato (scala APE, requisiti minimi giugno 2026) e cosa arriverà nel medio periodo per le classi basse. Ispirato da news: procedura infrazione UE, EPBD in vigore.</t>
-        </is>
-      </c>
-      <c r="F147" s="30" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G147" s="30" t="inlineStr">
-        <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H147" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I147" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J147" s="30" t="n"/>
-    </row>
-    <row r="148" ht="45.75" customHeight="1" s="17">
-      <c r="A148" s="29" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B148" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C148" s="31" t="inlineStr">
-        <is>
-          <t>Pompa di calore affiancata alla caldaia: esiste davvero e funziona meglio di quanto pensi</t>
-        </is>
-      </c>
-      <c r="D148" s="31" t="inlineStr">
-        <is>
-          <t>Vorrei una pompa di calore ma ho già una caldaia che funziona e temo di dover buttare via tutto</t>
-        </is>
-      </c>
-      <c r="E148" s="31" t="inlineStr">
-        <is>
-          <t>Reel che spiega il sistema bivalente (pompa di calore + caldaia esistente): come si integrano, chi fa cosa al variare della temperatura esterna, e che ora è ammesso anche dal Conto Termico 3.0. Risolve il blocco psicologico 'devo rifare tutto'.</t>
-        </is>
-      </c>
-      <c r="F148" s="30" t="inlineStr">
-        <is>
-          <t>Prodotto - Pompe di Calore</t>
-        </is>
-      </c>
-      <c r="G148" s="30" t="inlineStr">
-        <is>
-          <t>Come funziona</t>
-        </is>
-      </c>
-      <c r="H148" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I148" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J148" s="30" t="n"/>
-    </row>
-    <row r="149" ht="45.75" customHeight="1" s="17">
-      <c r="A149" s="29" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B149" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C149" s="31" t="inlineStr">
-        <is>
-          <t>Detrazioni al 50%: il 31 dicembre 2026 non è solo una scadenza — è un bivio che non puoi ignorare</t>
-        </is>
-      </c>
-      <c r="D149" s="31" t="inlineStr">
-        <is>
-          <t>Non so se fare i lavori adesso o aspettare — ho paura di sbagliare i tempi</t>
-        </is>
-      </c>
-      <c r="E149" s="31" t="inlineStr">
-        <is>
-          <t>Reel che spiega con chiarezza: bonus edilizi confermati al 50% prima casa solo fino al 31/12/2026, dal 2027 scendono al 36%. Nessun calcolo di risparmio, solo il meccanismo normativo e la domanda semplice: 'I lavori li vuoi fare entro fine anno o aspetti?'. Ispirato da news: Bonus edilizi 2026 ultima finestra.</t>
-        </is>
-      </c>
-      <c r="F149" s="30" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G149" s="30" t="inlineStr">
-        <is>
-          <t>Domanda economica</t>
-        </is>
-      </c>
-      <c r="H149" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I149" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J149" s="30" t="n"/>
-    </row>
-    <row r="150" ht="60.75" customHeight="1" s="17">
-      <c r="A150" s="29" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B150" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C150" s="31" t="inlineStr">
-        <is>
-          <t>Climatizzatore che fatica a raffreddare: lo ripari ancora o è il momento di cambiarlo?</t>
-        </is>
-      </c>
-      <c r="D150" s="31" t="inlineStr">
-        <is>
-          <t>Il mio climatizzatore non funziona più bene — non so se spendere per ripararlo o comprarne uno nuovo</t>
-        </is>
-      </c>
-      <c r="E150" s="31" t="inlineStr">
-        <is>
-          <t>Reel evergreen perfetto per luglio: segnali chiari che indicano quando ha senso riparare (guasto isolato, impianto giovane) vs quando conviene sostituire (più di 10-12 anni, gas fuori produzione, consumi alti). Nessuna cifra, solo criteri pratici da capire al volo.</t>
-        </is>
-      </c>
-      <c r="F150" s="30" t="inlineStr">
-        <is>
-          <t>Prodotto - Climatizzatore</t>
-        </is>
-      </c>
-      <c r="G150" s="30" t="inlineStr">
-        <is>
-          <t>Quando sostituirlo</t>
-        </is>
-      </c>
-      <c r="H150" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I150" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J150" s="30" t="n"/>
-    </row>
-    <row r="151" ht="45.75" customHeight="1" s="17">
-      <c r="A151" s="29" t="n">
-        <v>46228</v>
-      </c>
-      <c r="B151" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C151" s="31" t="inlineStr">
-        <is>
-          <t>L'Europa ha aperto una procedura d'infrazione sull'Italia per la Direttiva Case Green: cosa cambia davvero per chi ha una casa?</t>
-        </is>
-      </c>
-      <c r="D151" s="31" t="inlineStr">
-        <is>
-          <t>Paura di obbligo immediato di ristrutturare dopo la notizia dell'infrazione UE</t>
-        </is>
-      </c>
-      <c r="E151" s="31" t="inlineStr">
-        <is>
-          <t>Il reel spiega che la procedura d'infrazione riguarda lo Stato italiano, non il singolo proprietario. Nessun obbligo immediato di ristrutturare. Significa però che il recepimento della direttiva accelererà e i requisiti minimi arriveranno. Meglio conoscere già la classe energetica della propria casa e sapere che esistono incentivi attivi oggi.</t>
-        </is>
-      </c>
-      <c r="F151" s="30" t="inlineStr">
-        <is>
-          <t>FAQ</t>
-        </is>
-      </c>
-      <c r="G151" s="30" t="inlineStr">
-        <is>
-          <t>Domanda burocratica/normativa</t>
-        </is>
-      </c>
-      <c r="H151" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I151" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J151" s="30" t="n"/>
-    </row>
-    <row r="152" ht="45.75" customHeight="1" s="17">
-      <c r="A152" s="29" t="n">
-        <v>46228</v>
-      </c>
-      <c r="B152" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C152" s="31" t="inlineStr">
-        <is>
-          <t>Il portale Conto Termico 3.0 era bloccato a marzo — ma ha riaperto: puoi ancora fare domanda per la pompa di calore</t>
-        </is>
-      </c>
-      <c r="D152" s="31" t="inlineStr">
-        <is>
-          <t>Non sa che dopo il blocco del portale si può ancora accedere all'incentivo CT3.0</t>
-        </is>
-      </c>
-      <c r="E152" s="31" t="inlineStr">
-        <is>
-          <t>Il reel racconta cosa è successo: il portale GSE ha aperto a febbraio, poi si è bloccato a marzo per eccesso di domande, ed è riaperto ad aprile con proroga dei termini. Chi vuole installare una pompa di calore può ancora presentare domanda nel 2026. Spiega i tre passi essenziali: preventivo tecnico, tecnico abilitato, IBAN per il rimborso diretto.</t>
-        </is>
-      </c>
-      <c r="F152" s="30" t="inlineStr">
-        <is>
-          <t>Prodotto - Pompe di Calore</t>
-        </is>
-      </c>
-      <c r="G152" s="30" t="inlineStr">
-        <is>
-          <t>Incentivi</t>
-        </is>
-      </c>
-      <c r="H152" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I152" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J152" s="30" t="n"/>
-    </row>
-    <row r="153" ht="60.75" customHeight="1" s="17">
-      <c r="A153" s="29" t="n">
-        <v>46228</v>
-      </c>
-      <c r="B153" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C153" s="31" t="inlineStr">
-        <is>
-          <t>Pompa di calore: in tanti pensano serva solo per riscaldare — ma fa anche il lavoro del climatizzatore. Ecco come funziona</t>
-        </is>
-      </c>
-      <c r="D153" s="31" t="inlineStr">
-        <is>
-          <t>Ha caldaia e climatizzatore separati e non sa che potrebbe avere un unico sistema</t>
-        </is>
-      </c>
-      <c r="E153" s="31" t="inlineStr">
-        <is>
-          <t>Il reel spiega la doppia funzione della pompa di calore: riscalda d'inverno, raffredda d'estate. È un sostituto sia della caldaia che del climatizzatore. Un solo impianto, meno manutenzione, meno spazio. Con gli incentivi 2026 (CT3.0 o Ecobonus) il momento è favorevole.</t>
-        </is>
-      </c>
-      <c r="F153" s="30" t="inlineStr">
-        <is>
-          <t>Prodotto - Pompe di Calore</t>
-        </is>
-      </c>
-      <c r="G153" s="30" t="inlineStr">
-        <is>
-          <t>A cosa viene sostituito</t>
-        </is>
-      </c>
-      <c r="H153" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I153" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J153" s="30" t="n"/>
-    </row>
-    <row r="154" ht="60.75" customHeight="1" s="17">
-      <c r="A154" s="29" t="n">
-        <v>46228</v>
-      </c>
-      <c r="B154" s="30" t="inlineStr">
-        <is>
-          <t>Scheduled Task</t>
-        </is>
-      </c>
-      <c r="C154" s="31" t="inlineStr">
-        <is>
-          <t>Caldaia nuova nel 2026 o nel 2027? C'è una differenza che vale — e non è il prezzo della caldaia</t>
-        </is>
-      </c>
-      <c r="D154" s="31" t="inlineStr">
-        <is>
-          <t>Non sa che la detrazione per la sostituzione della caldaia scende dal 50% al 36% a gennaio 2027</t>
-        </is>
-      </c>
-      <c r="E154" s="31" t="inlineStr">
-        <is>
-          <t>Il reel spiega in modo semplice: chi sostituisce la caldaia entro il 31 dicembre 2026 ha la detrazione al 50% (prima casa). Dal 1° gennaio 2027 scende al 36%. Non è un invito a decidere in fretta — è un'informazione che molti non hanno e che può influenzare la pianificazione dei lavori.</t>
-        </is>
-      </c>
-      <c r="F154" s="30" t="inlineStr">
-        <is>
-          <t>Prodotto - Caldaie</t>
-        </is>
-      </c>
-      <c r="G154" s="30" t="inlineStr">
-        <is>
-          <t>Incentivi</t>
-        </is>
-      </c>
-      <c r="H154" s="31" t="inlineStr">
-        <is>
-          <t>Generato automaticamente di notte (news-informed)</t>
-        </is>
-      </c>
-      <c r="I154" s="30" t="inlineStr">
-        <is>
-          <t>Nuova</t>
-        </is>
-      </c>
-      <c r="J154" s="30" t="n"/>
-    </row>
+    <row r="147" ht="60.75" customHeight="1" s="17"/>
+    <row r="148" ht="45.75" customHeight="1" s="17"/>
+    <row r="149" ht="45.75" customHeight="1" s="17"/>
+    <row r="150" ht="60.75" customHeight="1" s="17"/>
+    <row r="151" ht="45.75" customHeight="1" s="17"/>
+    <row r="152" ht="45.75" customHeight="1" s="17"/>
+    <row r="153" ht="60.75" customHeight="1" s="17"/>
+    <row r="154" ht="60.75" customHeight="1" s="17"/>
     <row r="155" ht="60.75" customHeight="1" s="17"/>
     <row r="156" ht="60.75" customHeight="1" s="17"/>
     <row r="157" ht="60.75" customHeight="1" s="17"/>
@@ -8318,840 +7946,6 @@
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9971,7 +8765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -10285,6 +9079,386 @@
         </is>
       </c>
       <c r="J10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Topic mese</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore a 26° tutto il giorno o solo qualche ora a 18°?</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>Confusi su come usare il climatizzatore — spesso fanno il contrario di quel che servirebbe</t>
+        </is>
+      </c>
+      <c r="E11" s="31" t="inlineStr">
+        <is>
+          <t>L'errore d'uso che gonfia la bolletta + la regola semplice per usarlo efficiente d'estate.</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G11" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>Topic mese: climatizzazione estiva privati</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J11" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore: prima di accenderlo a giugno, fai queste 3 cose</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>Accende il clima dopo mesi di fermo senza fare nulla, poi si lamenta che puzza, non rinfresca o consuma troppo.</t>
+        </is>
+      </c>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>Lista pratica in 60 secondi: pulizia filtri, controllo che non perda, sanificazione veloce. Tre gesti casalinghi che evitano una chiamata d'emergenza ad agosto.</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I12" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J12" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>Pannelli fotovoltaici: davvero non vanno mai puliti?</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>Pensano siano 'installa e dimentica' e perdono resa senza accorgersene.</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Cosa succede ai pannelli dopo 2-3 anni (polvere, pollini, salsedine) e quando una pulizia ha senso davvero, senza promesse miracolose.</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte</t>
+        </is>
+      </c>
+      <c r="I13" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J13" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>Climatizzatore: come scelgo il modello giusto per casa mia?</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>Non sa da dove partire nella scelta — marca, BTU, classe energetica gli sembrano tutti uguali</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>I 3 parametri pratici che fanno la differenza nella scelta di un climatizzatore, spiegati senza tecnicismi.</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J14" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico: copre anche la sostituzione del vecchio condizionatore?</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>Pensa che il Conto Termico valga solo per caldaie e pompe di calore, non per i climatizzatori</t>
+        </is>
+      </c>
+      <c r="E15" s="31" t="inlineStr">
+        <is>
+          <t>Quando la rottamazione di un vecchio climatizzatore dà diritto al Conto Termico e come richiederlo.</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica / normativa</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="n"/>
+      <c r="I15" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J15" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: non devi rifare tutto l'impianto. E il fotovoltaico può aiutarti.</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>Rinunciano alla PdC convinti serva un cantiere enorme — non sanno che si può partire in piccolo</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>Perché in molti casi basta un impianto più contenuto, e come il fotovoltaico aiuta a sostenere il consumo elettrico della PdC.</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G16" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H16" s="31" t="n"/>
+      <c r="I16" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J16" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>Con cosa arriviamo a casa tua: i mezzi della squadra Solare Italiano</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>Non sa quanta preparazione professionale c'è dietro ogni intervento</t>
+        </is>
+      </c>
+      <c r="E17" s="31" t="inlineStr">
+        <is>
+          <t>Ripresa dei furgoni e della piattaforma aerea per mostrare l'attrezzatura sul campo. Nessuna improvvisazione.</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Conosci Solare Italiano</t>
+        </is>
+      </c>
+      <c r="G17" s="30" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J17" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Interna</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>Cosa facciamo prima di venire da te: la preparazione del furgone</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>Non immagina il lavoro di preparazione dietro ogni uscita — pensa che i tecnici partano senza organizzazione</t>
+        </is>
+      </c>
+      <c r="E18" s="31" t="inlineStr">
+        <is>
+          <t>Il team che carica il furgone, controlla gli strumenti e prepara il materiale prima di partire. Dietro le quinte della professionalità.</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="G18" s="30" t="inlineStr">
+        <is>
+          <t>Dietro le quinte squadra</t>
+        </is>
+      </c>
+      <c r="H18" s="31" t="n"/>
+      <c r="I18" s="30" t="inlineStr">
+        <is>
+          <t>Produzione</t>
+        </is>
+      </c>
+      <c r="J18" s="30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-29: idee notturne news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J999"/>
+  <dimension ref="A1:J159"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8307,851 +8307,242 @@
       </c>
       <c r="J154" s="30" t="n"/>
     </row>
-    <row r="155" ht="60.75" customHeight="1" s="17"/>
-    <row r="156" ht="60.75" customHeight="1" s="17"/>
-    <row r="157" ht="60.75" customHeight="1" s="17"/>
-    <row r="158" ht="45.75" customHeight="1" s="17"/>
-    <row r="159" ht="45.75" customHeight="1" s="17"/>
+    <row r="155" ht="60.75" customHeight="1" s="17">
+      <c r="A155" s="29" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B155" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C155" s="31" t="inlineStr">
+        <is>
+          <t>Fotovoltaico e Conto Termico 3.0: puoi chiederlo solo se installi anche la pompa di calore — ecco perché</t>
+        </is>
+      </c>
+      <c r="D155" s="31" t="inlineStr">
+        <is>
+          <t>Pensano di poter accedere al Conto Termico 3.0 per il fotovoltaico da solo, non sanno che la pompa di calore è obbligatoria come intervento principale</t>
+        </is>
+      </c>
+      <c r="E155" s="31" t="inlineStr">
+        <is>
+          <t>Reel spiegazione regola CT 3.0: il fotovoltaico (e le batterie) sono incentivabili solo come complemento a una pompa di calore nuova. Senza la pompa, non puoi accedere al Conto Termico per il solo fotovoltaico. Chiarisce un meccanismo oscuro che genera molte aspettative sbagliate. Collegato alle regole operative CT 3.0 aggiornate luglio 2026.</t>
+        </is>
+      </c>
+      <c r="F155" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G155" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H155" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I155" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J155" s="30" t="n"/>
+    </row>
+    <row r="156" ht="60.75" customHeight="1" s="17">
+      <c r="A156" s="29" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B156" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C156" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0: cosa devi davvero preparare per fare domanda al GSE (non basta la fattura)</t>
+        </is>
+      </c>
+      <c r="D156" s="31" t="inlineStr">
+        <is>
+          <t>Sanno che l'incentivo esiste ma non sanno quali documenti servono, temono di sbagliare la domanda o di dimenticare qualcosa</t>
+        </is>
+      </c>
+      <c r="E156" s="31" t="inlineStr">
+        <is>
+          <t>Reel pratico sulla documentazione necessaria per richiedere il CT 3.0 per la pompa di calore: foto ante-operam, scheda tecnica prodotto, relazione tecnica, dati catastali, IBAN. Ispira fiducia: 'non è complicato se sai cosa serve'. Collegato alle nuove FAQ GSE del 22 luglio 2026 che chiariscono procedure di verifica pagamenti.</t>
+        </is>
+      </c>
+      <c r="F156" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G156" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H156" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I156" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J156" s="30" t="n"/>
+    </row>
+    <row r="157" ht="60.75" customHeight="1" s="17">
+      <c r="A157" s="29" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B157" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C157" s="31" t="inlineStr">
+        <is>
+          <t>Inserto a pellet o inserto a legna: 3 domande per capire quale fa per te</t>
+        </is>
+      </c>
+      <c r="D157" s="31" t="inlineStr">
+        <is>
+          <t>Hanno un caminetto aperto e vogliono migliorarlo, ma non sanno scegliere tra inserto a pellet e inserto a legna</t>
+        </is>
+      </c>
+      <c r="E157" s="31" t="inlineStr">
+        <is>
+          <t>Reel con struttura '3 domande': 1) Hai accesso comodo alla legna? 2) Vuoi un calore automatico o ami il rituale del fuoco? 3) Hai qualcuno in casa durante il giorno? A ogni risposta corrisponde una direzione chiara. Evergreen, concreto, aiuta a decidere senza bisogno del tecnico come primo passo.</t>
+        </is>
+      </c>
+      <c r="F157" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G157" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H157" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I157" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J157" s="30" t="n"/>
+    </row>
+    <row r="158" ht="45.75" customHeight="1" s="17">
+      <c r="A158" s="29" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B158" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C158" s="31" t="inlineStr">
+        <is>
+          <t>Stufa a pellet: quando va pulita davvero e cosa succede se aspetti troppo</t>
+        </is>
+      </c>
+      <c r="D158" s="31" t="inlineStr">
+        <is>
+          <t>Hanno la stufa ma non sanno con quale frequenza fare manutenzione, temono di dimenticarla e di danneggiarla o di perdere la garanzia</t>
+        </is>
+      </c>
+      <c r="E158" s="31" t="inlineStr">
+        <is>
+          <t>Reel su frequenza e tipo di pulizia: pulizia settimanale fai-da-te (cenere, braciere), pulizia mensile (vetro, tubo fumo), revisione annuale dal tecnico. Cosa succede se non la fai: fumo in casa, rottura della valvola, decadimento garanzia. Pratico e rassicurante.</t>
+        </is>
+      </c>
+      <c r="F158" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Stufe</t>
+        </is>
+      </c>
+      <c r="G158" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione</t>
+        </is>
+      </c>
+      <c r="H158" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I158" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J158" s="30" t="n"/>
+    </row>
+    <row r="159" ht="45.75" customHeight="1" s="17">
+      <c r="A159" s="29" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B159" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C159" s="31" t="inlineStr">
+        <is>
+          <t>Il climatizzatore perde acqua dentro casa: è normale o è un guasto? Ecco come capirlo</t>
+        </is>
+      </c>
+      <c r="D159" s="31" t="inlineStr">
+        <is>
+          <t>Vedono acqua che cola dal climatizzatore sulla parete o sul pavimento e non capiscono se è normale o segnale di guasto grave</t>
+        </is>
+      </c>
+      <c r="E159" s="31" t="inlineStr">
+        <is>
+          <t>Reel diagnostico: spiega che una piccola condensa esterna è normale, ma l'acqua che cola dentro è quasi sempre segnale di un tubo di scarico ostruito o di un'installazione sbagliata. Come riconoscere la differenza in 30 secondi. Genera fiducia: 'ecco quando devi chiamare il tecnico subito e quando puoi stare tranquillo'.</t>
+        </is>
+      </c>
+      <c r="F159" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Climatizzatore</t>
+        </is>
+      </c>
+      <c r="G159" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H159" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I159" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J159" s="30" t="n"/>
+    </row>
     <row r="160" ht="60.75" customHeight="1" s="17"/>
     <row r="161" ht="76.5" customHeight="1" s="17"/>
     <row r="162" ht="60.75" customHeight="1" s="17"/>
     <row r="163" ht="60.75" customHeight="1" s="17"/>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
-    <row r="575"/>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
-    <row r="602"/>
-    <row r="603"/>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
-    <row r="711"/>
-    <row r="712"/>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
-    <row r="739"/>
-    <row r="740"/>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
-    <row r="781"/>
-    <row r="782"/>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
-    <row r="809"/>
-    <row r="810"/>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
-    <row r="837"/>
-    <row r="838"/>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
-    <row r="865"/>
-    <row r="866"/>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
-    <row r="952"/>
-    <row r="953"/>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-07-30: 4 idee notturne news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J159"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8537,10 +8537,190 @@
       </c>
       <c r="J159" s="30" t="n"/>
     </row>
-    <row r="160" ht="60.75" customHeight="1" s="17"/>
-    <row r="161" ht="76.5" customHeight="1" s="17"/>
-    <row r="162" ht="60.75" customHeight="1" s="17"/>
-    <row r="163" ht="60.75" customHeight="1" s="17"/>
+    <row r="160" ht="60.75" customHeight="1" s="17">
+      <c r="A160" s="29" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B160" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C160" s="31" t="inlineStr">
+        <is>
+          <t>Hai fatto lavori Ecobonus nel 2026? Il portale ENEA è riaperto dal 25 giugno — ecco cosa succede se non invii la comunicazione entro 90 giorni</t>
+        </is>
+      </c>
+      <c r="D160" s="31" t="inlineStr">
+        <is>
+          <t>Chi ha fatto lavori di efficienza energetica rischia di perdere la detrazione Ecobonus se non invia la comunicazione ENEA entro 90 giorni dalla fine dei lavori — scadenza che la maggior parte dei proprietari ignora</t>
+        </is>
+      </c>
+      <c r="E160" s="31" t="inlineStr">
+        <is>
+          <t>Reel informativo: spiegare che il portale ENEA (bonusfiscali.enea.it) era sospeso ed è riaperto il 25/06/2026. Da quella data riparte il conto dei 90 giorni per inviare la comunicazione obbligatoria. Chi non lo fa perde la detrazione fiscale. Call to action: 'chiedi a chi ti ha fatto i lavori se è stata inviata'.</t>
+        </is>
+      </c>
+      <c r="F160" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G160" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H160" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I160" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J160" s="30" t="n"/>
+    </row>
+    <row r="161" ht="76.5" customHeight="1" s="17">
+      <c r="A161" s="29" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B161" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C161" s="31" t="inlineStr">
+        <is>
+          <t>Termostufa e termocamino: sembrano quasi la stessa cosa ma non lo sono — come capire qual è quella giusta per la tua casa</t>
+        </is>
+      </c>
+      <c r="D161" s="31" t="inlineStr">
+        <is>
+          <t>La confusione tra termostufa (apparecchio autonomo che scalda anche l'acqua degli impianti) e termocamino (inserto connesso all'impianto) porta i proprietari a chiedere il prodotto sbagliato o a rinunciare senza capire le opzioni disponibili</t>
+        </is>
+      </c>
+      <c r="E161" s="31" t="inlineStr">
+        <is>
+          <t>Reel con comparazione visiva: termostufa sta da sola e si collega ai termosifoni, termocamino si inserisce dentro un camino esistente e si collega all'impianto. Spiegare in 3 domande quale fa per te: hai già un camino? Vuoi un arredo a vista o integrarlo? Riscaldamento di zona o di tutto l'impianto? Regola d'oro: SÌ.</t>
+        </is>
+      </c>
+      <c r="F161" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G161" s="30" t="inlineStr">
+        <is>
+          <t>Confronto tra prodotti</t>
+        </is>
+      </c>
+      <c r="H161" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I161" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J161" s="30" t="n"/>
+    </row>
+    <row r="162" ht="60.75" customHeight="1" s="17">
+      <c r="A162" s="29" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B162" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C162" s="31" t="inlineStr">
+        <is>
+          <t>I pannelli solari per l'acqua calda non sono fotovoltaici — cosa fanno davvero e quando conviene installarli</t>
+        </is>
+      </c>
+      <c r="D162" s="31" t="inlineStr">
+        <is>
+          <t>Confusione generalizzata tra pannelli solari termici (producono calore per l'acqua calda sanitaria) e fotovoltaici (producono elettricità) porta i proprietari a ignorare del tutto i solari termici o a installare il prodotto sbagliato per le proprie esigenze</t>
+        </is>
+      </c>
+      <c r="E162" s="31" t="inlineStr">
+        <is>
+          <t>Reel esplicativo: pannello solare termico → scalda l'acqua del boiler, abbatte bolletta gas/luce per acqua calda. Fotovoltaico → produce elettricità. Quando conviene il solare termico: casa con alto consumo di acqua calda, già connessa a gas, senza fotovoltaico o come complemento. Linguaggio semplice, niente numeri di risparmio.</t>
+        </is>
+      </c>
+      <c r="F162" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Solari</t>
+        </is>
+      </c>
+      <c r="G162" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H162" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I162" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J162" s="30" t="n"/>
+    </row>
+    <row r="163" ht="60.75" customHeight="1" s="17">
+      <c r="A163" s="29" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B163" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C163" s="31" t="inlineStr">
+        <is>
+          <t>Hai un'auto elettrica o ibrida ricaricabile? Ecco perché la presa normale a muro non basta e cosa cambia davvero con una wallbox</t>
+        </is>
+      </c>
+      <c r="D163" s="31" t="inlineStr">
+        <is>
+          <t>I proprietari con auto elettrica non capiscono la differenza concreta tra caricare dall'ordinaria presa Schuko (lenta, potenzialmente pericolosa per uso continuato) e avere una wallbox domestica certificata, rinunciando a installarla o aspettando anni</t>
+        </is>
+      </c>
+      <c r="E163" s="31" t="inlineStr">
+        <is>
+          <t>Reel con confronto pratico: presa normale = ~2,3 kW, ricarica lentissima (8-10 ore per auto media) e non progettata per uso continuativo. Wallbox = 7,4-11 kW, ricarica in 2-3 ore, sicura, monitorabile. Spiegare anche che con fotovoltaico la wallbox si può programmare per caricare con energia prodotta in casa. Call to action: 'se ricarichi da presa, chiedici una valutazione'.</t>
+        </is>
+      </c>
+      <c r="F163" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G163" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H163" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I163" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J163" s="30" t="n"/>
+    </row>
     <row r="164" ht="60.75" customHeight="1" s="17"/>
     <row r="165" ht="60.75" customHeight="1" s="17"/>
   </sheetData>

</xml_diff>

<commit_message>
Master Idee 2026-07-31: 5 idee news-informed + news brief luglio 2026
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J999"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8721,8 +8721,1067 @@
       </c>
       <c r="J163" s="30" t="n"/>
     </row>
-    <row r="164" ht="60.75" customHeight="1" s="17"/>
-    <row r="165" ht="60.75" customHeight="1" s="17"/>
+    <row r="164" ht="60.75" customHeight="1" s="17">
+      <c r="A164" s="29" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B164" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C164" s="31" t="inlineStr">
+        <is>
+          <t>Dal 3 giugno la classe energetica della tua casa potrebbe essere peggiorata — senza che tu abbia fatto nulla</t>
+        </is>
+      </c>
+      <c r="D164" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario ha un APE ancora valido ma non sa che con il nuovo calcolo (in vigore dal 3 giugno 2026) la sua classe potrebbe risultare peggiore se dovesse rifarlo oggi</t>
+        </is>
+      </c>
+      <c r="E164" s="31" t="inlineStr">
+        <is>
+          <t>Reel che spiega: il nuovo APE 2026 non invalida quello vecchio, ma se sei in procinto di vendere, affittare o ristrutturare e devi rinnovarlo, i criteri sono più stringenti. La tua classe E potrebbe diventare F/G. Cosa fare adesso per tutelarsi.</t>
+        </is>
+      </c>
+      <c r="F164" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G164" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H164" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I164" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J164" s="30" t="n"/>
+    </row>
+    <row r="165" ht="60.75" customHeight="1" s="17">
+      <c r="A165" s="29" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B165" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C165" s="31" t="inlineStr">
+        <is>
+          <t>Vuoi ancora il bonus per sostituire la caldaia a gas? Nel 2026 non esiste più — ecco le uniche 3 strade con incentivo</t>
+        </is>
+      </c>
+      <c r="D165" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario pensa ancora di avere un bonus per cambiare la vecchia caldaia a gas e scopre che non c'è</t>
+        </is>
+      </c>
+      <c r="E165" s="31" t="inlineStr">
+        <is>
+          <t>Reel che smonta l'equivoco: dal 2025 la detrazione fiscale per caldaie a gas è finita. Le uniche soluzioni incentivate oggi sono pompa di calore (Ecobonus 50% o Conto Termico 3.0 fino al 65%), sistema ibrido caldaia+pompa di calore, caldaia a biomassa. Niente bonus per la caldaia a gas pura.</t>
+        </is>
+      </c>
+      <c r="F165" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G165" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H165" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I165" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J165" s="30" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="29" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B166" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C166" s="31" t="inlineStr">
+        <is>
+          <t>La pompa di calore add-on: si aggancia alla tua caldaia esistente e ora il Conto Termico 3.0 la incentiva</t>
+        </is>
+      </c>
+      <c r="D166" s="31" t="inlineStr">
+        <is>
+          <t>Chi ha già una caldaia e pensa che per avere la pompa di calore debba buttare tutto e rifare l'impianto</t>
+        </is>
+      </c>
+      <c r="E166" s="31" t="inlineStr">
+        <is>
+          <t>Reel che presenta la pompa di calore add-on: un sistema che si affianca (non sostituisce) la caldaia esistente. Il Conto Termico 3.0 ha introdotto questa categoria nel 2026. Si installa più facilmente, costa meno di una sostituzione completa, e ora ha accesso all'incentivo GSE.</t>
+        </is>
+      </c>
+      <c r="F166" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G166" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H166" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I166" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J166" s="30" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="29" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B167" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C167" s="31" t="inlineStr">
+        <is>
+          <t>Hai il fotovoltaico ma non ancora la batteria? La detrazione del 50% scade il 31 dicembre 2026 — dopo non si sa</t>
+        </is>
+      </c>
+      <c r="D167" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario con fotovoltaico rimanda l'acquisto della batteria di accumulo senza sapere che la detrazione fiscale ha una scadenza precisa</t>
+        </is>
+      </c>
+      <c r="E167" s="31" t="inlineStr">
+        <is>
+          <t>Reel urgency-driven: chi installa una batteria di accumulo collegata al fotovoltaico entro il 31/12/2026 detrae il 50% in 10 anni (36% per seconda casa). La Legge di Bilancio 2026 ha confermato il bonus, ma per il 2027 non ci sono ancora garanzie. Meglio non aspettare.</t>
+        </is>
+      </c>
+      <c r="F167" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G167" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H167" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I167" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J167" s="30" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="29" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B168" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C168" s="31" t="inlineStr">
+        <is>
+          <t>Stufa o inserto a legna: in alcune zone della tua città potresti non poterlo accendere — sai se la tua casa è in una di queste aree?</t>
+        </is>
+      </c>
+      <c r="D168" s="31" t="inlineStr">
+        <is>
+          <t>Il proprietario vuole installare una stufa o un inserto a legna ma non sa che nelle ZTL ambientali o nelle zone con restrizioni PM10 ci sono limiti all'accensione</t>
+        </is>
+      </c>
+      <c r="E168" s="31" t="inlineStr">
+        <is>
+          <t>Reel che apre gli occhi su un aspetto ignorato: nelle aree metropolitane e nei comuni con alta densità abitativa esistono ordinanze anti-smog che vietano o limitano l'uso di stufe e caminetti a legna nei giorni di allerta. Prima di installare, vale la pena verificare la zona.</t>
+        </is>
+      </c>
+      <c r="F168" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G168" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H168" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I168" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J168" s="30" t="n"/>
+    </row>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-08-01: 5 idee news-informed + news brief
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J168"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8721,8 +8721,236 @@
       </c>
       <c r="J163" s="30" t="n"/>
     </row>
-    <row r="164" ht="60.75" customHeight="1" s="17"/>
-    <row r="165" ht="60.75" customHeight="1" s="17"/>
+    <row r="164" ht="60.75" customHeight="1" s="17">
+      <c r="A164" s="29" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B164" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C164" s="31" t="inlineStr">
+        <is>
+          <t>Dal 29 maggio 2026 la classe energetica della tua casa potrebbe essere cambiata — senza che tu abbia fatto niente</t>
+        </is>
+      </c>
+      <c r="D164" s="31" t="inlineStr">
+        <is>
+          <t>Ho ristrutturato la casa anni fa e so che classe era. Ora scopro che la scala APE è cambiata e non so più dove sono</t>
+        </is>
+      </c>
+      <c r="E164" s="31" t="inlineStr">
+        <is>
+          <t>Dal 29 maggio 2026 è in vigore una nuova scala di classificazione energetica (nuovi requisiti minimi EPBD). Una casa in vecchia classe B potrebbe risultare declassata con i nuovi criteri. Il reel spiega cosa è cambiato, perché (recepimento parziale Direttiva Case Green), e cosa fare prima di vendere o avviare lavori: richiedere un APE aggiornato.</t>
+        </is>
+      </c>
+      <c r="F164" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G164" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H164" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I164" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J164" s="30" t="n"/>
+    </row>
+    <row r="165" ht="60.75" customHeight="1" s="17">
+      <c r="A165" s="29" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B165" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C165" s="31" t="inlineStr">
+        <is>
+          <t>Si è rotta la caldaia a gas: la sostituisco ancora con una caldaia a gas o passo alla pompa di calore?</t>
+        </is>
+      </c>
+      <c r="D165" s="31" t="inlineStr">
+        <is>
+          <t>Ho la caldaia rotta, devo decidere in fretta, ho paura di sbagliare e non capisco cosa mi conviene davvero nel 2026</t>
+        </is>
+      </c>
+      <c r="E165" s="31" t="inlineStr">
+        <is>
+          <t>Pain urgente del proprietario con caldaia guasta. Situazione 2026: sostituire con gas è ancora legale ma i bonus per il gas sono finiti dal 2025. Passare alla pompa di calore dà accesso al Conto Termico 3.0 (fino al 65%). Il reel guida la decisione senza calcoli numerici: quando ha senso pianificare il passaggio, e quando la caldaia a gas rimane la soluzione pratica.</t>
+        </is>
+      </c>
+      <c r="F165" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G165" s="30" t="inlineStr">
+        <is>
+          <t>Quando sostituirlo</t>
+        </is>
+      </c>
+      <c r="H165" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I165" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J165" s="30" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="29" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B166" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C166" s="31" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0: dopo che mandi la domanda al GSE, i soldi arrivano subito o aspetti anni?</t>
+        </is>
+      </c>
+      <c r="D166" s="31" t="inlineStr">
+        <is>
+          <t>Ho fatto i lavori, ho inviato la domanda al GSE, ma non so quando mi pagano — ho paura che ci vogliano anni prima di vedere qualcosa</t>
+        </is>
+      </c>
+      <c r="E166" s="31" t="inlineStr">
+        <is>
+          <t>Pain frequentissimo mai risposto chiaramente. Il reel spiega i due casi: contributo sotto 15.000€ (pagamento unico entro 60 giorni dalla validazione GSE) e oltre (2-5 rate annuali). Contesto 2026: dopo la chiusura-riapertura del portale a marzo-aprile i tempi si sono allungati, ma non si parla di anni. Reel che rassicura con dati concreti senza numeri di risparmio.</t>
+        </is>
+      </c>
+      <c r="F166" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G166" s="30" t="inlineStr">
+        <is>
+          <t>Domanda economica</t>
+        </is>
+      </c>
+      <c r="H166" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I166" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J166" s="30" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="29" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B167" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C167" s="31" t="inlineStr">
+        <is>
+          <t>Hai già il fotovoltaico ma non la batteria? C'è ancora il 50% di detrazione per aggiungerla — ma solo fino al 31 dicembre 2026</t>
+        </is>
+      </c>
+      <c r="D167" s="31" t="inlineStr">
+        <is>
+          <t>Ho installato il fotovoltaico qualche anno fa senza batteria. Vorrei aggiungerla adesso ma non so se ci sono ancora incentivi o se ho già perso il treno</t>
+        </is>
+      </c>
+      <c r="E167" s="31" t="inlineStr">
+        <is>
+          <t>Pain di chi ha già l'impianto fotovoltaico e si chiede se aggiungere la batteria ha ancora incentivi. Nel 2026 il Bonus Casa al 50% si applica anche all'accumulo aggiunto su un impianto già esistente, fino al 31 dicembre 2026. Spiega il meccanismo senza calcoli numerici, con la scadenza come call to action all'informarsi.</t>
+        </is>
+      </c>
+      <c r="F167" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Batterie di Accumulo</t>
+        </is>
+      </c>
+      <c r="G167" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H167" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I167" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J167" s="30" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="29" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B168" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C168" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: 'quando fa -5°C fuori non scalda' — è vero o è il solito mito che blocca tutto?</t>
+        </is>
+      </c>
+      <c r="D168" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito dire che la pompa di calore si ferma quando fa molto freddo. Ho paura di installarla e trovarmi al gelo d'inverno</t>
+        </is>
+      </c>
+      <c r="E168" s="31" t="inlineStr">
+        <is>
+          <t>Scetticismo classico mai smontato onestamente nei reel. Risposta diretta: dipende dal modello. Le pompe di calore inverter moderne sono progettate per lavorare fino a -15°C / -20°C senza fermarsi, solo con potenza ridotta. Il reel spiega quando il freddo è davvero un problema (vecchi modelli o climi alpini estremi) e quando no — aiuta il 55enne scettico a capire se può fidarsi.</t>
+        </is>
+      </c>
+      <c r="F168" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G168" s="30" t="inlineStr">
+        <is>
+          <t>Errore comune</t>
+        </is>
+      </c>
+      <c r="H168" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I168" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J168" s="30" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Master Idee 2026-08-02: 4 idee news-informed + news brief
Idee aggiunte (righe 169-172):
- Pompa di calore: detrazione 50% vs 36% dal 2027
- Caldaia ibrida: alternativa incentivata per chi non vuole solo pompa di calore
- FAQ CT 3.0: non solo pompe di calore, copre anche pellet e solare
- Inserti/case classe F-G: nuova scala APE e impatto sul valore

News brief: Social/04_News_Feed/news_2026-08-02.md
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J168"/>
+  <dimension ref="A1:J172"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -8950,6 +8950,190 @@
         </is>
       </c>
       <c r="J168" s="30" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="29" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B169" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C169" s="31" t="inlineStr">
+        <is>
+          <t>Chi aspetta il 2027 per installare la pompa di calore perde il 14% di detrazione in più — non è un dettaglio</t>
+        </is>
+      </c>
+      <c r="D169" s="31" t="inlineStr">
+        <is>
+          <t>Non so se vale la pena fare i lavori ora o aspettare — i bonus ci sono sempre</t>
+        </is>
+      </c>
+      <c r="E169" s="31" t="inlineStr">
+        <is>
+          <t>Reel educativo sulla scadenza del 31/12/2026: spiega la differenza tra il fare l'installazione entro l'anno (detrazione 50% prima casa) e rimandarla al 2027 (36%). Dal 2027 la Legge di Bilancio prevede una riduzione secca. Non numeri di risparmio specifici, ma il meccanismo del 'prima casa 2026 vs 2027' spiegato in modo chiaro.</t>
+        </is>
+      </c>
+      <c r="F169" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G169" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H169" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I169" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J169" s="30" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="29" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B170" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C170" s="31" t="inlineStr">
+        <is>
+          <t>Non sai se passare subito alla pompa di calore o tenere ancora la caldaia a gas? La caldaia ibrida esiste ed è incentivata — ma quasi nessuno la conosce</t>
+        </is>
+      </c>
+      <c r="D170" s="31" t="inlineStr">
+        <is>
+          <t>Ho sentito che le caldaie a gas non hanno più bonus, ma la pompa di calore non mi convince del tutto — non so cosa fare</t>
+        </is>
+      </c>
+      <c r="E170" s="31" t="inlineStr">
+        <is>
+          <t>Spiega il sistema ibrido (caldaia a gas esistente + pompa di calore in parallelo): chi può installarlo, che rientra nel Conto Termico 3.0 e nell'Ecobonus, e perché è ideale per chi ha già radiatori e non vuole cambiare tutto l'impianto. Risponde alla notizia che le caldaie a gas pure sono fuori da tutti i bonus 2026.</t>
+        </is>
+      </c>
+      <c r="F170" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G170" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H170" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I170" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J170" s="30" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="29" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B171" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C171" s="31" t="inlineStr">
+        <is>
+          <t>Il Conto Termico 3.0 non è solo per le pompe di calore: copre anche le caldaie a pellet e i pannelli solari — ecco cosa rientra davvero</t>
+        </is>
+      </c>
+      <c r="D171" s="31" t="inlineStr">
+        <is>
+          <t>Pensavo il Conto Termico fosse solo per le pompe di calore — non so se il mio intervento rientra</t>
+        </is>
+      </c>
+      <c r="E171" s="31" t="inlineStr">
+        <is>
+          <t>Chiarisce il malinteso diffuso che il CT 3.0 riguardi solo le pompe di calore. Spiega che copre anche caldaie a biomassa (incluse quelle a pellet), pannelli solari termici e altri interventi di efficienza. Collegato all'aggiornamento FAQ GSE del 22 luglio 2026. Aiuta il target a capire se il loro prodotto è incentivabile prima di chiedere un preventivo.</t>
+        </is>
+      </c>
+      <c r="F171" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G171" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H171" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I171" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J171" s="30" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="29" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B172" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C172" s="31" t="inlineStr">
+        <is>
+          <t>Stai ristrutturando una casa in classe F o G? Prima di installare solo un inserto o una stufa, c'è una cosa che devi sapere sulla nuova classificazione energetica</t>
+        </is>
+      </c>
+      <c r="D172" s="31" t="inlineStr">
+        <is>
+          <t>Sto ristrutturando casa e voglio mettere un inserto a legna o una stufa, ma ho sentito che la classe energetica ora conta di più per il valore della casa</t>
+        </is>
+      </c>
+      <c r="E172" s="31" t="inlineStr">
+        <is>
+          <t>Collegato alla nuova scala APE in vigore dal 29 maggio 2026 (EPBD IV): le case in classe F/G perderanno valore rispetto alle classi D+. Spiega che l'inserto o la stufa è un ottimo complemento al riscaldamento, ma non migliora la classe energetica dell'edificio. Chi sta ristrutturando una casa in classe bassa dovrebbe valutare anche un intervento sull'isolamento o sull'impianto principale per non perdere valore al momento di vendere.</t>
+        </is>
+      </c>
+      <c r="F172" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G172" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H172" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I172" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J172" s="30" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>

</xml_diff>

<commit_message>
Master Idee 2026-08-03: 5 idee news-informed + news brief agosto 2026
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J172"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9134,6 +9134,236 @@
         </is>
       </c>
       <c r="J172" s="30" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="29" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B173" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C173" s="31" t="inlineStr">
+        <is>
+          <t>Hai mandato la domanda al Conto Termico 3.0 al GSE: come controllare lo stato della pratica e cosa fare se hai sbagliato l'IBAN</t>
+        </is>
+      </c>
+      <c r="D173" s="31" t="inlineStr">
+        <is>
+          <t>Ho inviato la domanda al GSE ma non so se è stata approvata, come tracciarla, o cosa fare se mi accorgo di aver inserito l'IBAN sbagliato</t>
+        </is>
+      </c>
+      <c r="E173" s="31" t="inlineStr">
+        <is>
+          <t>Il GSE ha aggiornato le FAQ operative il 22 luglio 2026 (KB0017867). Reel spiega: 1) dove controllare lo stato della pratica sul PortalTermico 3.0, 2) come richiedere la variazione IBAN tramite modulistica specifica, 3) come chiedere assistenza per problemi di pagamento. Ispirato da news reale GSE.</t>
+        </is>
+      </c>
+      <c r="F173" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G173" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H173" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I173" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J173" s="30" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="29" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B174" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C174" s="31" t="inlineStr">
+        <is>
+          <t>Pompa di calore: Conto Termico 3.0 o Ecobonus? Non è la stessa cosa — ecco quando uno vale più dell'altro</t>
+        </is>
+      </c>
+      <c r="D174" s="31" t="inlineStr">
+        <is>
+          <t>Voglio installare una pompa di calore e mi hanno parlato sia del Conto Termico 3.0 che dell'Ecobonus — non capisco quale scegliere e se si possono usare insieme</t>
+        </is>
+      </c>
+      <c r="E174" s="31" t="inlineStr">
+        <is>
+          <t>Reel confronta i due incentivi principali: CT 3.0 (contributo diretto fino al 65%, liquidità rapida, erogazione diretta GSE) vs Ecobonus (detrazione IRPEF 50%, recupero in 10 anni in dichiarazione). Spiega quando conviene uno rispetto all'altro in base al profilo IRPEF e alla spesa totale. News-informed: CT 3.0 in vigore dal 25/12/2025.</t>
+        </is>
+      </c>
+      <c r="F174" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pompe di Calore</t>
+        </is>
+      </c>
+      <c r="G174" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H174" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I174" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J174" s="30" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="29" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B175" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C175" s="31" t="inlineStr">
+        <is>
+          <t>Caldaia a pellet o pompa di calore? Non scegliere prima di aver risposto a queste 3 domande sulla tua casa</t>
+        </is>
+      </c>
+      <c r="D175" s="31" t="inlineStr">
+        <is>
+          <t>Non so se conviene installare una caldaia a pellet o una pompa di calore — sembrano entrambe valide e non capisco cosa cambia davvero per la mia situazione</t>
+        </is>
+      </c>
+      <c r="E175" s="31" t="inlineStr">
+        <is>
+          <t>Reel non promuove né l'una né l'altra ma aiuta a capire con 3 domande: 1) Hai radiatori ad alta temperatura? (→ caldaia a pellet è più compatibile), 2) La casa è ben isolata? (→ vantaggio pompa di calore), 3) Hai spazio per lo stoccaggio pellet? CTA: sopralluogo gratuito per la valutazione giusta.</t>
+        </is>
+      </c>
+      <c r="F175" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G175" s="30" t="inlineStr">
+        <is>
+          <t>Come scegliere il modello giusto</t>
+        </is>
+      </c>
+      <c r="H175" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I175" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J175" s="30" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="29" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B176" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C176" s="31" t="inlineStr">
+        <is>
+          <t>Wallbox a casa o colonnine pubbliche: sembrano intercambiabili ma non è così — ecco perché chi ha l'auto elettrica prima o poi installa la wallbox</t>
+        </is>
+      </c>
+      <c r="D176" s="31" t="inlineStr">
+        <is>
+          <t>Ho l'auto elettrica e uso le colonnine pubbliche — non so se ha senso installare anche la wallbox a casa o è un costo inutile</t>
+        </is>
+      </c>
+      <c r="E176" s="31" t="inlineStr">
+        <is>
+          <t>Reel spiega la differenza concreta: colonnina pubblica = lenta, cara al kWh, fila, non disponibile H24. Wallbox = ricarica di notte con energia propria (fotovoltaico o tariffa notturna bassa), costi ridotti, auto sempre pronta la mattina. Chiude con il bonus Ecobonus 50% per l'installazione della wallbox, valido fino a fine 2026.</t>
+        </is>
+      </c>
+      <c r="F176" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G176" s="30" t="inlineStr">
+        <is>
+          <t>Confronto con alternative</t>
+        </is>
+      </c>
+      <c r="H176" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I176" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J176" s="30" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="29" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B177" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C177" s="31" t="inlineStr">
+        <is>
+          <t>Il fotovoltaico produce energia anche quando non sei a casa: cosa succede davvero all'elettricità in eccesso (non è buttata via)</t>
+        </is>
+      </c>
+      <c r="D177" s="31" t="inlineStr">
+        <is>
+          <t>Ho il fotovoltaico e non capisco cosa succede all'energia che non consumo — finisce in rete? Me la pagano? La perdo?</t>
+        </is>
+      </c>
+      <c r="E177" s="31" t="inlineStr">
+        <is>
+          <t>Reel spiega in modo semplice lo scambio sul posto: l'energia in eccesso va in rete e viene contabilizzata come credito, recuperato poi quando si usa energia dalla rete (es. di notte). Spiega la differenza rispetto a chi ha la batteria di accumulo (recupero diretto senza passare dalla rete). CTA: se vuoi trattenere tutta la tua energia, la batteria è il passo successivo.</t>
+        </is>
+      </c>
+      <c r="F177" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Pannelli Fotovoltaici</t>
+        </is>
+      </c>
+      <c r="G177" s="30" t="inlineStr">
+        <is>
+          <t>Come funziona</t>
+        </is>
+      </c>
+      <c r="H177" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I177" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J177" s="30" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>

</xml_diff>

<commit_message>
Master Idee 2026-08-04: 5 idee news-informed + news brief agosto 2026
- 3 idee collegate a news (bonus colonnine, Ecobonus caldaie gas sparito, EPBD infrazione UE)
- 2 idee evergreen (camino aperto → inserto, caldaia pellet spazio)
- News brief: 5 notizie rilevanti su incentivi e normativa agosto 2026
</commit_message>
<xml_diff>
--- a/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
+++ b/Social/01_Tracker/Solare_Italiano_Content_System.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J172"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9134,6 +9134,236 @@
         </is>
       </c>
       <c r="J172" s="30" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="29" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B173" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C173" s="31" t="inlineStr">
+        <is>
+          <t>Il bonus colonnine 2026 rimborsa l'80% del costo ma le domande non sono ancora aperte — cosa fare adesso per arrivare preparato</t>
+        </is>
+      </c>
+      <c r="D173" s="31" t="inlineStr">
+        <is>
+          <t>Ha l'auto elettrica o ibrida plug-in, sa che esiste il bonus, ma non sa quando si apre lo sportello né come non perdere il turno</t>
+        </is>
+      </c>
+      <c r="E173" s="31" t="inlineStr">
+        <is>
+          <t>Reel news-informed: il bonus wallbox 2026 copre il 40-80% (fino a 1.500€ privati, 8.000€ condomini). Le domande non sono ancora aperte. Il reel spiega: cos'è il bonus, chi ne ha diritto, e cosa conviene fare ora (ottenere il preventivo, controllare il sito MIMIT) per essere pronti quando apre lo sportello.</t>
+        </is>
+      </c>
+      <c r="F173" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Colonnine di Ricarica</t>
+        </is>
+      </c>
+      <c r="G173" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H173" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I173" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J173" s="30" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="29" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B174" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C174" s="31" t="inlineStr">
+        <is>
+          <t>Dal 2025 l'Ecobonus per sostituire la caldaia a gas è sparito — ma ci sono altri due incentivi che quasi nessuno conosce</t>
+        </is>
+      </c>
+      <c r="D174" s="31" t="inlineStr">
+        <is>
+          <t>Vuole cambiare la vecchia caldaia a gas e cerca il bonus che 'c'era prima', non sa che l'Ecobonus per le caldaie a gas è stato eliminato</t>
+        </is>
+      </c>
+      <c r="E174" s="31" t="inlineStr">
+        <is>
+          <t>Reel news-informed: molti proprietari cercano ancora l'Ecobonus per la caldaia a gas, ma dal 2025 non esiste più per i fossili. Il reel chiarisce cosa è rimasto: il Bonus Ristrutturazioni al 36% (qualsiasi caldaia) e il Conto Termico (solo per caldaie a pellet o pompe di calore). Utile per chi deve decidere cosa fare.</t>
+        </is>
+      </c>
+      <c r="F174" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G174" s="30" t="inlineStr">
+        <is>
+          <t>Incentivi</t>
+        </is>
+      </c>
+      <c r="H174" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I174" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J174" s="30" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="29" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B175" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C175" s="31" t="inlineStr">
+        <is>
+          <t>L'Italia sta prendendo una multa dall'UE sulle case green — cosa cambia concretamente per chi ha una casa in classe E, F o G</t>
+        </is>
+      </c>
+      <c r="D175" s="31" t="inlineStr">
+        <is>
+          <t>Ha sentito di procedure d'infrazione e multa UE sulle case verdi, è confuso e preoccupato per la sua casa, non sa cosa significhi per lui</t>
+        </is>
+      </c>
+      <c r="E175" s="31" t="inlineStr">
+        <is>
+          <t>Reel news-informed: l'Italia è sotto procedura d'infrazione UE per non aver recepito la direttiva EPBD (Case Green). Il reel demistifica: non c'è obbligo immediato di ristrutturazione per i privati, ma le scadenze 2030-2035 si avvicinano. Spiega cosa significa avere una casa in classe bassa e quali interventi (pompa di calore, isolamento, fotovoltaico) preparano la casa al futuro con incentivi ancora attivi.</t>
+        </is>
+      </c>
+      <c r="F175" s="30" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="G175" s="30" t="inlineStr">
+        <is>
+          <t>Domanda burocratica/normativa</t>
+        </is>
+      </c>
+      <c r="H175" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I175" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J175" s="30" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="29" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B176" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C176" s="31" t="inlineStr">
+        <is>
+          <t>Hai un camino aperto a legna che non scalda quasi niente e raffredda la casa quando è spento? Esiste una soluzione senza murare tutto</t>
+        </is>
+      </c>
+      <c r="D176" s="31" t="inlineStr">
+        <is>
+          <t>Ha un camino decorativo o poco efficiente, sa che spreca calore, vorrebbe una soluzione ma crede che richieda lavori enormi</t>
+        </is>
+      </c>
+      <c r="E176" s="31" t="inlineStr">
+        <is>
+          <t>Reel evergreen: i camini aperti tradizionali disperdono fino all'85% del calore su per il camino e, quando sono spenti, creano correnti fredde. La soluzione è l'inserto a legna o a pellet: si installa dentro il vano esistente senza demolizioni, chiude il tiraggio e porta il rendimento sopra l'85%. Reel 'prima/dopo' con spiegazione semplice.</t>
+        </is>
+      </c>
+      <c r="F176" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Inserti e Camini</t>
+        </is>
+      </c>
+      <c r="G176" s="30" t="inlineStr">
+        <is>
+          <t>A cosa viene sostituito</t>
+        </is>
+      </c>
+      <c r="H176" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I176" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J176" s="30" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="29" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B177" s="30" t="inlineStr">
+        <is>
+          <t>Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C177" s="31" t="inlineStr">
+        <is>
+          <t>Vuoi installare una caldaia a pellet ma non sai dove mettere la caldaia e il serbatoio? Ecco quanto spazio serve davvero</t>
+        </is>
+      </c>
+      <c r="D177" s="31" t="inlineStr">
+        <is>
+          <t>È interessato alla caldaia a pellet ma frena perché pensa che occupi troppo spazio o che serva un locale tecnico enorme</t>
+        </is>
+      </c>
+      <c r="E177" s="31" t="inlineStr">
+        <is>
+          <t>Reel evergreen operativo: uno dei dubbi pratici più comuni sulla caldaia a pellet è lo spazio. Il reel mostra le dimensioni reali di una caldaia a pellet standard, spiega le opzioni di stoccaggio pellet (sacco stagionale vs silo tessile vs silo rigido), e indica quale soluzione si adatta a diversi tipi di casa (appartamento con ripostiglio, villetta con cantina, casa con garage).</t>
+        </is>
+      </c>
+      <c r="F177" s="30" t="inlineStr">
+        <is>
+          <t>Prodotto - Caldaie</t>
+        </is>
+      </c>
+      <c r="G177" s="30" t="inlineStr">
+        <is>
+          <t>Dove si può installare</t>
+        </is>
+      </c>
+      <c r="H177" s="31" t="inlineStr">
+        <is>
+          <t>Generato automaticamente di notte (news-informed)</t>
+        </is>
+      </c>
+      <c r="I177" s="30" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="J177" s="30" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:M97"/>

</xml_diff>